<commit_message>
JSON to json personal history
</commit_message>
<xml_diff>
--- a/Future Features/New Features - Family Tree.xlsx
+++ b/Future Features/New Features - Family Tree.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://srcincgov1-my.sharepoint.us/personal/lauko_srcinc_com/Documents/Desktop/Personal/geneology/GED Keepers/Future Features/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="328" documentId="8_{D1FEEEA7-0E84-49B9-AD17-37D0BB95FB37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{56F36171-9998-42BF-86CE-46526890FB38}"/>
+  <xr:revisionPtr revIDLastSave="349" documentId="8_{D1FEEEA7-0E84-49B9-AD17-37D0BB95FB37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B4914AF7-F3AA-4AC3-A2FB-9CDAE4F5A54A}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{8067922A-00B7-4646-9500-13902203F407}"/>
+    <workbookView minimized="1" xWindow="3120" yWindow="3120" windowWidth="21600" windowHeight="11235" xr2:uid="{8067922A-00B7-4646-9500-13902203F407}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$B$3:$I$33</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$B$3:$I$34</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="72">
   <si>
     <t>Feature</t>
   </si>
@@ -233,9 +233,6 @@
     <t>display spouse, brothers/sisters/ etc…</t>
   </si>
   <si>
-    <t xml:space="preserve">Make ipad compatible </t>
-  </si>
-  <si>
     <t>need to make right and left clicks accessible on ipad for instance</t>
   </si>
   <si>
@@ -243,13 +240,50 @@
   </si>
   <si>
     <t>When adding an attachment, if it is the first and only attachment, automatically use it as the picture for that person</t>
+  </si>
+  <si>
+    <t>need to have a better URL</t>
+  </si>
+  <si>
+    <t>Detect and optimize for operation on an iPad and/or iPhone</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">clicks are working, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">!pull down menus are not working! </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>need to optimize for screenspace on phone</t>
+    </r>
+  </si>
+  <si>
+    <t>integrate personal histories more elegantly</t>
+  </si>
+  <si>
+    <t>how to include additional pictures, pdfs , etc…</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -324,6 +358,19 @@
       <strike/>
       <sz val="12"/>
       <color theme="0" tint="-0.249977111117893"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FFFF0000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -456,7 +503,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -605,6 +652,15 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -941,7 +997,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{11BA4F79-2AB7-4A24-A4BE-758442E1F8CB}">
   <sheetPr filterMode="1"/>
-  <dimension ref="B1:N45"/>
+  <dimension ref="B1:N46"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="49.28515625" style="8" customWidth="1"/>
@@ -1029,7 +1085,7 @@
         <v>3</v>
       </c>
       <c r="H4" s="38">
-        <f t="shared" ref="H4:H33" si="0">SUM(E4:G4)</f>
+        <f t="shared" ref="H4" si="0">SUM(E4:G4)</f>
         <v>8</v>
       </c>
       <c r="I4" s="40">
@@ -1047,10 +1103,10 @@
         <v>2</v>
       </c>
       <c r="C5" s="35" t="s">
+        <v>68</v>
+      </c>
+      <c r="D5" s="35" t="s">
         <v>64</v>
-      </c>
-      <c r="D5" s="35" t="s">
-        <v>65</v>
       </c>
       <c r="E5" s="42">
         <v>3</v>
@@ -1062,13 +1118,15 @@
         <v>3</v>
       </c>
       <c r="H5" s="21">
-        <f>SUM(E5:G5)</f>
+        <f t="shared" ref="H5:H34" si="1">SUM(E5:G5)</f>
         <v>8</v>
       </c>
       <c r="I5" s="9">
-        <v>4</v>
-      </c>
-      <c r="J5" s="20"/>
+        <v>3</v>
+      </c>
+      <c r="J5" s="20" t="s">
+        <v>69</v>
+      </c>
       <c r="K5" s="1"/>
       <c r="L5" s="1"/>
       <c r="M5" s="1"/>
@@ -1095,7 +1153,7 @@
         <v>2</v>
       </c>
       <c r="H6" s="46">
-        <f>SUM(E6:G6)</f>
+        <f t="shared" si="1"/>
         <v>7</v>
       </c>
       <c r="I6" s="48">
@@ -1128,7 +1186,7 @@
         <v>3</v>
       </c>
       <c r="H7" s="32">
-        <f>SUM(E7:G7)</f>
+        <f t="shared" si="1"/>
         <v>7</v>
       </c>
       <c r="I7" s="34">
@@ -1161,7 +1219,7 @@
         <v>2</v>
       </c>
       <c r="H8" s="21">
-        <f>SUM(E8:G8)</f>
+        <f t="shared" si="1"/>
         <v>7</v>
       </c>
       <c r="I8" s="9">
@@ -1179,21 +1237,21 @@
         <v>5</v>
       </c>
       <c r="C9" s="35" t="s">
-        <v>67</v>
-      </c>
-      <c r="D9" s="31"/>
-      <c r="E9" s="32">
-        <v>2</v>
-      </c>
-      <c r="F9" s="33">
-        <v>2</v>
-      </c>
-      <c r="G9" s="32">
+        <v>66</v>
+      </c>
+      <c r="D9" s="51"/>
+      <c r="E9" s="52">
+        <v>1</v>
+      </c>
+      <c r="F9" s="53">
+        <v>1</v>
+      </c>
+      <c r="G9" s="52">
         <v>3</v>
       </c>
-      <c r="H9" s="21">
-        <f>SUM(E9:G9)</f>
-        <v>7</v>
+      <c r="H9" s="52">
+        <f t="shared" si="1"/>
+        <v>5</v>
       </c>
       <c r="I9" s="9">
         <v>0</v>
@@ -1223,7 +1281,7 @@
         <v>3</v>
       </c>
       <c r="H10" s="46">
-        <f>SUM(E10:G10)</f>
+        <f t="shared" si="1"/>
         <v>7</v>
       </c>
       <c r="I10" s="48">
@@ -1258,7 +1316,7 @@
         <v>2</v>
       </c>
       <c r="H11" s="32">
-        <f>SUM(E11:G11)</f>
+        <f t="shared" si="1"/>
         <v>6</v>
       </c>
       <c r="I11" s="34">
@@ -1291,11 +1349,14 @@
         <v>2</v>
       </c>
       <c r="H12" s="21">
-        <f>SUM(E12:G12)</f>
+        <f t="shared" si="1"/>
         <v>7</v>
       </c>
       <c r="I12" s="9">
-        <v>0</v>
+        <v>4</v>
+      </c>
+      <c r="J12" s="41" t="s">
+        <v>67</v>
       </c>
       <c r="K12" s="1"/>
       <c r="L12" s="1"/>
@@ -1323,7 +1384,7 @@
         <v>2</v>
       </c>
       <c r="H13" s="21">
-        <f>SUM(E13:G13)</f>
+        <f t="shared" si="1"/>
         <v>6</v>
       </c>
       <c r="I13" s="9">
@@ -1336,7 +1397,7 @@
     </row>
     <row r="14" spans="2:14" ht="47.25" x14ac:dyDescent="0.25">
       <c r="B14" s="9">
-        <f>B13+1</f>
+        <f t="shared" ref="B14:B34" si="2">B13+1</f>
         <v>9</v>
       </c>
       <c r="C14" s="4" t="s">
@@ -1355,7 +1416,7 @@
         <v>2</v>
       </c>
       <c r="H14" s="21">
-        <f>SUM(E14:G14)</f>
+        <f t="shared" si="1"/>
         <v>6</v>
       </c>
       <c r="I14" s="9">
@@ -1368,7 +1429,7 @@
     </row>
     <row r="15" spans="2:14" ht="78.75" x14ac:dyDescent="0.25">
       <c r="B15" s="9">
-        <f>B14+1</f>
+        <f t="shared" si="2"/>
         <v>10</v>
       </c>
       <c r="C15" s="4" t="s">
@@ -1387,7 +1448,7 @@
         <v>2</v>
       </c>
       <c r="H15" s="21">
-        <f>SUM(E15:G15)</f>
+        <f t="shared" si="1"/>
         <v>6</v>
       </c>
       <c r="I15" s="9">
@@ -1401,16 +1462,16 @@
       <c r="M15" s="1"/>
       <c r="N15" s="1"/>
     </row>
-    <row r="16" spans="2:14" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B16" s="9">
-        <f>B15+1</f>
+        <f t="shared" si="2"/>
         <v>11</v>
       </c>
-      <c r="C16" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="D16" s="5" t="s">
-        <v>12</v>
+      <c r="C16" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="D16" s="12" t="s">
+        <v>71</v>
       </c>
       <c r="E16" s="21">
         <v>2</v>
@@ -1422,15 +1483,13 @@
         <v>2</v>
       </c>
       <c r="H16" s="21">
-        <f>SUM(E16:G16)</f>
+        <f t="shared" si="1"/>
         <v>6</v>
       </c>
       <c r="I16" s="9">
-        <v>2</v>
-      </c>
-      <c r="J16" s="20" t="s">
-        <v>66</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="J16" s="20"/>
       <c r="K16" s="1"/>
       <c r="L16" s="1"/>
       <c r="M16" s="1"/>
@@ -1438,14 +1497,14 @@
     </row>
     <row r="17" spans="2:14" ht="31.5" x14ac:dyDescent="0.25">
       <c r="B17" s="9">
-        <f>B16+1</f>
+        <f t="shared" si="2"/>
         <v>12</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="D17" s="23" t="s">
-        <v>21</v>
+        <v>11</v>
+      </c>
+      <c r="D17" s="5" t="s">
+        <v>12</v>
       </c>
       <c r="E17" s="21">
         <v>2</v>
@@ -1457,13 +1516,15 @@
         <v>2</v>
       </c>
       <c r="H17" s="21">
-        <f>SUM(E17:G17)</f>
+        <f t="shared" si="1"/>
         <v>6</v>
       </c>
       <c r="I17" s="9">
-        <v>0</v>
-      </c>
-      <c r="J17" s="20"/>
+        <v>2</v>
+      </c>
+      <c r="J17" s="20" t="s">
+        <v>65</v>
+      </c>
       <c r="K17" s="1"/>
       <c r="L17" s="1"/>
       <c r="M17" s="1"/>
@@ -1471,14 +1532,14 @@
     </row>
     <row r="18" spans="2:14" ht="31.5" x14ac:dyDescent="0.25">
       <c r="B18" s="9">
-        <f>B17+1</f>
+        <f t="shared" si="2"/>
         <v>13</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>57</v>
+        <v>20</v>
       </c>
       <c r="D18" s="23" t="s">
-        <v>58</v>
+        <v>21</v>
       </c>
       <c r="E18" s="21">
         <v>2</v>
@@ -1490,7 +1551,7 @@
         <v>2</v>
       </c>
       <c r="H18" s="21">
-        <f>SUM(E18:G18)</f>
+        <f t="shared" si="1"/>
         <v>6</v>
       </c>
       <c r="I18" s="9">
@@ -1502,16 +1563,16 @@
       <c r="M18" s="1"/>
       <c r="N18" s="1"/>
     </row>
-    <row r="19" spans="2:14" ht="83.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:14" ht="31.5" x14ac:dyDescent="0.25">
       <c r="B19" s="9">
-        <f>B18+1</f>
+        <f t="shared" si="2"/>
         <v>14</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="D19" s="5" t="s">
-        <v>49</v>
+        <v>57</v>
+      </c>
+      <c r="D19" s="23" t="s">
+        <v>58</v>
       </c>
       <c r="E19" s="21">
         <v>2</v>
@@ -1523,7 +1584,7 @@
         <v>2</v>
       </c>
       <c r="H19" s="21">
-        <f>SUM(E19:G19)</f>
+        <f t="shared" si="1"/>
         <v>6</v>
       </c>
       <c r="I19" s="9">
@@ -1535,32 +1596,32 @@
       <c r="M19" s="1"/>
       <c r="N19" s="1"/>
     </row>
-    <row r="20" spans="2:14" ht="83.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="29">
-        <f>B19+1</f>
+    <row r="20" spans="2:14" ht="83.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B20" s="9">
+        <f t="shared" si="2"/>
         <v>15</v>
       </c>
-      <c r="C20" s="30" t="s">
-        <v>31</v>
-      </c>
-      <c r="D20" s="31" t="s">
-        <v>32</v>
-      </c>
-      <c r="E20" s="32">
-        <v>2</v>
-      </c>
-      <c r="F20" s="33">
-        <v>1</v>
-      </c>
-      <c r="G20" s="32">
-        <v>3</v>
-      </c>
-      <c r="H20" s="32">
-        <f>SUM(E20:G20)</f>
+      <c r="C20" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="D20" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="E20" s="21">
+        <v>2</v>
+      </c>
+      <c r="F20" s="24">
+        <v>2</v>
+      </c>
+      <c r="G20" s="21">
+        <v>2</v>
+      </c>
+      <c r="H20" s="21">
+        <f t="shared" si="1"/>
         <v>6</v>
       </c>
-      <c r="I20" s="34">
-        <v>5</v>
+      <c r="I20" s="9">
+        <v>0</v>
       </c>
       <c r="J20" s="20"/>
       <c r="K20" s="1"/>
@@ -1568,32 +1629,32 @@
       <c r="M20" s="1"/>
       <c r="N20" s="1"/>
     </row>
-    <row r="21" spans="2:14" ht="83.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="9">
-        <f>B20+1</f>
+    <row r="21" spans="2:14" ht="83.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B21" s="29">
+        <f t="shared" si="2"/>
         <v>16</v>
       </c>
-      <c r="C21" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="D21" s="12" t="s">
-        <v>40</v>
-      </c>
-      <c r="E21" s="21">
-        <v>1</v>
-      </c>
-      <c r="F21" s="24">
-        <v>2</v>
-      </c>
-      <c r="G21" s="21">
+      <c r="C21" s="30" t="s">
+        <v>31</v>
+      </c>
+      <c r="D21" s="31" t="s">
+        <v>32</v>
+      </c>
+      <c r="E21" s="32">
+        <v>2</v>
+      </c>
+      <c r="F21" s="33">
+        <v>1</v>
+      </c>
+      <c r="G21" s="32">
         <v>3</v>
       </c>
-      <c r="H21" s="21">
-        <f>SUM(E21:G21)</f>
+      <c r="H21" s="32">
+        <f t="shared" si="1"/>
         <v>6</v>
       </c>
-      <c r="I21" s="9">
-        <v>0</v>
+      <c r="I21" s="34">
+        <v>5</v>
       </c>
       <c r="J21" s="20"/>
       <c r="K21" s="1"/>
@@ -1603,26 +1664,26 @@
     </row>
     <row r="22" spans="2:14" ht="83.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B22" s="9">
-        <f>B21+1</f>
+        <f t="shared" si="2"/>
         <v>17</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="D22" s="23" t="s">
-        <v>62</v>
+        <v>39</v>
+      </c>
+      <c r="D22" s="12" t="s">
+        <v>40</v>
       </c>
       <c r="E22" s="21">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F22" s="24">
         <v>2</v>
       </c>
       <c r="G22" s="21">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H22" s="21">
-        <f>SUM(E22:G22)</f>
+        <f t="shared" si="1"/>
         <v>6</v>
       </c>
       <c r="I22" s="9">
@@ -1634,16 +1695,16 @@
       <c r="M22" s="1"/>
       <c r="N22" s="1"/>
     </row>
-    <row r="23" spans="2:14" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:14" ht="83.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B23" s="9">
-        <f>B22+1</f>
+        <f t="shared" si="2"/>
         <v>18</v>
       </c>
-      <c r="C23" s="23" t="s">
-        <v>22</v>
+      <c r="C23" s="5" t="s">
+        <v>63</v>
       </c>
       <c r="D23" s="23" t="s">
-        <v>23</v>
+        <v>62</v>
       </c>
       <c r="E23" s="21">
         <v>2</v>
@@ -1652,11 +1713,11 @@
         <v>2</v>
       </c>
       <c r="G23" s="21">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H23" s="21">
-        <f>SUM(E23:G23)</f>
-        <v>5</v>
+        <f t="shared" si="1"/>
+        <v>6</v>
       </c>
       <c r="I23" s="9">
         <v>0</v>
@@ -1667,28 +1728,28 @@
       <c r="M23" s="1"/>
       <c r="N23" s="1"/>
     </row>
-    <row r="24" spans="2:14" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:14" ht="47.25" x14ac:dyDescent="0.25">
       <c r="B24" s="9">
-        <f>B23+1</f>
+        <f t="shared" si="2"/>
         <v>19</v>
       </c>
-      <c r="C24" s="26" t="s">
-        <v>9</v>
-      </c>
-      <c r="D24" s="12" t="s">
-        <v>10</v>
+      <c r="C24" s="23" t="s">
+        <v>22</v>
+      </c>
+      <c r="D24" s="23" t="s">
+        <v>23</v>
       </c>
       <c r="E24" s="21">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F24" s="24">
         <v>2</v>
       </c>
       <c r="G24" s="21">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H24" s="21">
-        <f>SUM(E24:G24)</f>
+        <f t="shared" si="1"/>
         <v>5</v>
       </c>
       <c r="I24" s="9">
@@ -1702,25 +1763,27 @@
     </row>
     <row r="25" spans="2:14" ht="31.5" x14ac:dyDescent="0.25">
       <c r="B25" s="9">
-        <f>B24+1</f>
+        <f t="shared" si="2"/>
         <v>20</v>
       </c>
-      <c r="C25" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="D25" s="12"/>
+      <c r="C25" s="26" t="s">
+        <v>9</v>
+      </c>
+      <c r="D25" s="12" t="s">
+        <v>10</v>
+      </c>
       <c r="E25" s="21">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F25" s="24">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G25" s="21">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H25" s="21">
-        <f>SUM(E25:G25)</f>
-        <v>5</v>
+        <f t="shared" si="1"/>
+        <v>7</v>
       </c>
       <c r="I25" s="9">
         <v>0</v>
@@ -1731,32 +1794,30 @@
       <c r="M25" s="1"/>
       <c r="N25" s="1"/>
     </row>
-    <row r="26" spans="2:14" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B26" s="48">
-        <f>B25+1</f>
+    <row r="26" spans="2:14" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="B26" s="9">
+        <f t="shared" si="2"/>
         <v>21</v>
       </c>
-      <c r="C26" s="44" t="s">
-        <v>45</v>
-      </c>
-      <c r="D26" s="50" t="s">
-        <v>46</v>
-      </c>
-      <c r="E26" s="46">
-        <v>2</v>
-      </c>
-      <c r="F26" s="47">
-        <v>1</v>
-      </c>
-      <c r="G26" s="46">
-        <v>1</v>
-      </c>
-      <c r="H26" s="46">
-        <f>SUM(E26:G26)</f>
-        <v>4</v>
-      </c>
-      <c r="I26" s="48">
+      <c r="C26" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="D26" s="12"/>
+      <c r="E26" s="21">
+        <v>1</v>
+      </c>
+      <c r="F26" s="24">
+        <v>1</v>
+      </c>
+      <c r="G26" s="21">
+        <v>3</v>
+      </c>
+      <c r="H26" s="21">
+        <f t="shared" si="1"/>
         <v>5</v>
+      </c>
+      <c r="I26" s="9">
+        <v>0</v>
       </c>
       <c r="J26" s="20"/>
       <c r="K26" s="1"/>
@@ -1764,32 +1825,32 @@
       <c r="M26" s="1"/>
       <c r="N26" s="1"/>
     </row>
-    <row r="27" spans="2:14" ht="47.25" x14ac:dyDescent="0.25">
-      <c r="B27" s="9">
-        <f>B26+1</f>
+    <row r="27" spans="2:14" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B27" s="48">
+        <f t="shared" si="2"/>
         <v>22</v>
       </c>
-      <c r="C27" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="D27" s="12" t="s">
-        <v>44</v>
-      </c>
-      <c r="E27" s="21">
-        <v>2</v>
-      </c>
-      <c r="F27" s="24">
-        <v>1</v>
-      </c>
-      <c r="G27" s="21">
-        <v>1</v>
-      </c>
-      <c r="H27" s="21">
-        <f>SUM(E27:G27)</f>
+      <c r="C27" s="44" t="s">
+        <v>45</v>
+      </c>
+      <c r="D27" s="50" t="s">
+        <v>46</v>
+      </c>
+      <c r="E27" s="46">
+        <v>2</v>
+      </c>
+      <c r="F27" s="47">
+        <v>1</v>
+      </c>
+      <c r="G27" s="46">
+        <v>1</v>
+      </c>
+      <c r="H27" s="46">
+        <f t="shared" si="1"/>
         <v>4</v>
       </c>
-      <c r="I27" s="9">
-        <v>0</v>
+      <c r="I27" s="48">
+        <v>5</v>
       </c>
       <c r="J27" s="20"/>
       <c r="K27" s="1"/>
@@ -1797,28 +1858,28 @@
       <c r="M27" s="1"/>
       <c r="N27" s="1"/>
     </row>
-    <row r="28" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:14" ht="47.25" x14ac:dyDescent="0.25">
       <c r="B28" s="9">
-        <f>B27+1</f>
+        <f t="shared" si="2"/>
         <v>23</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>7</v>
+        <v>43</v>
       </c>
       <c r="D28" s="12" t="s">
-        <v>8</v>
+        <v>44</v>
       </c>
       <c r="E28" s="21">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F28" s="24">
         <v>1</v>
       </c>
       <c r="G28" s="21">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H28" s="21">
-        <f>SUM(E28:G28)</f>
+        <f t="shared" si="1"/>
         <v>4</v>
       </c>
       <c r="I28" s="9">
@@ -1830,16 +1891,16 @@
       <c r="M28" s="1"/>
       <c r="N28" s="1"/>
     </row>
-    <row r="29" spans="2:14" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B29" s="9">
-        <f>B28+1</f>
+        <f t="shared" si="2"/>
         <v>24</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>37</v>
+        <v>7</v>
       </c>
       <c r="D29" s="12" t="s">
-        <v>38</v>
+        <v>8</v>
       </c>
       <c r="E29" s="21">
         <v>1</v>
@@ -1851,7 +1912,7 @@
         <v>2</v>
       </c>
       <c r="H29" s="21">
-        <f>SUM(E29:G29)</f>
+        <f t="shared" si="1"/>
         <v>4</v>
       </c>
       <c r="I29" s="9">
@@ -1865,14 +1926,14 @@
     </row>
     <row r="30" spans="2:14" ht="31.5" x14ac:dyDescent="0.25">
       <c r="B30" s="9">
-        <f>B29+1</f>
+        <f t="shared" si="2"/>
         <v>25</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="D30" s="12" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="E30" s="21">
         <v>1</v>
@@ -1884,7 +1945,7 @@
         <v>2</v>
       </c>
       <c r="H30" s="21">
-        <f>SUM(E30:G30)</f>
+        <f t="shared" si="1"/>
         <v>4</v>
       </c>
       <c r="I30" s="9">
@@ -1898,27 +1959,27 @@
     </row>
     <row r="31" spans="2:14" ht="31.5" x14ac:dyDescent="0.25">
       <c r="B31" s="9">
-        <f>B30+1</f>
+        <f t="shared" si="2"/>
         <v>26</v>
       </c>
-      <c r="C31" s="4" t="s">
-        <v>3</v>
+      <c r="C31" s="5" t="s">
+        <v>41</v>
       </c>
       <c r="D31" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="E31" s="21">
+        <v>1</v>
+      </c>
+      <c r="F31" s="24">
+        <v>1</v>
+      </c>
+      <c r="G31" s="21">
+        <v>2</v>
+      </c>
+      <c r="H31" s="21">
+        <f t="shared" si="1"/>
         <v>4</v>
-      </c>
-      <c r="E31" s="21">
-        <v>1</v>
-      </c>
-      <c r="F31" s="24">
-        <v>1</v>
-      </c>
-      <c r="G31" s="21">
-        <v>1</v>
-      </c>
-      <c r="H31" s="21">
-        <f>SUM(E31:G31)</f>
-        <v>3</v>
       </c>
       <c r="I31" s="9">
         <v>0</v>
@@ -1929,15 +1990,17 @@
       <c r="M31" s="1"/>
       <c r="N31" s="1"/>
     </row>
-    <row r="32" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:14" ht="31.5" x14ac:dyDescent="0.25">
       <c r="B32" s="9">
-        <f>B31+1</f>
+        <f t="shared" si="2"/>
         <v>27</v>
       </c>
-      <c r="C32" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="D32" s="12"/>
+      <c r="C32" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="D32" s="12" t="s">
+        <v>4</v>
+      </c>
       <c r="E32" s="21">
         <v>1</v>
       </c>
@@ -1948,7 +2011,7 @@
         <v>1</v>
       </c>
       <c r="H32" s="21">
-        <f>SUM(E32:G32)</f>
+        <f t="shared" si="1"/>
         <v>3</v>
       </c>
       <c r="I32" s="9">
@@ -1960,29 +2023,29 @@
       <c r="M32" s="1"/>
       <c r="N32" s="1"/>
     </row>
-    <row r="33" spans="2:14" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B33" s="9">
-        <f>B32+1</f>
+        <f t="shared" si="2"/>
         <v>28</v>
       </c>
-      <c r="C33" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="D33" s="13"/>
-      <c r="E33" s="22">
-        <v>1</v>
-      </c>
-      <c r="F33" s="25">
-        <v>1</v>
-      </c>
-      <c r="G33" s="22">
-        <v>1</v>
-      </c>
-      <c r="H33" s="22">
-        <f>SUM(E33:G33)</f>
+      <c r="C33" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D33" s="12"/>
+      <c r="E33" s="21">
+        <v>1</v>
+      </c>
+      <c r="F33" s="24">
+        <v>1</v>
+      </c>
+      <c r="G33" s="21">
+        <v>1</v>
+      </c>
+      <c r="H33" s="21">
+        <f t="shared" si="1"/>
         <v>3</v>
       </c>
-      <c r="I33" s="28">
+      <c r="I33" s="9">
         <v>0</v>
       </c>
       <c r="J33" s="20"/>
@@ -1991,8 +2054,31 @@
       <c r="M33" s="1"/>
       <c r="N33" s="1"/>
     </row>
-    <row r="34" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="I34" s="10"/>
+    <row r="34" spans="2:14" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B34" s="9">
+        <f t="shared" si="2"/>
+        <v>29</v>
+      </c>
+      <c r="C34" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="D34" s="13"/>
+      <c r="E34" s="22">
+        <v>1</v>
+      </c>
+      <c r="F34" s="25">
+        <v>1</v>
+      </c>
+      <c r="G34" s="22">
+        <v>1</v>
+      </c>
+      <c r="H34" s="22">
+        <f t="shared" si="1"/>
+        <v>3</v>
+      </c>
+      <c r="I34" s="28">
+        <v>0</v>
+      </c>
       <c r="J34" s="20"/>
       <c r="K34" s="1"/>
       <c r="L34" s="1"/>
@@ -2000,13 +2086,6 @@
       <c r="N34" s="1"/>
     </row>
     <row r="35" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B35" s="10"/>
-      <c r="C35" s="26"/>
-      <c r="D35" s="27"/>
-      <c r="E35" s="20"/>
-      <c r="F35" s="20"/>
-      <c r="G35" s="20"/>
-      <c r="H35" s="20"/>
       <c r="I35" s="10"/>
       <c r="J35" s="20"/>
       <c r="K35" s="1"/>
@@ -2015,13 +2094,13 @@
       <c r="N35" s="1"/>
     </row>
     <row r="36" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B36" s="1"/>
-      <c r="C36" s="7"/>
-      <c r="D36" s="2"/>
-      <c r="E36" s="10"/>
-      <c r="F36" s="10"/>
-      <c r="G36" s="10"/>
-      <c r="H36" s="10"/>
+      <c r="B36" s="10"/>
+      <c r="C36" s="26"/>
+      <c r="D36" s="27"/>
+      <c r="E36" s="20"/>
+      <c r="F36" s="20"/>
+      <c r="G36" s="20"/>
+      <c r="H36" s="20"/>
       <c r="I36" s="10"/>
       <c r="J36" s="20"/>
       <c r="K36" s="1"/>
@@ -2164,8 +2243,23 @@
       <c r="M45" s="1"/>
       <c r="N45" s="1"/>
     </row>
+    <row r="46" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B46" s="1"/>
+      <c r="C46" s="7"/>
+      <c r="D46" s="2"/>
+      <c r="E46" s="10"/>
+      <c r="F46" s="10"/>
+      <c r="G46" s="10"/>
+      <c r="H46" s="10"/>
+      <c r="I46" s="10"/>
+      <c r="J46" s="20"/>
+      <c r="K46" s="1"/>
+      <c r="L46" s="1"/>
+      <c r="M46" s="1"/>
+      <c r="N46" s="1"/>
+    </row>
   </sheetData>
-  <autoFilter ref="B3:I33" xr:uid="{11BA4F79-2AB7-4A24-A4BE-758442E1F8CB}">
+  <autoFilter ref="B3:I34" xr:uid="{11BA4F79-2AB7-4A24-A4BE-758442E1F8CB}">
     <filterColumn colId="7">
       <filters>
         <filter val="0"/>
@@ -2173,16 +2267,16 @@
         <filter val="2"/>
       </filters>
     </filterColumn>
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B5:I33">
-      <sortCondition descending="1" ref="H4:H33"/>
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B5:I34">
+      <sortCondition descending="1" ref="H4:H34"/>
     </sortState>
   </autoFilter>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B4:I33">
-    <sortCondition descending="1" ref="H4:H33"/>
-    <sortCondition descending="1" ref="E4:E33"/>
-    <sortCondition descending="1" ref="F4:F33"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B4:I34">
+    <sortCondition descending="1" ref="H4:H34"/>
+    <sortCondition descending="1" ref="E4:E34"/>
+    <sortCondition descending="1" ref="F4:F34"/>
   </sortState>
-  <conditionalFormatting sqref="H4:H33">
+  <conditionalFormatting sqref="H4:H34">
     <cfRule type="colorScale" priority="3">
       <colorScale>
         <cfvo type="min"/>
@@ -2194,7 +2288,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I4:I33">
+  <conditionalFormatting sqref="I4:I34">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>

</xml_diff>

<commit_message>
Fixed non-highlighted clusters disappearing
</commit_message>
<xml_diff>
--- a/Future Features/New Features - Family Tree.xlsx
+++ b/Future Features/New Features - Family Tree.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://srcincgov1-my.sharepoint.us/personal/lauko_srcinc_com/Documents/Desktop/Personal/geneology/GED Keepers/Future Features/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="357" documentId="8_{D1FEEEA7-0E84-49B9-AD17-37D0BB95FB37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{01D614A8-5669-433A-811D-6F7593E59CDC}"/>
+  <xr:revisionPtr revIDLastSave="373" documentId="8_{D1FEEEA7-0E84-49B9-AD17-37D0BB95FB37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8049F723-D40B-4A4A-9C96-8BE3D47123ED}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{8067922A-00B7-4646-9500-13902203F407}"/>
+    <workbookView xWindow="1260" yWindow="150" windowWidth="26700" windowHeight="13980" xr2:uid="{8067922A-00B7-4646-9500-13902203F407}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$B$3:$I$34</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$B$3:$I$35</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="74">
   <si>
     <t>Feature</t>
   </si>
@@ -161,9 +161,6 @@
     <t>clean up side panel, aesthetically</t>
   </si>
   <si>
-    <t xml:space="preserve">dividers between sections, consistent fonts </t>
-  </si>
-  <si>
     <t xml:space="preserve">Add shrinking and expanding components to the right hadnd </t>
   </si>
   <si>
@@ -255,6 +252,15 @@
   </si>
   <si>
     <t>clicks are working, not bad for a tablet, need to optimize for screenspace on phone</t>
+  </si>
+  <si>
+    <t>Clean up cluster area since only using Birth Clusters</t>
+  </si>
+  <si>
+    <t>Add Help Button</t>
+  </si>
+  <si>
+    <t>add a button that will launch guided tour</t>
   </si>
 </sst>
 </file>
@@ -639,7 +645,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -977,7 +983,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{11BA4F79-2AB7-4A24-A4BE-758442E1F8CB}">
   <sheetPr filterMode="1"/>
-  <dimension ref="B1:N46"/>
+  <dimension ref="B1:N47"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="49.28515625" style="8" customWidth="1"/>
@@ -1008,7 +1014,7 @@
       </c>
       <c r="H2" s="20"/>
       <c r="I2" s="10" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="J2" s="20"/>
       <c r="K2" s="1"/>
@@ -1037,7 +1043,7 @@
         <v>18</v>
       </c>
       <c r="I3" s="16" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="J3" s="20"/>
       <c r="K3" s="2"/>
@@ -1050,10 +1056,10 @@
         <v>1</v>
       </c>
       <c r="C4" s="36" t="s">
+        <v>49</v>
+      </c>
+      <c r="D4" s="37" t="s">
         <v>50</v>
-      </c>
-      <c r="D4" s="37" t="s">
-        <v>51</v>
       </c>
       <c r="E4" s="38">
         <v>3</v>
@@ -1083,10 +1089,10 @@
         <v>2</v>
       </c>
       <c r="C5" s="35" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D5" s="35" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E5" s="42">
         <v>3</v>
@@ -1105,7 +1111,7 @@
         <v>3</v>
       </c>
       <c r="J5" s="20" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="K5" s="1"/>
       <c r="L5" s="1"/>
@@ -1118,10 +1124,10 @@
         <v>3</v>
       </c>
       <c r="C6" s="44" t="s">
+        <v>54</v>
+      </c>
+      <c r="D6" s="45" t="s">
         <v>55</v>
-      </c>
-      <c r="D6" s="45" t="s">
-        <v>56</v>
       </c>
       <c r="E6" s="46">
         <v>3</v>
@@ -1178,16 +1184,16 @@
       <c r="M7" s="1"/>
       <c r="N7" s="1"/>
     </row>
-    <row r="8" spans="2:14" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B8" s="9">
         <f>B7+1</f>
         <v>5</v>
       </c>
-      <c r="C8" s="4" t="s">
-        <v>25</v>
+      <c r="C8" s="5" t="s">
+        <v>72</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>24</v>
+        <v>73</v>
       </c>
       <c r="E8" s="21">
         <v>3</v>
@@ -1196,39 +1202,38 @@
         <v>2</v>
       </c>
       <c r="G8" s="21">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H8" s="21">
         <f>SUM(E8:G8)</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="I8" s="9">
-        <v>1</v>
-      </c>
-      <c r="J8" s="20"/>
+        <v>0</v>
+      </c>
       <c r="K8" s="1"/>
       <c r="L8" s="1"/>
       <c r="M8" s="1"/>
       <c r="N8" s="1"/>
     </row>
-    <row r="9" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:14" ht="31.5" x14ac:dyDescent="0.25">
       <c r="B9" s="9">
         <f>B8+1</f>
         <v>6</v>
       </c>
-      <c r="C9" s="35" t="s">
-        <v>53</v>
-      </c>
-      <c r="D9" s="35" t="s">
-        <v>54</v>
-      </c>
-      <c r="E9" s="42">
-        <v>3</v>
-      </c>
-      <c r="F9" s="43">
-        <v>2</v>
-      </c>
-      <c r="G9" s="42">
+      <c r="C9" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="D9" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="E9" s="21">
+        <v>3</v>
+      </c>
+      <c r="F9" s="24">
+        <v>2</v>
+      </c>
+      <c r="G9" s="21">
         <v>2</v>
       </c>
       <c r="H9" s="21">
@@ -1236,7 +1241,7 @@
         <v>7</v>
       </c>
       <c r="I9" s="9">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J9" s="20"/>
       <c r="K9" s="1"/>
@@ -1250,7 +1255,7 @@
         <v>7</v>
       </c>
       <c r="C10" s="49" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D10" s="50"/>
       <c r="E10" s="46">
@@ -1270,7 +1275,7 @@
         <v>5</v>
       </c>
       <c r="J10" s="20" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="K10" s="1"/>
       <c r="L10" s="1"/>
@@ -1310,24 +1315,24 @@
       <c r="M11" s="1"/>
       <c r="N11" s="1"/>
     </row>
-    <row r="12" spans="2:14" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B12" s="9">
         <f>B11+1</f>
         <v>9</v>
       </c>
-      <c r="C12" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="D12" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="E12" s="21">
-        <v>3</v>
-      </c>
-      <c r="F12" s="24">
-        <v>2</v>
-      </c>
-      <c r="G12" s="21">
+      <c r="C12" s="35" t="s">
+        <v>52</v>
+      </c>
+      <c r="D12" s="35" t="s">
+        <v>53</v>
+      </c>
+      <c r="E12" s="42">
+        <v>3</v>
+      </c>
+      <c r="F12" s="43">
+        <v>2</v>
+      </c>
+      <c r="G12" s="42">
         <v>2</v>
       </c>
       <c r="H12" s="21">
@@ -1335,29 +1340,29 @@
         <v>7</v>
       </c>
       <c r="I12" s="9">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="J12" s="41" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="K12" s="1"/>
       <c r="L12" s="1"/>
       <c r="M12" s="1"/>
       <c r="N12" s="1"/>
     </row>
-    <row r="13" spans="2:14" ht="78.75" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:14" ht="31.5" x14ac:dyDescent="0.25">
       <c r="B13" s="9">
-        <f>B11+1</f>
+        <f>B12+1</f>
+        <v>10</v>
+      </c>
+      <c r="C13" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="C13" s="4" t="s">
-        <v>30</v>
-      </c>
       <c r="D13" s="12" t="s">
-        <v>35</v>
+        <v>10</v>
       </c>
       <c r="E13" s="21">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F13" s="24">
         <v>2</v>
@@ -1367,7 +1372,7 @@
       </c>
       <c r="H13" s="21">
         <f>SUM(E13:G13)</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I13" s="9">
         <v>0</v>
@@ -1377,54 +1382,55 @@
       <c r="M13" s="1"/>
       <c r="N13" s="1"/>
     </row>
-    <row r="14" spans="2:14" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B14" s="9">
         <f>B13+1</f>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>5</v>
+        <v>67</v>
       </c>
       <c r="D14" s="12" t="s">
-        <v>6</v>
+        <v>68</v>
       </c>
       <c r="E14" s="21">
         <v>3</v>
       </c>
       <c r="F14" s="24">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G14" s="21">
         <v>2</v>
       </c>
       <c r="H14" s="21">
         <f>SUM(E14:G14)</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I14" s="9">
         <v>0</v>
       </c>
+      <c r="J14" s="20"/>
       <c r="K14" s="1"/>
       <c r="L14" s="1"/>
       <c r="M14" s="1"/>
       <c r="N14" s="1"/>
     </row>
-    <row r="15" spans="2:14" ht="78.75" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:14" ht="31.5" x14ac:dyDescent="0.25">
       <c r="B15" s="9">
         <f>B14+1</f>
+        <v>12</v>
+      </c>
+      <c r="C15" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="C15" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="D15" s="12" t="s">
-        <v>34</v>
+      <c r="D15" s="5" t="s">
+        <v>12</v>
       </c>
       <c r="E15" s="21">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F15" s="24">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G15" s="21">
         <v>2</v>
@@ -1437,23 +1443,23 @@
         <v>2</v>
       </c>
       <c r="J15" s="20" t="s">
-        <v>52</v>
+        <v>63</v>
       </c>
       <c r="K15" s="1"/>
       <c r="L15" s="1"/>
       <c r="M15" s="1"/>
       <c r="N15" s="1"/>
     </row>
-    <row r="16" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:14" ht="31.5" x14ac:dyDescent="0.25">
       <c r="B16" s="9">
         <f>B15+1</f>
-        <v>12</v>
-      </c>
-      <c r="C16" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="D16" s="12" t="s">
-        <v>69</v>
+        <v>13</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="D16" s="23" t="s">
+        <v>21</v>
       </c>
       <c r="E16" s="21">
         <v>2</v>
@@ -1480,13 +1486,13 @@
     <row r="17" spans="2:14" ht="31.5" x14ac:dyDescent="0.25">
       <c r="B17" s="9">
         <f>B16+1</f>
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="D17" s="5" t="s">
-        <v>12</v>
+        <v>56</v>
+      </c>
+      <c r="D17" s="23" t="s">
+        <v>57</v>
       </c>
       <c r="E17" s="21">
         <v>2</v>
@@ -1502,26 +1508,24 @@
         <v>6</v>
       </c>
       <c r="I17" s="9">
-        <v>2</v>
-      </c>
-      <c r="J17" s="20" t="s">
-        <v>64</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="J17" s="20"/>
       <c r="K17" s="1"/>
       <c r="L17" s="1"/>
       <c r="M17" s="1"/>
       <c r="N17" s="1"/>
     </row>
-    <row r="18" spans="2:14" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:14" ht="47.25" x14ac:dyDescent="0.25">
       <c r="B18" s="9">
         <f>B17+1</f>
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="D18" s="23" t="s">
-        <v>21</v>
+        <v>36</v>
+      </c>
+      <c r="D18" s="5" t="s">
+        <v>48</v>
       </c>
       <c r="E18" s="21">
         <v>2</v>
@@ -1545,25 +1549,25 @@
       <c r="M18" s="1"/>
       <c r="N18" s="1"/>
     </row>
-    <row r="19" spans="2:14" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B19" s="9">
         <f>B18+1</f>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="D19" s="23" t="s">
-        <v>58</v>
+        <v>39</v>
+      </c>
+      <c r="D19" s="12" t="s">
+        <v>71</v>
       </c>
       <c r="E19" s="21">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F19" s="24">
         <v>2</v>
       </c>
       <c r="G19" s="21">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H19" s="21">
         <f>SUM(E19:G19)</f>
@@ -1578,16 +1582,16 @@
       <c r="M19" s="1"/>
       <c r="N19" s="1"/>
     </row>
-    <row r="20" spans="2:14" ht="83.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:14" ht="47.25" x14ac:dyDescent="0.25">
       <c r="B20" s="9">
         <f>B19+1</f>
-        <v>16</v>
-      </c>
-      <c r="C20" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="D20" s="5" t="s">
-        <v>49</v>
+        <v>17</v>
+      </c>
+      <c r="C20" s="23" t="s">
+        <v>22</v>
+      </c>
+      <c r="D20" s="23" t="s">
+        <v>23</v>
       </c>
       <c r="E20" s="21">
         <v>2</v>
@@ -1596,11 +1600,11 @@
         <v>2</v>
       </c>
       <c r="G20" s="21">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H20" s="21">
         <f>SUM(E20:G20)</f>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I20" s="9">
         <v>0</v>
@@ -1611,65 +1615,64 @@
       <c r="M20" s="1"/>
       <c r="N20" s="1"/>
     </row>
-    <row r="21" spans="2:14" ht="83.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="29">
+    <row r="21" spans="2:14" ht="83.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B21" s="9">
         <f>B20+1</f>
-        <v>17</v>
-      </c>
-      <c r="C21" s="30" t="s">
-        <v>31</v>
-      </c>
-      <c r="D21" s="31" t="s">
-        <v>32</v>
-      </c>
-      <c r="E21" s="32">
-        <v>2</v>
-      </c>
-      <c r="F21" s="33">
-        <v>1</v>
-      </c>
-      <c r="G21" s="32">
-        <v>3</v>
-      </c>
-      <c r="H21" s="32">
+        <v>18</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="D21" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="E21" s="21">
+        <v>1</v>
+      </c>
+      <c r="F21" s="24">
+        <v>2</v>
+      </c>
+      <c r="G21" s="21">
+        <v>2</v>
+      </c>
+      <c r="H21" s="21">
         <f>SUM(E21:G21)</f>
-        <v>6</v>
-      </c>
-      <c r="I21" s="34">
         <v>5</v>
       </c>
-      <c r="J21" s="20"/>
+      <c r="I21" s="9">
+        <v>0</v>
+      </c>
       <c r="K21" s="1"/>
       <c r="L21" s="1"/>
       <c r="M21" s="1"/>
       <c r="N21" s="1"/>
     </row>
-    <row r="22" spans="2:14" ht="83.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B22" s="9">
+    <row r="22" spans="2:14" ht="83.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B22" s="29">
         <f>B21+1</f>
-        <v>18</v>
-      </c>
-      <c r="C22" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="D22" s="12" t="s">
-        <v>40</v>
-      </c>
-      <c r="E22" s="21">
-        <v>1</v>
-      </c>
-      <c r="F22" s="24">
-        <v>2</v>
-      </c>
-      <c r="G22" s="21">
-        <v>3</v>
-      </c>
-      <c r="H22" s="21">
+        <v>19</v>
+      </c>
+      <c r="C22" s="30" t="s">
+        <v>31</v>
+      </c>
+      <c r="D22" s="31" t="s">
+        <v>32</v>
+      </c>
+      <c r="E22" s="32">
+        <v>2</v>
+      </c>
+      <c r="F22" s="33">
+        <v>1</v>
+      </c>
+      <c r="G22" s="32">
+        <v>3</v>
+      </c>
+      <c r="H22" s="32">
         <f>SUM(E22:G22)</f>
         <v>6</v>
       </c>
-      <c r="I22" s="9">
-        <v>0</v>
+      <c r="I22" s="34">
+        <v>5</v>
       </c>
       <c r="J22" s="20"/>
       <c r="K22" s="1"/>
@@ -1677,32 +1680,30 @@
       <c r="M22" s="1"/>
       <c r="N22" s="1"/>
     </row>
-    <row r="23" spans="2:14" ht="83.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="34">
-        <f>B22+1</f>
+    <row r="23" spans="2:14" ht="83.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B23" s="9">
+        <f>B21+1</f>
         <v>19</v>
       </c>
-      <c r="C23" s="54" t="s">
-        <v>63</v>
-      </c>
-      <c r="D23" s="55" t="s">
-        <v>62</v>
-      </c>
-      <c r="E23" s="32">
-        <v>2</v>
-      </c>
-      <c r="F23" s="33">
-        <v>2</v>
-      </c>
-      <c r="G23" s="32">
-        <v>2</v>
-      </c>
-      <c r="H23" s="32">
+      <c r="C23" s="35" t="s">
+        <v>64</v>
+      </c>
+      <c r="D23" s="51"/>
+      <c r="E23" s="52">
+        <v>1</v>
+      </c>
+      <c r="F23" s="53">
+        <v>1</v>
+      </c>
+      <c r="G23" s="52">
+        <v>3</v>
+      </c>
+      <c r="H23" s="52">
         <f>SUM(E23:G23)</f>
-        <v>6</v>
-      </c>
-      <c r="I23" s="34">
         <v>5</v>
+      </c>
+      <c r="I23" s="9">
+        <v>0</v>
       </c>
       <c r="J23" s="20"/>
       <c r="K23" s="1"/>
@@ -1710,30 +1711,32 @@
       <c r="M23" s="1"/>
       <c r="N23" s="1"/>
     </row>
-    <row r="24" spans="2:14" ht="47.25" x14ac:dyDescent="0.25">
-      <c r="B24" s="9">
-        <f>B22+1</f>
-        <v>19</v>
-      </c>
-      <c r="C24" s="35" t="s">
-        <v>65</v>
-      </c>
-      <c r="D24" s="51"/>
-      <c r="E24" s="52">
-        <v>1</v>
-      </c>
-      <c r="F24" s="53">
-        <v>1</v>
-      </c>
-      <c r="G24" s="52">
-        <v>3</v>
-      </c>
-      <c r="H24" s="52">
+    <row r="24" spans="2:14" ht="83.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B24" s="34">
+        <f>B23+1</f>
+        <v>20</v>
+      </c>
+      <c r="C24" s="54" t="s">
+        <v>62</v>
+      </c>
+      <c r="D24" s="55" t="s">
+        <v>61</v>
+      </c>
+      <c r="E24" s="32">
+        <v>2</v>
+      </c>
+      <c r="F24" s="33">
+        <v>2</v>
+      </c>
+      <c r="G24" s="32">
+        <v>2</v>
+      </c>
+      <c r="H24" s="32">
         <f>SUM(E24:G24)</f>
+        <v>6</v>
+      </c>
+      <c r="I24" s="34">
         <v>5</v>
-      </c>
-      <c r="I24" s="9">
-        <v>0</v>
       </c>
       <c r="J24" s="20"/>
       <c r="K24" s="1"/>
@@ -1741,25 +1744,23 @@
       <c r="M24" s="1"/>
       <c r="N24" s="1"/>
     </row>
-    <row r="25" spans="2:14" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:14" ht="31.5" x14ac:dyDescent="0.25">
       <c r="B25" s="9">
         <f>B24+1</f>
-        <v>20</v>
-      </c>
-      <c r="C25" s="56" t="s">
-        <v>22</v>
-      </c>
-      <c r="D25" s="23" t="s">
-        <v>23</v>
-      </c>
+        <v>21</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="D25" s="12"/>
       <c r="E25" s="21">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F25" s="24">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G25" s="21">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H25" s="21">
         <f>SUM(E25:G25)</f>
@@ -1774,27 +1775,29 @@
       <c r="M25" s="1"/>
       <c r="N25" s="1"/>
     </row>
-    <row r="26" spans="2:14" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:14" ht="47.25" x14ac:dyDescent="0.25">
       <c r="B26" s="9">
         <f>B25+1</f>
-        <v>21</v>
-      </c>
-      <c r="C26" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="D26" s="12"/>
+        <v>22</v>
+      </c>
+      <c r="C26" s="56" t="s">
+        <v>42</v>
+      </c>
+      <c r="D26" s="12" t="s">
+        <v>43</v>
+      </c>
       <c r="E26" s="21">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F26" s="24">
         <v>1</v>
       </c>
       <c r="G26" s="21">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H26" s="21">
         <f>SUM(E26:G26)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I26" s="9">
         <v>0</v>
@@ -1805,65 +1808,64 @@
       <c r="M26" s="1"/>
       <c r="N26" s="1"/>
     </row>
-    <row r="27" spans="2:14" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B27" s="48">
+    <row r="27" spans="2:14" ht="47.25" x14ac:dyDescent="0.25">
+      <c r="B27" s="9">
         <f>B26+1</f>
-        <v>22</v>
-      </c>
-      <c r="C27" s="44" t="s">
-        <v>45</v>
-      </c>
-      <c r="D27" s="50" t="s">
-        <v>46</v>
-      </c>
-      <c r="E27" s="46">
-        <v>2</v>
-      </c>
-      <c r="F27" s="47">
-        <v>1</v>
-      </c>
-      <c r="G27" s="46">
-        <v>1</v>
-      </c>
-      <c r="H27" s="46">
+        <v>23</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="D27" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="E27" s="21">
+        <v>1</v>
+      </c>
+      <c r="F27" s="24">
+        <v>1</v>
+      </c>
+      <c r="G27" s="21">
+        <v>2</v>
+      </c>
+      <c r="H27" s="21">
         <f>SUM(E27:G27)</f>
         <v>4</v>
       </c>
-      <c r="I27" s="48">
-        <v>5</v>
-      </c>
-      <c r="J27" s="20"/>
+      <c r="I27" s="9">
+        <v>0</v>
+      </c>
       <c r="K27" s="1"/>
       <c r="L27" s="1"/>
       <c r="M27" s="1"/>
       <c r="N27" s="1"/>
     </row>
-    <row r="28" spans="2:14" ht="47.25" x14ac:dyDescent="0.25">
-      <c r="B28" s="9">
+    <row r="28" spans="2:14" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B28" s="48">
         <f>B27+1</f>
-        <v>23</v>
-      </c>
-      <c r="C28" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="D28" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="C28" s="44" t="s">
         <v>44</v>
       </c>
-      <c r="E28" s="21">
-        <v>2</v>
-      </c>
-      <c r="F28" s="24">
-        <v>1</v>
-      </c>
-      <c r="G28" s="21">
-        <v>1</v>
-      </c>
-      <c r="H28" s="21">
+      <c r="D28" s="50" t="s">
+        <v>45</v>
+      </c>
+      <c r="E28" s="46">
+        <v>2</v>
+      </c>
+      <c r="F28" s="47">
+        <v>1</v>
+      </c>
+      <c r="G28" s="46">
+        <v>1</v>
+      </c>
+      <c r="H28" s="46">
         <f>SUM(E28:G28)</f>
         <v>4</v>
       </c>
-      <c r="I28" s="9">
-        <v>0</v>
+      <c r="I28" s="48">
+        <v>5</v>
       </c>
       <c r="J28" s="20"/>
       <c r="K28" s="1"/>
@@ -1871,16 +1873,16 @@
       <c r="M28" s="1"/>
       <c r="N28" s="1"/>
     </row>
-    <row r="29" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:14" ht="78.75" x14ac:dyDescent="0.25">
       <c r="B29" s="9">
         <f>B28+1</f>
-        <v>24</v>
-      </c>
-      <c r="C29" s="5" t="s">
-        <v>7</v>
+        <v>25</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>33</v>
       </c>
       <c r="D29" s="12" t="s">
-        <v>8</v>
+        <v>34</v>
       </c>
       <c r="E29" s="21">
         <v>1</v>
@@ -1896,24 +1898,26 @@
         <v>4</v>
       </c>
       <c r="I29" s="9">
-        <v>0</v>
-      </c>
-      <c r="J29" s="20"/>
+        <v>2</v>
+      </c>
+      <c r="J29" s="20" t="s">
+        <v>51</v>
+      </c>
       <c r="K29" s="1"/>
       <c r="L29" s="1"/>
       <c r="M29" s="1"/>
       <c r="N29" s="1"/>
     </row>
-    <row r="30" spans="2:14" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B30" s="9">
         <f>B29+1</f>
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>37</v>
+        <v>7</v>
       </c>
       <c r="D30" s="12" t="s">
-        <v>38</v>
+        <v>8</v>
       </c>
       <c r="E30" s="21">
         <v>1</v>
@@ -1940,13 +1944,13 @@
     <row r="31" spans="2:14" ht="31.5" x14ac:dyDescent="0.25">
       <c r="B31" s="9">
         <f>B30+1</f>
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="D31" s="12" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="E31" s="21">
         <v>1</v>
@@ -1973,13 +1977,13 @@
     <row r="32" spans="2:14" ht="31.5" x14ac:dyDescent="0.25">
       <c r="B32" s="9">
         <f>B31+1</f>
-        <v>27</v>
-      </c>
-      <c r="C32" s="4" t="s">
-        <v>3</v>
+        <v>28</v>
+      </c>
+      <c r="C32" s="5" t="s">
+        <v>40</v>
       </c>
       <c r="D32" s="12" t="s">
-        <v>4</v>
+        <v>41</v>
       </c>
       <c r="E32" s="21">
         <v>1</v>
@@ -1988,11 +1992,11 @@
         <v>1</v>
       </c>
       <c r="G32" s="21">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H32" s="21">
         <f>SUM(E32:G32)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I32" s="9">
         <v>0</v>
@@ -2003,15 +2007,17 @@
       <c r="M32" s="1"/>
       <c r="N32" s="1"/>
     </row>
-    <row r="33" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:14" ht="31.5" x14ac:dyDescent="0.25">
       <c r="B33" s="9">
         <f>B32+1</f>
-        <v>28</v>
-      </c>
-      <c r="C33" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="D33" s="12"/>
+        <v>29</v>
+      </c>
+      <c r="C33" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="D33" s="12" t="s">
+        <v>4</v>
+      </c>
       <c r="E33" s="21">
         <v>1</v>
       </c>
@@ -2034,29 +2040,29 @@
       <c r="M33" s="1"/>
       <c r="N33" s="1"/>
     </row>
-    <row r="34" spans="2:14" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B34" s="9">
         <f>B33+1</f>
-        <v>29</v>
-      </c>
-      <c r="C34" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="D34" s="13"/>
-      <c r="E34" s="22">
-        <v>1</v>
-      </c>
-      <c r="F34" s="25">
-        <v>1</v>
-      </c>
-      <c r="G34" s="22">
-        <v>1</v>
-      </c>
-      <c r="H34" s="22">
+        <v>30</v>
+      </c>
+      <c r="C34" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D34" s="12"/>
+      <c r="E34" s="21">
+        <v>1</v>
+      </c>
+      <c r="F34" s="24">
+        <v>1</v>
+      </c>
+      <c r="G34" s="21">
+        <v>1</v>
+      </c>
+      <c r="H34" s="21">
         <f>SUM(E34:G34)</f>
         <v>3</v>
       </c>
-      <c r="I34" s="28">
+      <c r="I34" s="9">
         <v>0</v>
       </c>
       <c r="J34" s="20"/>
@@ -2065,8 +2071,31 @@
       <c r="M34" s="1"/>
       <c r="N34" s="1"/>
     </row>
-    <row r="35" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="I35" s="10"/>
+    <row r="35" spans="2:14" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B35" s="9">
+        <f>B34+1</f>
+        <v>31</v>
+      </c>
+      <c r="C35" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="D35" s="13"/>
+      <c r="E35" s="22">
+        <v>1</v>
+      </c>
+      <c r="F35" s="25">
+        <v>1</v>
+      </c>
+      <c r="G35" s="22">
+        <v>1</v>
+      </c>
+      <c r="H35" s="22">
+        <f>SUM(E35:G35)</f>
+        <v>3</v>
+      </c>
+      <c r="I35" s="28">
+        <v>0</v>
+      </c>
       <c r="J35" s="20"/>
       <c r="K35" s="1"/>
       <c r="L35" s="1"/>
@@ -2074,13 +2103,6 @@
       <c r="N35" s="1"/>
     </row>
     <row r="36" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B36" s="10"/>
-      <c r="C36" s="26"/>
-      <c r="D36" s="27"/>
-      <c r="E36" s="20"/>
-      <c r="F36" s="20"/>
-      <c r="G36" s="20"/>
-      <c r="H36" s="20"/>
       <c r="I36" s="10"/>
       <c r="J36" s="20"/>
       <c r="K36" s="1"/>
@@ -2089,13 +2111,13 @@
       <c r="N36" s="1"/>
     </row>
     <row r="37" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B37" s="1"/>
-      <c r="C37" s="7"/>
-      <c r="D37" s="2"/>
-      <c r="E37" s="10"/>
-      <c r="F37" s="10"/>
-      <c r="G37" s="10"/>
-      <c r="H37" s="10"/>
+      <c r="B37" s="10"/>
+      <c r="C37" s="26"/>
+      <c r="D37" s="27"/>
+      <c r="E37" s="20"/>
+      <c r="F37" s="20"/>
+      <c r="G37" s="20"/>
+      <c r="H37" s="20"/>
       <c r="I37" s="10"/>
       <c r="J37" s="20"/>
       <c r="K37" s="1"/>
@@ -2238,8 +2260,23 @@
       <c r="M46" s="1"/>
       <c r="N46" s="1"/>
     </row>
+    <row r="47" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B47" s="1"/>
+      <c r="C47" s="7"/>
+      <c r="D47" s="2"/>
+      <c r="E47" s="10"/>
+      <c r="F47" s="10"/>
+      <c r="G47" s="10"/>
+      <c r="H47" s="10"/>
+      <c r="I47" s="10"/>
+      <c r="J47" s="20"/>
+      <c r="K47" s="1"/>
+      <c r="L47" s="1"/>
+      <c r="M47" s="1"/>
+      <c r="N47" s="1"/>
+    </row>
   </sheetData>
-  <autoFilter ref="B3:I34" xr:uid="{11BA4F79-2AB7-4A24-A4BE-758442E1F8CB}">
+  <autoFilter ref="B3:I35" xr:uid="{11BA4F79-2AB7-4A24-A4BE-758442E1F8CB}">
     <filterColumn colId="7">
       <filters>
         <filter val="0"/>
@@ -2247,16 +2284,16 @@
         <filter val="2"/>
       </filters>
     </filterColumn>
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B5:I34">
-      <sortCondition descending="1" ref="H4:H34"/>
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B5:I35">
+      <sortCondition descending="1" ref="H4:H35"/>
     </sortState>
   </autoFilter>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B4:I34">
-    <sortCondition descending="1" ref="H4:H34"/>
-    <sortCondition descending="1" ref="E4:E34"/>
-    <sortCondition descending="1" ref="F4:F34"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B5:J35">
+    <sortCondition descending="1" ref="H4:H35"/>
+    <sortCondition descending="1" ref="E4:E35"/>
+    <sortCondition descending="1" ref="F4:F35"/>
   </sortState>
-  <conditionalFormatting sqref="H4:H34">
+  <conditionalFormatting sqref="H4:H35">
     <cfRule type="colorScale" priority="3">
       <colorScale>
         <cfvo type="min"/>
@@ -2268,7 +2305,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I4:I34">
+  <conditionalFormatting sqref="I4:I35">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>

</xml_diff>

<commit_message>
Fixed bug on startup around spouses
Fixed error on startup.  Was not creating nodes for spouses of descendants
</commit_message>
<xml_diff>
--- a/Future Features/New Features - Family Tree.xlsx
+++ b/Future Features/New Features - Family Tree.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://srcincgov1-my.sharepoint.us/personal/lauko_srcinc_com/Documents/Desktop/Personal/geneology/GED Keepers/Future Features/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="382" documentId="8_{D1FEEEA7-0E84-49B9-AD17-37D0BB95FB37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{24EFBADC-D4BA-495B-AF58-34CB81242483}"/>
+  <xr:revisionPtr revIDLastSave="395" documentId="8_{D1FEEEA7-0E84-49B9-AD17-37D0BB95FB37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AE2D1D0E-B6BB-4B28-801B-D0551587A1FC}"/>
   <bookViews>
-    <workbookView xWindow="1260" yWindow="150" windowWidth="26700" windowHeight="13980" xr2:uid="{8067922A-00B7-4646-9500-13902203F407}"/>
+    <workbookView xWindow="15" yWindow="0" windowWidth="23010" windowHeight="12330" xr2:uid="{8067922A-00B7-4646-9500-13902203F407}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$B$3:$I$36</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$B$3:$I$37</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="77">
   <si>
     <t>Feature</t>
   </si>
@@ -264,6 +264,12 @@
   </si>
   <si>
     <t>add birth/death dates to people in the search lookup list</t>
+  </si>
+  <si>
+    <t>Fix spouse nodes on startup</t>
+  </si>
+  <si>
+    <t>spouse nodes of decendents are misplaced in time at startup, they reset and are correct after the tree is reconfigured with root individual or generations inputs</t>
   </si>
 </sst>
 </file>
@@ -986,7 +992,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{11BA4F79-2AB7-4A24-A4BE-758442E1F8CB}">
   <sheetPr filterMode="1"/>
-  <dimension ref="B1:N48"/>
+  <dimension ref="B1:N49"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="49.28515625" style="8" customWidth="1"/>
@@ -1219,30 +1225,32 @@
       <c r="M8" s="1"/>
       <c r="N8" s="1"/>
     </row>
-    <row r="9" spans="2:14" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:14" ht="47.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="B9" s="9">
         <f t="shared" ref="B9:B10" si="1">B8+1</f>
         <v>6</v>
       </c>
-      <c r="C9" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="D9" s="12"/>
-      <c r="E9" s="21">
-        <v>3</v>
-      </c>
-      <c r="F9" s="24">
-        <v>2</v>
-      </c>
-      <c r="G9" s="21">
-        <v>2</v>
-      </c>
-      <c r="H9" s="21">
+      <c r="C9" s="44" t="s">
+        <v>75</v>
+      </c>
+      <c r="D9" s="50" t="s">
+        <v>76</v>
+      </c>
+      <c r="E9" s="46">
+        <v>3</v>
+      </c>
+      <c r="F9" s="47">
+        <v>3</v>
+      </c>
+      <c r="G9" s="46">
+        <v>3</v>
+      </c>
+      <c r="H9" s="46">
         <f>SUM(E9:G9)</f>
-        <v>7</v>
-      </c>
-      <c r="I9" s="9">
-        <v>0</v>
+        <v>9</v>
+      </c>
+      <c r="I9" s="48">
+        <v>5</v>
       </c>
       <c r="K9" s="1"/>
       <c r="L9" s="1"/>
@@ -1254,12 +1262,10 @@
         <f t="shared" si="1"/>
         <v>7</v>
       </c>
-      <c r="C10" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="D10" s="12" t="s">
-        <v>24</v>
-      </c>
+      <c r="C10" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="D10" s="12"/>
       <c r="E10" s="21">
         <v>3</v>
       </c>
@@ -1274,133 +1280,130 @@
         <v>7</v>
       </c>
       <c r="I10" s="9">
-        <v>1</v>
-      </c>
-      <c r="J10" s="20"/>
+        <v>0</v>
+      </c>
       <c r="K10" s="1"/>
       <c r="L10" s="1"/>
       <c r="M10" s="1"/>
       <c r="N10" s="1"/>
     </row>
-    <row r="11" spans="2:14" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="48">
-        <f>B10+1</f>
+    <row r="11" spans="2:14" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="B11" s="9">
+        <f t="shared" ref="B11" si="2">B10+1</f>
         <v>8</v>
       </c>
-      <c r="C11" s="49" t="s">
-        <v>58</v>
-      </c>
-      <c r="D11" s="50"/>
-      <c r="E11" s="46">
-        <v>2</v>
-      </c>
-      <c r="F11" s="47">
-        <v>2</v>
-      </c>
-      <c r="G11" s="46">
-        <v>3</v>
-      </c>
-      <c r="H11" s="46">
+      <c r="C11" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="D11" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="E11" s="21">
+        <v>3</v>
+      </c>
+      <c r="F11" s="24">
+        <v>2</v>
+      </c>
+      <c r="G11" s="21">
+        <v>2</v>
+      </c>
+      <c r="H11" s="21">
         <f>SUM(E11:G11)</f>
         <v>7</v>
       </c>
-      <c r="I11" s="48">
-        <v>5</v>
-      </c>
-      <c r="J11" s="20" t="s">
-        <v>60</v>
-      </c>
+      <c r="I11" s="9">
+        <v>1</v>
+      </c>
+      <c r="J11" s="20"/>
       <c r="K11" s="1"/>
       <c r="L11" s="1"/>
       <c r="M11" s="1"/>
       <c r="N11" s="1"/>
     </row>
-    <row r="12" spans="2:14" ht="63" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B12" s="9">
+    <row r="12" spans="2:14" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B12" s="48">
         <f>B11+1</f>
         <v>9</v>
       </c>
-      <c r="C12" s="30" t="s">
-        <v>27</v>
-      </c>
-      <c r="D12" s="31" t="s">
-        <v>26</v>
-      </c>
-      <c r="E12" s="32">
-        <v>3</v>
-      </c>
-      <c r="F12" s="33">
-        <v>1</v>
-      </c>
-      <c r="G12" s="32">
-        <v>2</v>
-      </c>
-      <c r="H12" s="32">
+      <c r="C12" s="49" t="s">
+        <v>58</v>
+      </c>
+      <c r="D12" s="50"/>
+      <c r="E12" s="46">
+        <v>2</v>
+      </c>
+      <c r="F12" s="47">
+        <v>2</v>
+      </c>
+      <c r="G12" s="46">
+        <v>3</v>
+      </c>
+      <c r="H12" s="46">
         <f>SUM(E12:G12)</f>
-        <v>6</v>
-      </c>
-      <c r="I12" s="34">
+        <v>7</v>
+      </c>
+      <c r="I12" s="48">
         <v>5</v>
       </c>
-      <c r="J12" s="20"/>
+      <c r="J12" s="20" t="s">
+        <v>60</v>
+      </c>
       <c r="K12" s="1"/>
       <c r="L12" s="1"/>
       <c r="M12" s="1"/>
       <c r="N12" s="1"/>
     </row>
-    <row r="13" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:14" ht="63" hidden="1" x14ac:dyDescent="0.25">
       <c r="B13" s="9">
         <f>B12+1</f>
         <v>10</v>
       </c>
-      <c r="C13" s="35" t="s">
-        <v>52</v>
-      </c>
-      <c r="D13" s="35" t="s">
-        <v>53</v>
-      </c>
-      <c r="E13" s="42">
-        <v>3</v>
-      </c>
-      <c r="F13" s="43">
-        <v>2</v>
-      </c>
-      <c r="G13" s="42">
-        <v>2</v>
-      </c>
-      <c r="H13" s="21">
+      <c r="C13" s="30" t="s">
+        <v>27</v>
+      </c>
+      <c r="D13" s="31" t="s">
+        <v>26</v>
+      </c>
+      <c r="E13" s="32">
+        <v>3</v>
+      </c>
+      <c r="F13" s="33">
+        <v>1</v>
+      </c>
+      <c r="G13" s="32">
+        <v>2</v>
+      </c>
+      <c r="H13" s="32">
         <f>SUM(E13:G13)</f>
-        <v>7</v>
-      </c>
-      <c r="I13" s="9">
-        <v>4</v>
-      </c>
-      <c r="J13" s="41" t="s">
-        <v>65</v>
-      </c>
+        <v>6</v>
+      </c>
+      <c r="I13" s="34">
+        <v>5</v>
+      </c>
+      <c r="J13" s="20"/>
       <c r="K13" s="1"/>
       <c r="L13" s="1"/>
       <c r="M13" s="1"/>
       <c r="N13" s="1"/>
     </row>
-    <row r="14" spans="2:14" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B14" s="9">
         <f>B13+1</f>
         <v>11</v>
       </c>
-      <c r="C14" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="D14" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="E14" s="21">
-        <v>3</v>
-      </c>
-      <c r="F14" s="24">
-        <v>2</v>
-      </c>
-      <c r="G14" s="21">
+      <c r="C14" s="35" t="s">
+        <v>52</v>
+      </c>
+      <c r="D14" s="35" t="s">
+        <v>53</v>
+      </c>
+      <c r="E14" s="42">
+        <v>3</v>
+      </c>
+      <c r="F14" s="43">
+        <v>2</v>
+      </c>
+      <c r="G14" s="42">
         <v>2</v>
       </c>
       <c r="H14" s="21">
@@ -1408,23 +1411,26 @@
         <v>7</v>
       </c>
       <c r="I14" s="9">
-        <v>0</v>
+        <v>4</v>
+      </c>
+      <c r="J14" s="41" t="s">
+        <v>65</v>
       </c>
       <c r="K14" s="1"/>
       <c r="L14" s="1"/>
       <c r="M14" s="1"/>
       <c r="N14" s="1"/>
     </row>
-    <row r="15" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:14" ht="31.5" x14ac:dyDescent="0.25">
       <c r="B15" s="9">
         <f>B14+1</f>
         <v>12</v>
       </c>
-      <c r="C15" s="4" t="s">
-        <v>67</v>
+      <c r="C15" s="5" t="s">
+        <v>9</v>
       </c>
       <c r="D15" s="12" t="s">
-        <v>68</v>
+        <v>10</v>
       </c>
       <c r="E15" s="21">
         <v>3</v>
@@ -1442,25 +1448,24 @@
       <c r="I15" s="9">
         <v>0</v>
       </c>
-      <c r="J15" s="20"/>
       <c r="K15" s="1"/>
       <c r="L15" s="1"/>
       <c r="M15" s="1"/>
       <c r="N15" s="1"/>
     </row>
-    <row r="16" spans="2:14" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B16" s="9">
         <f>B15+1</f>
         <v>13</v>
       </c>
-      <c r="C16" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="D16" s="5" t="s">
-        <v>12</v>
+      <c r="C16" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="D16" s="12" t="s">
+        <v>68</v>
       </c>
       <c r="E16" s="21">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F16" s="24">
         <v>2</v>
@@ -1470,14 +1475,12 @@
       </c>
       <c r="H16" s="21">
         <f>SUM(E16:G16)</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I16" s="9">
-        <v>2</v>
-      </c>
-      <c r="J16" s="20" t="s">
-        <v>63</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="J16" s="20"/>
       <c r="K16" s="1"/>
       <c r="L16" s="1"/>
       <c r="M16" s="1"/>
@@ -1489,10 +1492,10 @@
         <v>14</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="D17" s="23" t="s">
-        <v>21</v>
+        <v>11</v>
+      </c>
+      <c r="D17" s="5" t="s">
+        <v>12</v>
       </c>
       <c r="E17" s="21">
         <v>2</v>
@@ -1508,9 +1511,11 @@
         <v>6</v>
       </c>
       <c r="I17" s="9">
-        <v>0</v>
-      </c>
-      <c r="J17" s="20"/>
+        <v>2</v>
+      </c>
+      <c r="J17" s="20" t="s">
+        <v>63</v>
+      </c>
       <c r="K17" s="1"/>
       <c r="L17" s="1"/>
       <c r="M17" s="1"/>
@@ -1522,10 +1527,10 @@
         <v>15</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>56</v>
+        <v>20</v>
       </c>
       <c r="D18" s="23" t="s">
-        <v>57</v>
+        <v>21</v>
       </c>
       <c r="E18" s="21">
         <v>2</v>
@@ -1549,16 +1554,16 @@
       <c r="M18" s="1"/>
       <c r="N18" s="1"/>
     </row>
-    <row r="19" spans="2:14" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:14" ht="31.5" x14ac:dyDescent="0.25">
       <c r="B19" s="9">
         <f>B18+1</f>
         <v>16</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="D19" s="5" t="s">
-        <v>48</v>
+        <v>56</v>
+      </c>
+      <c r="D19" s="23" t="s">
+        <v>57</v>
       </c>
       <c r="E19" s="21">
         <v>2</v>
@@ -1582,25 +1587,25 @@
       <c r="M19" s="1"/>
       <c r="N19" s="1"/>
     </row>
-    <row r="20" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:14" ht="47.25" x14ac:dyDescent="0.25">
       <c r="B20" s="9">
         <f>B19+1</f>
         <v>17</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="D20" s="12" t="s">
-        <v>71</v>
+        <v>36</v>
+      </c>
+      <c r="D20" s="5" t="s">
+        <v>48</v>
       </c>
       <c r="E20" s="21">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F20" s="24">
         <v>2</v>
       </c>
       <c r="G20" s="21">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H20" s="21">
         <f>SUM(E20:G20)</f>
@@ -1615,29 +1620,29 @@
       <c r="M20" s="1"/>
       <c r="N20" s="1"/>
     </row>
-    <row r="21" spans="2:14" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B21" s="9">
         <f>B20+1</f>
         <v>18</v>
       </c>
-      <c r="C21" s="23" t="s">
-        <v>22</v>
-      </c>
-      <c r="D21" s="23" t="s">
-        <v>23</v>
+      <c r="C21" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="D21" s="12" t="s">
+        <v>71</v>
       </c>
       <c r="E21" s="21">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F21" s="24">
         <v>2</v>
       </c>
       <c r="G21" s="21">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H21" s="21">
         <f>SUM(E21:G21)</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I21" s="9">
         <v>0</v>
@@ -1648,25 +1653,25 @@
       <c r="M21" s="1"/>
       <c r="N21" s="1"/>
     </row>
-    <row r="22" spans="2:14" ht="83.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:14" ht="47.25" x14ac:dyDescent="0.25">
       <c r="B22" s="9">
         <f>B21+1</f>
         <v>19</v>
       </c>
-      <c r="C22" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="D22" s="12" t="s">
-        <v>35</v>
+      <c r="C22" s="23" t="s">
+        <v>22</v>
+      </c>
+      <c r="D22" s="23" t="s">
+        <v>23</v>
       </c>
       <c r="E22" s="21">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F22" s="24">
         <v>2</v>
       </c>
       <c r="G22" s="21">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H22" s="21">
         <f>SUM(E22:G22)</f>
@@ -1675,68 +1680,70 @@
       <c r="I22" s="9">
         <v>0</v>
       </c>
+      <c r="J22" s="20"/>
       <c r="K22" s="1"/>
       <c r="L22" s="1"/>
       <c r="M22" s="1"/>
       <c r="N22" s="1"/>
     </row>
-    <row r="23" spans="2:14" ht="83.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="29">
+    <row r="23" spans="2:14" ht="83.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B23" s="9">
         <f>B22+1</f>
         <v>20</v>
       </c>
-      <c r="C23" s="30" t="s">
-        <v>31</v>
-      </c>
-      <c r="D23" s="31" t="s">
-        <v>32</v>
-      </c>
-      <c r="E23" s="32">
-        <v>2</v>
-      </c>
-      <c r="F23" s="33">
-        <v>1</v>
-      </c>
-      <c r="G23" s="32">
-        <v>3</v>
-      </c>
-      <c r="H23" s="32">
+      <c r="C23" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="D23" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="E23" s="21">
+        <v>1</v>
+      </c>
+      <c r="F23" s="24">
+        <v>2</v>
+      </c>
+      <c r="G23" s="21">
+        <v>2</v>
+      </c>
+      <c r="H23" s="21">
         <f>SUM(E23:G23)</f>
-        <v>6</v>
-      </c>
-      <c r="I23" s="34">
         <v>5</v>
       </c>
-      <c r="J23" s="20"/>
+      <c r="I23" s="9">
+        <v>0</v>
+      </c>
       <c r="K23" s="1"/>
       <c r="L23" s="1"/>
       <c r="M23" s="1"/>
       <c r="N23" s="1"/>
     </row>
-    <row r="24" spans="2:14" ht="83.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B24" s="9">
-        <f>B22+1</f>
-        <v>20</v>
-      </c>
-      <c r="C24" s="35" t="s">
-        <v>64</v>
-      </c>
-      <c r="D24" s="51"/>
-      <c r="E24" s="52">
-        <v>1</v>
-      </c>
-      <c r="F24" s="53">
-        <v>1</v>
-      </c>
-      <c r="G24" s="52">
-        <v>3</v>
-      </c>
-      <c r="H24" s="52">
+    <row r="24" spans="2:14" ht="83.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B24" s="29">
+        <f>B23+1</f>
+        <v>21</v>
+      </c>
+      <c r="C24" s="30" t="s">
+        <v>31</v>
+      </c>
+      <c r="D24" s="31" t="s">
+        <v>32</v>
+      </c>
+      <c r="E24" s="32">
+        <v>2</v>
+      </c>
+      <c r="F24" s="33">
+        <v>1</v>
+      </c>
+      <c r="G24" s="32">
+        <v>3</v>
+      </c>
+      <c r="H24" s="32">
         <f>SUM(E24:G24)</f>
+        <v>6</v>
+      </c>
+      <c r="I24" s="34">
         <v>5</v>
-      </c>
-      <c r="I24" s="9">
-        <v>0</v>
       </c>
       <c r="J24" s="20"/>
       <c r="K24" s="1"/>
@@ -1744,32 +1751,30 @@
       <c r="M24" s="1"/>
       <c r="N24" s="1"/>
     </row>
-    <row r="25" spans="2:14" ht="83.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="34">
-        <f>B24+1</f>
+    <row r="25" spans="2:14" ht="83.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B25" s="9">
+        <f>B23+1</f>
         <v>21</v>
       </c>
-      <c r="C25" s="54" t="s">
-        <v>62</v>
-      </c>
-      <c r="D25" s="55" t="s">
-        <v>61</v>
-      </c>
-      <c r="E25" s="32">
-        <v>2</v>
-      </c>
-      <c r="F25" s="33">
-        <v>2</v>
-      </c>
-      <c r="G25" s="32">
-        <v>2</v>
-      </c>
-      <c r="H25" s="32">
+      <c r="C25" s="35" t="s">
+        <v>64</v>
+      </c>
+      <c r="D25" s="51"/>
+      <c r="E25" s="52">
+        <v>1</v>
+      </c>
+      <c r="F25" s="53">
+        <v>1</v>
+      </c>
+      <c r="G25" s="52">
+        <v>3</v>
+      </c>
+      <c r="H25" s="52">
         <f>SUM(E25:G25)</f>
-        <v>6</v>
-      </c>
-      <c r="I25" s="34">
         <v>5</v>
+      </c>
+      <c r="I25" s="9">
+        <v>0</v>
       </c>
       <c r="J25" s="20"/>
       <c r="K25" s="1"/>
@@ -1777,30 +1782,32 @@
       <c r="M25" s="1"/>
       <c r="N25" s="1"/>
     </row>
-    <row r="26" spans="2:14" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="B26" s="9">
+    <row r="26" spans="2:14" ht="83.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B26" s="34">
         <f>B25+1</f>
         <v>22</v>
       </c>
-      <c r="C26" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="D26" s="12"/>
-      <c r="E26" s="21">
-        <v>1</v>
-      </c>
-      <c r="F26" s="24">
-        <v>1</v>
-      </c>
-      <c r="G26" s="21">
-        <v>3</v>
-      </c>
-      <c r="H26" s="21">
+      <c r="C26" s="54" t="s">
+        <v>62</v>
+      </c>
+      <c r="D26" s="55" t="s">
+        <v>61</v>
+      </c>
+      <c r="E26" s="32">
+        <v>2</v>
+      </c>
+      <c r="F26" s="33">
+        <v>2</v>
+      </c>
+      <c r="G26" s="32">
+        <v>2</v>
+      </c>
+      <c r="H26" s="32">
         <f>SUM(E26:G26)</f>
+        <v>6</v>
+      </c>
+      <c r="I26" s="34">
         <v>5</v>
-      </c>
-      <c r="I26" s="9">
-        <v>0</v>
       </c>
       <c r="J26" s="20"/>
       <c r="K26" s="1"/>
@@ -1808,29 +1815,27 @@
       <c r="M26" s="1"/>
       <c r="N26" s="1"/>
     </row>
-    <row r="27" spans="2:14" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:14" ht="31.5" x14ac:dyDescent="0.25">
       <c r="B27" s="9">
         <f>B26+1</f>
         <v>23</v>
       </c>
-      <c r="C27" s="56" t="s">
-        <v>42</v>
-      </c>
-      <c r="D27" s="12" t="s">
-        <v>43</v>
-      </c>
+      <c r="C27" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="D27" s="12"/>
       <c r="E27" s="21">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F27" s="24">
         <v>1</v>
       </c>
       <c r="G27" s="21">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H27" s="21">
         <f>SUM(E27:G27)</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I27" s="9">
         <v>0</v>
@@ -1846,20 +1851,20 @@
         <f>B27+1</f>
         <v>24</v>
       </c>
-      <c r="C28" s="4" t="s">
-        <v>5</v>
+      <c r="C28" s="56" t="s">
+        <v>42</v>
       </c>
       <c r="D28" s="12" t="s">
-        <v>6</v>
+        <v>43</v>
       </c>
       <c r="E28" s="21">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F28" s="24">
         <v>1</v>
       </c>
       <c r="G28" s="21">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H28" s="21">
         <f>SUM(E28:G28)</f>
@@ -1868,89 +1873,87 @@
       <c r="I28" s="9">
         <v>0</v>
       </c>
+      <c r="J28" s="20"/>
       <c r="K28" s="1"/>
       <c r="L28" s="1"/>
       <c r="M28" s="1"/>
       <c r="N28" s="1"/>
     </row>
-    <row r="29" spans="2:14" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B29" s="48">
+    <row r="29" spans="2:14" ht="47.25" x14ac:dyDescent="0.25">
+      <c r="B29" s="9">
         <f>B28+1</f>
         <v>25</v>
       </c>
-      <c r="C29" s="44" t="s">
-        <v>44</v>
-      </c>
-      <c r="D29" s="50" t="s">
-        <v>45</v>
-      </c>
-      <c r="E29" s="46">
-        <v>2</v>
-      </c>
-      <c r="F29" s="47">
-        <v>1</v>
-      </c>
-      <c r="G29" s="46">
-        <v>1</v>
-      </c>
-      <c r="H29" s="46">
+      <c r="C29" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="D29" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="E29" s="21">
+        <v>1</v>
+      </c>
+      <c r="F29" s="24">
+        <v>1</v>
+      </c>
+      <c r="G29" s="21">
+        <v>2</v>
+      </c>
+      <c r="H29" s="21">
         <f>SUM(E29:G29)</f>
         <v>4</v>
       </c>
-      <c r="I29" s="48">
-        <v>5</v>
-      </c>
-      <c r="J29" s="20"/>
+      <c r="I29" s="9">
+        <v>0</v>
+      </c>
       <c r="K29" s="1"/>
       <c r="L29" s="1"/>
       <c r="M29" s="1"/>
       <c r="N29" s="1"/>
     </row>
-    <row r="30" spans="2:14" ht="78.75" x14ac:dyDescent="0.25">
-      <c r="B30" s="9">
+    <row r="30" spans="2:14" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B30" s="48">
         <f>B29+1</f>
         <v>26</v>
       </c>
-      <c r="C30" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="D30" s="12" t="s">
-        <v>34</v>
-      </c>
-      <c r="E30" s="21">
-        <v>1</v>
-      </c>
-      <c r="F30" s="24">
-        <v>1</v>
-      </c>
-      <c r="G30" s="21">
-        <v>2</v>
-      </c>
-      <c r="H30" s="21">
+      <c r="C30" s="44" t="s">
+        <v>44</v>
+      </c>
+      <c r="D30" s="50" t="s">
+        <v>45</v>
+      </c>
+      <c r="E30" s="46">
+        <v>2</v>
+      </c>
+      <c r="F30" s="47">
+        <v>1</v>
+      </c>
+      <c r="G30" s="46">
+        <v>1</v>
+      </c>
+      <c r="H30" s="46">
         <f>SUM(E30:G30)</f>
         <v>4</v>
       </c>
-      <c r="I30" s="9">
-        <v>2</v>
-      </c>
-      <c r="J30" s="20" t="s">
-        <v>51</v>
-      </c>
+      <c r="I30" s="48">
+        <v>5</v>
+      </c>
+      <c r="J30" s="20"/>
       <c r="K30" s="1"/>
       <c r="L30" s="1"/>
       <c r="M30" s="1"/>
       <c r="N30" s="1"/>
     </row>
-    <row r="31" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:14" ht="78.75" x14ac:dyDescent="0.25">
       <c r="B31" s="9">
         <f>B30+1</f>
         <v>27</v>
       </c>
-      <c r="C31" s="5" t="s">
-        <v>7</v>
+      <c r="C31" s="4" t="s">
+        <v>33</v>
       </c>
       <c r="D31" s="12" t="s">
-        <v>8</v>
+        <v>34</v>
       </c>
       <c r="E31" s="21">
         <v>1</v>
@@ -1966,24 +1969,26 @@
         <v>4</v>
       </c>
       <c r="I31" s="9">
-        <v>0</v>
-      </c>
-      <c r="J31" s="20"/>
+        <v>2</v>
+      </c>
+      <c r="J31" s="20" t="s">
+        <v>51</v>
+      </c>
       <c r="K31" s="1"/>
       <c r="L31" s="1"/>
       <c r="M31" s="1"/>
       <c r="N31" s="1"/>
     </row>
-    <row r="32" spans="2:14" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B32" s="9">
         <f>B31+1</f>
         <v>28</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>37</v>
+        <v>7</v>
       </c>
       <c r="D32" s="12" t="s">
-        <v>38</v>
+        <v>8</v>
       </c>
       <c r="E32" s="21">
         <v>1</v>
@@ -2013,10 +2018,10 @@
         <v>29</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="D33" s="12" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="E33" s="21">
         <v>1</v>
@@ -2045,11 +2050,11 @@
         <f>B33+1</f>
         <v>30</v>
       </c>
-      <c r="C34" s="4" t="s">
-        <v>3</v>
+      <c r="C34" s="5" t="s">
+        <v>40</v>
       </c>
       <c r="D34" s="12" t="s">
-        <v>4</v>
+        <v>41</v>
       </c>
       <c r="E34" s="21">
         <v>1</v>
@@ -2058,11 +2063,11 @@
         <v>1</v>
       </c>
       <c r="G34" s="21">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H34" s="21">
         <f>SUM(E34:G34)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I34" s="9">
         <v>0</v>
@@ -2073,15 +2078,17 @@
       <c r="M34" s="1"/>
       <c r="N34" s="1"/>
     </row>
-    <row r="35" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:14" ht="31.5" x14ac:dyDescent="0.25">
       <c r="B35" s="9">
         <f>B34+1</f>
         <v>31</v>
       </c>
-      <c r="C35" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="D35" s="12"/>
+      <c r="C35" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="D35" s="12" t="s">
+        <v>4</v>
+      </c>
       <c r="E35" s="21">
         <v>1</v>
       </c>
@@ -2104,29 +2111,29 @@
       <c r="M35" s="1"/>
       <c r="N35" s="1"/>
     </row>
-    <row r="36" spans="2:14" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B36" s="9">
         <f>B35+1</f>
         <v>32</v>
       </c>
-      <c r="C36" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="D36" s="13"/>
-      <c r="E36" s="22">
-        <v>1</v>
-      </c>
-      <c r="F36" s="25">
-        <v>1</v>
-      </c>
-      <c r="G36" s="22">
-        <v>1</v>
-      </c>
-      <c r="H36" s="22">
+      <c r="C36" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D36" s="12"/>
+      <c r="E36" s="21">
+        <v>1</v>
+      </c>
+      <c r="F36" s="24">
+        <v>1</v>
+      </c>
+      <c r="G36" s="21">
+        <v>1</v>
+      </c>
+      <c r="H36" s="21">
         <f>SUM(E36:G36)</f>
         <v>3</v>
       </c>
-      <c r="I36" s="28">
+      <c r="I36" s="9">
         <v>0</v>
       </c>
       <c r="J36" s="20"/>
@@ -2135,8 +2142,31 @@
       <c r="M36" s="1"/>
       <c r="N36" s="1"/>
     </row>
-    <row r="37" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="I37" s="10"/>
+    <row r="37" spans="2:14" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B37" s="9">
+        <f>B36+1</f>
+        <v>33</v>
+      </c>
+      <c r="C37" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="D37" s="13"/>
+      <c r="E37" s="22">
+        <v>1</v>
+      </c>
+      <c r="F37" s="25">
+        <v>1</v>
+      </c>
+      <c r="G37" s="22">
+        <v>1</v>
+      </c>
+      <c r="H37" s="22">
+        <f>SUM(E37:G37)</f>
+        <v>3</v>
+      </c>
+      <c r="I37" s="28">
+        <v>0</v>
+      </c>
       <c r="J37" s="20"/>
       <c r="K37" s="1"/>
       <c r="L37" s="1"/>
@@ -2144,13 +2174,6 @@
       <c r="N37" s="1"/>
     </row>
     <row r="38" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B38" s="10"/>
-      <c r="C38" s="26"/>
-      <c r="D38" s="27"/>
-      <c r="E38" s="20"/>
-      <c r="F38" s="20"/>
-      <c r="G38" s="20"/>
-      <c r="H38" s="20"/>
       <c r="I38" s="10"/>
       <c r="J38" s="20"/>
       <c r="K38" s="1"/>
@@ -2159,13 +2182,13 @@
       <c r="N38" s="1"/>
     </row>
     <row r="39" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B39" s="1"/>
-      <c r="C39" s="7"/>
-      <c r="D39" s="2"/>
-      <c r="E39" s="10"/>
-      <c r="F39" s="10"/>
-      <c r="G39" s="10"/>
-      <c r="H39" s="10"/>
+      <c r="B39" s="10"/>
+      <c r="C39" s="26"/>
+      <c r="D39" s="27"/>
+      <c r="E39" s="20"/>
+      <c r="F39" s="20"/>
+      <c r="G39" s="20"/>
+      <c r="H39" s="20"/>
       <c r="I39" s="10"/>
       <c r="J39" s="20"/>
       <c r="K39" s="1"/>
@@ -2308,25 +2331,42 @@
       <c r="M48" s="1"/>
       <c r="N48" s="1"/>
     </row>
+    <row r="49" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B49" s="1"/>
+      <c r="C49" s="7"/>
+      <c r="D49" s="2"/>
+      <c r="E49" s="10"/>
+      <c r="F49" s="10"/>
+      <c r="G49" s="10"/>
+      <c r="H49" s="10"/>
+      <c r="I49" s="10"/>
+      <c r="J49" s="20"/>
+      <c r="K49" s="1"/>
+      <c r="L49" s="1"/>
+      <c r="M49" s="1"/>
+      <c r="N49" s="1"/>
+    </row>
   </sheetData>
-  <autoFilter ref="B3:I36" xr:uid="{11BA4F79-2AB7-4A24-A4BE-758442E1F8CB}">
+  <autoFilter ref="B3:I37" xr:uid="{11BA4F79-2AB7-4A24-A4BE-758442E1F8CB}">
     <filterColumn colId="7">
       <filters>
         <filter val="0"/>
         <filter val="1"/>
         <filter val="2"/>
+        <filter val="3"/>
+        <filter val="4"/>
       </filters>
     </filterColumn>
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B5:I36">
-      <sortCondition descending="1" ref="H4:H36"/>
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B5:I37">
+      <sortCondition descending="1" ref="H4:H37"/>
     </sortState>
   </autoFilter>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B5:J36">
-    <sortCondition descending="1" ref="H4:H36"/>
-    <sortCondition descending="1" ref="E4:E36"/>
-    <sortCondition descending="1" ref="F4:F36"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B5:J37">
+    <sortCondition descending="1" ref="H4:H37"/>
+    <sortCondition descending="1" ref="E4:E37"/>
+    <sortCondition descending="1" ref="F4:F37"/>
   </sortState>
-  <conditionalFormatting sqref="H4:H36">
+  <conditionalFormatting sqref="H4:H37">
     <cfRule type="colorScale" priority="3">
       <colorScale>
         <cfvo type="min"/>
@@ -2338,7 +2378,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I4:I36">
+  <conditionalFormatting sqref="I4:I37">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>

</xml_diff>

<commit_message>
cleaning up the righthand panel
deleted a bunch of the .css and html for functions not currently used
</commit_message>
<xml_diff>
--- a/Future Features/New Features - Family Tree.xlsx
+++ b/Future Features/New Features - Family Tree.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://srcincgov1-my.sharepoint.us/personal/lauko_srcinc_com/Documents/Desktop/Personal/geneology/GED Keepers/Future Features/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="395" documentId="8_{D1FEEEA7-0E84-49B9-AD17-37D0BB95FB37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AE2D1D0E-B6BB-4B28-801B-D0551587A1FC}"/>
+  <xr:revisionPtr revIDLastSave="397" documentId="8_{D1FEEEA7-0E84-49B9-AD17-37D0BB95FB37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FC7046C6-96AE-416F-9AD4-D1FF80A3BA71}"/>
   <bookViews>
     <workbookView xWindow="15" yWindow="0" windowWidth="23010" windowHeight="12330" xr2:uid="{8067922A-00B7-4646-9500-13902203F407}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="78">
   <si>
     <t>Feature</t>
   </si>
@@ -270,6 +270,9 @@
   </si>
   <si>
     <t>spouse nodes of decendents are misplaced in time at startup, they reset and are correct after the tree is reconfigured with root individual or generations inputs</t>
+  </si>
+  <si>
+    <t>The search function/Root individual needs some work.  The Root Ind function seems struggles when the person selected is not on the screen</t>
   </si>
 </sst>
 </file>
@@ -1257,7 +1260,7 @@
       <c r="M9" s="1"/>
       <c r="N9" s="1"/>
     </row>
-    <row r="10" spans="2:14" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:14" ht="47.25" x14ac:dyDescent="0.25">
       <c r="B10" s="9">
         <f t="shared" si="1"/>
         <v>7</v>
@@ -1265,7 +1268,9 @@
       <c r="C10" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="D10" s="12"/>
+      <c r="D10" s="12" t="s">
+        <v>77</v>
+      </c>
       <c r="E10" s="21">
         <v>3</v>
       </c>

</xml_diff>

<commit_message>
fixed location search, speed improvements in clusters
eliminated computationally intensive algorithm in cluster.draw()
</commit_message>
<xml_diff>
--- a/Future Features/New Features - Family Tree.xlsx
+++ b/Future Features/New Features - Family Tree.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://srcincgov1-my.sharepoint.us/personal/lauko_srcinc_com/Documents/Desktop/Personal/geneology/GED Keepers/Future Features/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="401" documentId="8_{D1FEEEA7-0E84-49B9-AD17-37D0BB95FB37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1C1AF6D6-8A9D-49A0-BD61-6736A57D547C}"/>
+  <xr:revisionPtr revIDLastSave="418" documentId="8_{D1FEEEA7-0E84-49B9-AD17-37D0BB95FB37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{143F75FF-9DF9-416C-AC00-15308AFB06BE}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{8067922A-00B7-4646-9500-13902203F407}"/>
   </bookViews>
@@ -16,9 +16,9 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$B$3:$I$37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$B$3:$I$38</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" calcCompleted="0"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="79">
   <si>
     <t>Feature</t>
   </si>
@@ -273,6 +273,9 @@
   </si>
   <si>
     <t>The search function/Root individual needs some work.  The Root Ind function seems struggles when the person selected is not on the screen</t>
+  </si>
+  <si>
+    <t>Location search should be on the whole family tree, not just the part that is visible.</t>
   </si>
 </sst>
 </file>
@@ -992,7 +995,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{11BA4F79-2AB7-4A24-A4BE-758442E1F8CB}">
   <sheetPr filterMode="1"/>
-  <dimension ref="B1:N49"/>
+  <dimension ref="B1:N50"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="49.28515625" style="8" customWidth="1"/>
@@ -1097,31 +1100,27 @@
         <f>B4+1</f>
         <v>2</v>
       </c>
-      <c r="C5" s="35" t="s">
-        <v>66</v>
-      </c>
-      <c r="D5" s="35" t="s">
-        <v>69</v>
-      </c>
-      <c r="E5" s="42">
-        <v>3</v>
-      </c>
-      <c r="F5" s="43">
-        <v>2</v>
-      </c>
-      <c r="G5" s="42">
-        <v>3</v>
+      <c r="C5" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="D5" s="5"/>
+      <c r="E5" s="21">
+        <v>3</v>
+      </c>
+      <c r="F5" s="24">
+        <v>3</v>
+      </c>
+      <c r="G5" s="21">
+        <v>2</v>
       </c>
       <c r="H5" s="21">
-        <f t="shared" ref="H5:H37" si="1">SUM(E5:G5)</f>
+        <f>SUM(E5:G5)</f>
         <v>8</v>
       </c>
       <c r="I5" s="9">
-        <v>3</v>
-      </c>
-      <c r="J5" s="20" t="s">
-        <v>70</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="J5" s="20"/>
       <c r="K5" s="1"/>
       <c r="L5" s="1"/>
       <c r="M5" s="1"/>
@@ -1148,7 +1147,7 @@
         <v>2</v>
       </c>
       <c r="H6" s="46">
-        <f t="shared" si="1"/>
+        <f>SUM(E6:G6)</f>
         <v>7</v>
       </c>
       <c r="I6" s="48">
@@ -1181,7 +1180,7 @@
         <v>3</v>
       </c>
       <c r="H7" s="32">
-        <f t="shared" si="1"/>
+        <f>SUM(E7:G7)</f>
         <v>7</v>
       </c>
       <c r="I7" s="34">
@@ -1193,32 +1192,35 @@
       <c r="M7" s="1"/>
       <c r="N7" s="1"/>
     </row>
-    <row r="8" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B8" s="48">
+    <row r="8" spans="2:14" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="B8" s="9">
         <f>B7+1</f>
         <v>5</v>
       </c>
-      <c r="C8" s="44" t="s">
-        <v>72</v>
-      </c>
-      <c r="D8" s="50" t="s">
-        <v>73</v>
-      </c>
-      <c r="E8" s="46">
-        <v>3</v>
-      </c>
-      <c r="F8" s="47">
-        <v>2</v>
-      </c>
-      <c r="G8" s="46">
-        <v>3</v>
-      </c>
-      <c r="H8" s="46">
-        <f t="shared" si="1"/>
+      <c r="C8" s="35" t="s">
+        <v>66</v>
+      </c>
+      <c r="D8" s="35" t="s">
+        <v>69</v>
+      </c>
+      <c r="E8" s="42">
+        <v>3</v>
+      </c>
+      <c r="F8" s="43">
+        <v>2</v>
+      </c>
+      <c r="G8" s="42">
+        <v>3</v>
+      </c>
+      <c r="H8" s="21">
+        <f>SUM(E8:G8)</f>
         <v>8</v>
       </c>
-      <c r="I8" s="48">
-        <v>5</v>
+      <c r="I8" s="9">
+        <v>3</v>
+      </c>
+      <c r="J8" s="20" t="s">
+        <v>70</v>
       </c>
       <c r="K8" s="1"/>
       <c r="L8" s="1"/>
@@ -1227,7 +1229,7 @@
     </row>
     <row r="9" spans="2:14" ht="47.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="B9" s="9">
-        <f t="shared" ref="B9:B10" si="2">B8+1</f>
+        <f>B8+1</f>
         <v>6</v>
       </c>
       <c r="C9" s="44" t="s">
@@ -1246,7 +1248,7 @@
         <v>3</v>
       </c>
       <c r="H9" s="46">
-        <f t="shared" si="1"/>
+        <f>SUM(E9:G9)</f>
         <v>9</v>
       </c>
       <c r="I9" s="48">
@@ -1257,66 +1259,65 @@
       <c r="M9" s="1"/>
       <c r="N9" s="1"/>
     </row>
-    <row r="10" spans="2:14" ht="47.25" x14ac:dyDescent="0.25">
-      <c r="B10" s="9">
-        <f t="shared" si="2"/>
+    <row r="10" spans="2:14" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B10" s="48">
+        <f>B9+1</f>
         <v>7</v>
       </c>
-      <c r="C10" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="D10" s="12" t="s">
-        <v>77</v>
-      </c>
-      <c r="E10" s="21">
-        <v>3</v>
-      </c>
-      <c r="F10" s="24">
-        <v>2</v>
-      </c>
-      <c r="G10" s="21">
-        <v>2</v>
-      </c>
-      <c r="H10" s="21">
-        <f t="shared" si="1"/>
-        <v>7</v>
-      </c>
-      <c r="I10" s="9">
-        <v>0</v>
+      <c r="C10" s="44" t="s">
+        <v>72</v>
+      </c>
+      <c r="D10" s="50" t="s">
+        <v>73</v>
+      </c>
+      <c r="E10" s="46">
+        <v>3</v>
+      </c>
+      <c r="F10" s="47">
+        <v>2</v>
+      </c>
+      <c r="G10" s="46">
+        <v>3</v>
+      </c>
+      <c r="H10" s="46">
+        <f>SUM(E10:G10)</f>
+        <v>8</v>
+      </c>
+      <c r="I10" s="48">
+        <v>5</v>
       </c>
       <c r="K10" s="1"/>
       <c r="L10" s="1"/>
       <c r="M10" s="1"/>
       <c r="N10" s="1"/>
     </row>
-    <row r="11" spans="2:14" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="B11" s="9">
-        <f t="shared" ref="B11" si="3">B10+1</f>
+    <row r="11" spans="2:14" ht="47.25" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B11" s="48">
+        <f>B10+1</f>
         <v>8</v>
       </c>
-      <c r="C11" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="D11" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="E11" s="21">
-        <v>3</v>
-      </c>
-      <c r="F11" s="24">
-        <v>2</v>
-      </c>
-      <c r="G11" s="21">
-        <v>2</v>
-      </c>
-      <c r="H11" s="21">
-        <f t="shared" si="1"/>
+      <c r="C11" s="44" t="s">
+        <v>74</v>
+      </c>
+      <c r="D11" s="50" t="s">
+        <v>77</v>
+      </c>
+      <c r="E11" s="46">
+        <v>3</v>
+      </c>
+      <c r="F11" s="47">
+        <v>2</v>
+      </c>
+      <c r="G11" s="46">
+        <v>2</v>
+      </c>
+      <c r="H11" s="46">
+        <f>SUM(E11:G11)</f>
         <v>7</v>
       </c>
-      <c r="I11" s="9">
-        <v>1</v>
-      </c>
-      <c r="J11" s="20"/>
+      <c r="I11" s="48">
+        <v>5</v>
+      </c>
       <c r="K11" s="1"/>
       <c r="L11" s="1"/>
       <c r="M11" s="1"/>
@@ -1324,7 +1325,7 @@
     </row>
     <row r="12" spans="2:14" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="B12" s="48">
-        <f t="shared" ref="B12:B24" si="4">B11+1</f>
+        <f>B11+1</f>
         <v>9</v>
       </c>
       <c r="C12" s="49" t="s">
@@ -1341,7 +1342,7 @@
         <v>3</v>
       </c>
       <c r="H12" s="46">
-        <f t="shared" si="1"/>
+        <f>SUM(E12:G12)</f>
         <v>7</v>
       </c>
       <c r="I12" s="48">
@@ -1357,7 +1358,7 @@
     </row>
     <row r="13" spans="2:14" ht="63" hidden="1" x14ac:dyDescent="0.25">
       <c r="B13" s="9">
-        <f t="shared" si="4"/>
+        <f>B12+1</f>
         <v>10</v>
       </c>
       <c r="C13" s="30" t="s">
@@ -1376,7 +1377,7 @@
         <v>2</v>
       </c>
       <c r="H13" s="32">
-        <f t="shared" si="1"/>
+        <f>SUM(E13:G13)</f>
         <v>6</v>
       </c>
       <c r="I13" s="34">
@@ -1388,119 +1389,119 @@
       <c r="M13" s="1"/>
       <c r="N13" s="1"/>
     </row>
-    <row r="14" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:14" ht="31.5" x14ac:dyDescent="0.25">
       <c r="B14" s="9">
-        <f t="shared" si="4"/>
+        <f>B13+1</f>
         <v>11</v>
       </c>
-      <c r="C14" s="35" t="s">
-        <v>52</v>
-      </c>
-      <c r="D14" s="35" t="s">
-        <v>53</v>
-      </c>
-      <c r="E14" s="42">
-        <v>3</v>
-      </c>
-      <c r="F14" s="43">
-        <v>2</v>
-      </c>
-      <c r="G14" s="42">
+      <c r="C14" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="D14" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="E14" s="21">
+        <v>3</v>
+      </c>
+      <c r="F14" s="24">
+        <v>2</v>
+      </c>
+      <c r="G14" s="21">
         <v>2</v>
       </c>
       <c r="H14" s="21">
-        <f t="shared" si="1"/>
+        <f>SUM(E14:G14)</f>
         <v>7</v>
       </c>
       <c r="I14" s="9">
-        <v>4</v>
-      </c>
-      <c r="J14" s="41" t="s">
-        <v>65</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="J14" s="20"/>
       <c r="K14" s="1"/>
       <c r="L14" s="1"/>
       <c r="M14" s="1"/>
       <c r="N14" s="1"/>
     </row>
-    <row r="15" spans="2:14" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B15" s="9">
-        <f t="shared" si="4"/>
+        <f>B14+1</f>
         <v>12</v>
       </c>
-      <c r="C15" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="D15" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="E15" s="21">
-        <v>3</v>
-      </c>
-      <c r="F15" s="24">
-        <v>2</v>
-      </c>
-      <c r="G15" s="21">
+      <c r="C15" s="35" t="s">
+        <v>52</v>
+      </c>
+      <c r="D15" s="35" t="s">
+        <v>53</v>
+      </c>
+      <c r="E15" s="42">
+        <v>3</v>
+      </c>
+      <c r="F15" s="43">
+        <v>2</v>
+      </c>
+      <c r="G15" s="42">
         <v>2</v>
       </c>
       <c r="H15" s="21">
-        <f t="shared" si="1"/>
+        <f>SUM(E15:G15)</f>
         <v>7</v>
       </c>
       <c r="I15" s="9">
-        <v>0</v>
+        <v>4</v>
+      </c>
+      <c r="J15" s="41" t="s">
+        <v>65</v>
       </c>
       <c r="K15" s="1"/>
       <c r="L15" s="1"/>
       <c r="M15" s="1"/>
       <c r="N15" s="1"/>
     </row>
-    <row r="16" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B16" s="9">
-        <f t="shared" si="4"/>
+    <row r="16" spans="2:14" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B16" s="48">
+        <f>B15+1</f>
         <v>13</v>
       </c>
-      <c r="C16" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="D16" s="12" t="s">
-        <v>68</v>
-      </c>
-      <c r="E16" s="21">
-        <v>3</v>
-      </c>
-      <c r="F16" s="24">
-        <v>2</v>
-      </c>
-      <c r="G16" s="21">
-        <v>2</v>
-      </c>
-      <c r="H16" s="21">
-        <f t="shared" si="1"/>
+      <c r="C16" s="44" t="s">
+        <v>9</v>
+      </c>
+      <c r="D16" s="50" t="s">
+        <v>10</v>
+      </c>
+      <c r="E16" s="46">
+        <v>3</v>
+      </c>
+      <c r="F16" s="47">
+        <v>2</v>
+      </c>
+      <c r="G16" s="46">
+        <v>2</v>
+      </c>
+      <c r="H16" s="46">
+        <f>SUM(E16:G16)</f>
         <v>7</v>
       </c>
-      <c r="I16" s="9">
-        <v>0</v>
-      </c>
-      <c r="J16" s="20"/>
+      <c r="I16" s="48">
+        <v>5</v>
+      </c>
       <c r="K16" s="1"/>
       <c r="L16" s="1"/>
       <c r="M16" s="1"/>
       <c r="N16" s="1"/>
     </row>
-    <row r="17" spans="2:14" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B17" s="9">
-        <f t="shared" si="4"/>
+        <f>B16+1</f>
         <v>14</v>
       </c>
-      <c r="C17" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="D17" s="5" t="s">
-        <v>12</v>
+      <c r="C17" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="D17" s="12" t="s">
+        <v>68</v>
       </c>
       <c r="E17" s="21">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F17" s="24">
         <v>2</v>
@@ -1509,15 +1510,13 @@
         <v>2</v>
       </c>
       <c r="H17" s="21">
-        <f t="shared" si="1"/>
-        <v>6</v>
+        <f>SUM(E17:G17)</f>
+        <v>7</v>
       </c>
       <c r="I17" s="9">
-        <v>2</v>
-      </c>
-      <c r="J17" s="20" t="s">
-        <v>63</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="J17" s="20"/>
       <c r="K17" s="1"/>
       <c r="L17" s="1"/>
       <c r="M17" s="1"/>
@@ -1525,14 +1524,14 @@
     </row>
     <row r="18" spans="2:14" ht="31.5" x14ac:dyDescent="0.25">
       <c r="B18" s="9">
-        <f t="shared" si="4"/>
+        <f>B17+1</f>
         <v>15</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="D18" s="23" t="s">
-        <v>21</v>
+        <v>11</v>
+      </c>
+      <c r="D18" s="5" t="s">
+        <v>12</v>
       </c>
       <c r="E18" s="21">
         <v>2</v>
@@ -1544,13 +1543,15 @@
         <v>2</v>
       </c>
       <c r="H18" s="21">
-        <f t="shared" si="1"/>
+        <f>SUM(E18:G18)</f>
         <v>6</v>
       </c>
       <c r="I18" s="9">
-        <v>0</v>
-      </c>
-      <c r="J18" s="20"/>
+        <v>2</v>
+      </c>
+      <c r="J18" s="20" t="s">
+        <v>63</v>
+      </c>
       <c r="K18" s="1"/>
       <c r="L18" s="1"/>
       <c r="M18" s="1"/>
@@ -1558,14 +1559,14 @@
     </row>
     <row r="19" spans="2:14" ht="31.5" x14ac:dyDescent="0.25">
       <c r="B19" s="9">
-        <f t="shared" si="4"/>
+        <f>B18+1</f>
         <v>16</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>56</v>
+        <v>20</v>
       </c>
       <c r="D19" s="23" t="s">
-        <v>57</v>
+        <v>21</v>
       </c>
       <c r="E19" s="21">
         <v>2</v>
@@ -1577,7 +1578,7 @@
         <v>2</v>
       </c>
       <c r="H19" s="21">
-        <f t="shared" si="1"/>
+        <f>SUM(E19:G19)</f>
         <v>6</v>
       </c>
       <c r="I19" s="9">
@@ -1589,16 +1590,16 @@
       <c r="M19" s="1"/>
       <c r="N19" s="1"/>
     </row>
-    <row r="20" spans="2:14" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:14" ht="31.5" x14ac:dyDescent="0.25">
       <c r="B20" s="9">
-        <f t="shared" si="4"/>
+        <f>B19+1</f>
         <v>17</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="D20" s="5" t="s">
-        <v>48</v>
+        <v>56</v>
+      </c>
+      <c r="D20" s="23" t="s">
+        <v>57</v>
       </c>
       <c r="E20" s="21">
         <v>2</v>
@@ -1610,7 +1611,7 @@
         <v>2</v>
       </c>
       <c r="H20" s="21">
-        <f t="shared" si="1"/>
+        <f>SUM(E20:G20)</f>
         <v>6</v>
       </c>
       <c r="I20" s="9">
@@ -1622,28 +1623,28 @@
       <c r="M20" s="1"/>
       <c r="N20" s="1"/>
     </row>
-    <row r="21" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:14" ht="47.25" x14ac:dyDescent="0.25">
       <c r="B21" s="9">
-        <f t="shared" si="4"/>
+        <f>B20+1</f>
         <v>18</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="D21" s="12" t="s">
-        <v>71</v>
+        <v>36</v>
+      </c>
+      <c r="D21" s="5" t="s">
+        <v>48</v>
       </c>
       <c r="E21" s="21">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F21" s="24">
         <v>2</v>
       </c>
       <c r="G21" s="21">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H21" s="21">
-        <f t="shared" si="1"/>
+        <f>SUM(E21:G21)</f>
         <v>6</v>
       </c>
       <c r="I21" s="9">
@@ -1655,29 +1656,29 @@
       <c r="M21" s="1"/>
       <c r="N21" s="1"/>
     </row>
-    <row r="22" spans="2:14" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B22" s="9">
-        <f t="shared" si="4"/>
+        <f>B21+1</f>
         <v>19</v>
       </c>
-      <c r="C22" s="23" t="s">
-        <v>22</v>
-      </c>
-      <c r="D22" s="23" t="s">
-        <v>23</v>
+      <c r="C22" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="D22" s="12" t="s">
+        <v>71</v>
       </c>
       <c r="E22" s="21">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F22" s="24">
         <v>2</v>
       </c>
       <c r="G22" s="21">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H22" s="21">
-        <f t="shared" si="1"/>
-        <v>5</v>
+        <f>SUM(E22:G22)</f>
+        <v>6</v>
       </c>
       <c r="I22" s="9">
         <v>0</v>
@@ -1688,95 +1689,97 @@
       <c r="M22" s="1"/>
       <c r="N22" s="1"/>
     </row>
-    <row r="23" spans="2:14" ht="83.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:14" ht="47.25" x14ac:dyDescent="0.25">
       <c r="B23" s="9">
-        <f t="shared" si="4"/>
+        <f>B22+1</f>
         <v>20</v>
       </c>
-      <c r="C23" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="D23" s="12" t="s">
-        <v>35</v>
+      <c r="C23" s="23" t="s">
+        <v>22</v>
+      </c>
+      <c r="D23" s="23" t="s">
+        <v>23</v>
       </c>
       <c r="E23" s="21">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F23" s="24">
         <v>2</v>
       </c>
       <c r="G23" s="21">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H23" s="21">
-        <f t="shared" si="1"/>
+        <f>SUM(E23:G23)</f>
         <v>5</v>
       </c>
       <c r="I23" s="9">
         <v>0</v>
       </c>
+      <c r="J23" s="20"/>
       <c r="K23" s="1"/>
       <c r="L23" s="1"/>
       <c r="M23" s="1"/>
       <c r="N23" s="1"/>
     </row>
-    <row r="24" spans="2:14" ht="83.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B24" s="29">
-        <f t="shared" si="4"/>
+    <row r="24" spans="2:14" ht="83.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B24" s="9">
+        <f>B23+1</f>
         <v>21</v>
       </c>
-      <c r="C24" s="30" t="s">
-        <v>31</v>
-      </c>
-      <c r="D24" s="31" t="s">
-        <v>32</v>
-      </c>
-      <c r="E24" s="32">
-        <v>2</v>
-      </c>
-      <c r="F24" s="33">
-        <v>1</v>
-      </c>
-      <c r="G24" s="32">
-        <v>3</v>
-      </c>
-      <c r="H24" s="32">
-        <f t="shared" si="1"/>
-        <v>6</v>
-      </c>
-      <c r="I24" s="34">
+      <c r="C24" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="D24" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="E24" s="21">
+        <v>1</v>
+      </c>
+      <c r="F24" s="24">
+        <v>2</v>
+      </c>
+      <c r="G24" s="21">
+        <v>2</v>
+      </c>
+      <c r="H24" s="21">
+        <f>SUM(E24:G24)</f>
         <v>5</v>
       </c>
-      <c r="J24" s="20"/>
+      <c r="I24" s="9">
+        <v>0</v>
+      </c>
       <c r="K24" s="1"/>
       <c r="L24" s="1"/>
       <c r="M24" s="1"/>
       <c r="N24" s="1"/>
     </row>
-    <row r="25" spans="2:14" ht="83.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="9">
-        <f>B23+1</f>
-        <v>21</v>
-      </c>
-      <c r="C25" s="35" t="s">
-        <v>64</v>
-      </c>
-      <c r="D25" s="51"/>
-      <c r="E25" s="52">
-        <v>1</v>
-      </c>
-      <c r="F25" s="53">
-        <v>1</v>
-      </c>
-      <c r="G25" s="52">
-        <v>3</v>
-      </c>
-      <c r="H25" s="52">
-        <f t="shared" si="1"/>
+    <row r="25" spans="2:14" ht="83.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B25" s="29">
+        <f>B24+1</f>
+        <v>22</v>
+      </c>
+      <c r="C25" s="30" t="s">
+        <v>31</v>
+      </c>
+      <c r="D25" s="31" t="s">
+        <v>32</v>
+      </c>
+      <c r="E25" s="32">
+        <v>2</v>
+      </c>
+      <c r="F25" s="33">
+        <v>1</v>
+      </c>
+      <c r="G25" s="32">
+        <v>3</v>
+      </c>
+      <c r="H25" s="32">
+        <f>SUM(E25:G25)</f>
+        <v>6</v>
+      </c>
+      <c r="I25" s="34">
         <v>5</v>
-      </c>
-      <c r="I25" s="9">
-        <v>0</v>
       </c>
       <c r="J25" s="20"/>
       <c r="K25" s="1"/>
@@ -1784,32 +1787,30 @@
       <c r="M25" s="1"/>
       <c r="N25" s="1"/>
     </row>
-    <row r="26" spans="2:14" ht="83.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B26" s="34">
-        <f t="shared" ref="B26:B37" si="5">B25+1</f>
+    <row r="26" spans="2:14" ht="83.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B26" s="9">
+        <f>B24+1</f>
         <v>22</v>
       </c>
-      <c r="C26" s="54" t="s">
-        <v>62</v>
-      </c>
-      <c r="D26" s="55" t="s">
-        <v>61</v>
-      </c>
-      <c r="E26" s="32">
-        <v>2</v>
-      </c>
-      <c r="F26" s="33">
-        <v>2</v>
-      </c>
-      <c r="G26" s="32">
-        <v>2</v>
-      </c>
-      <c r="H26" s="32">
-        <f t="shared" si="1"/>
-        <v>6</v>
-      </c>
-      <c r="I26" s="34">
+      <c r="C26" s="35" t="s">
+        <v>64</v>
+      </c>
+      <c r="D26" s="51"/>
+      <c r="E26" s="52">
+        <v>1</v>
+      </c>
+      <c r="F26" s="53">
+        <v>1</v>
+      </c>
+      <c r="G26" s="52">
+        <v>3</v>
+      </c>
+      <c r="H26" s="52">
+        <f>SUM(E26:G26)</f>
         <v>5</v>
+      </c>
+      <c r="I26" s="9">
+        <v>0</v>
       </c>
       <c r="J26" s="20"/>
       <c r="K26" s="1"/>
@@ -1817,30 +1818,32 @@
       <c r="M26" s="1"/>
       <c r="N26" s="1"/>
     </row>
-    <row r="27" spans="2:14" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="B27" s="9">
-        <f t="shared" si="5"/>
+    <row r="27" spans="2:14" ht="83.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B27" s="34">
+        <f>B26+1</f>
         <v>23</v>
       </c>
-      <c r="C27" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="D27" s="12"/>
-      <c r="E27" s="21">
-        <v>1</v>
-      </c>
-      <c r="F27" s="24">
-        <v>1</v>
-      </c>
-      <c r="G27" s="21">
-        <v>3</v>
-      </c>
-      <c r="H27" s="21">
-        <f t="shared" si="1"/>
+      <c r="C27" s="54" t="s">
+        <v>62</v>
+      </c>
+      <c r="D27" s="55" t="s">
+        <v>61</v>
+      </c>
+      <c r="E27" s="32">
+        <v>2</v>
+      </c>
+      <c r="F27" s="33">
+        <v>2</v>
+      </c>
+      <c r="G27" s="32">
+        <v>2</v>
+      </c>
+      <c r="H27" s="32">
+        <f>SUM(E27:G27)</f>
+        <v>6</v>
+      </c>
+      <c r="I27" s="34">
         <v>5</v>
-      </c>
-      <c r="I27" s="9">
-        <v>0</v>
       </c>
       <c r="J27" s="20"/>
       <c r="K27" s="1"/>
@@ -1848,29 +1851,27 @@
       <c r="M27" s="1"/>
       <c r="N27" s="1"/>
     </row>
-    <row r="28" spans="2:14" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:14" ht="31.5" x14ac:dyDescent="0.25">
       <c r="B28" s="9">
-        <f t="shared" si="5"/>
+        <f>B27+1</f>
         <v>24</v>
       </c>
-      <c r="C28" s="26" t="s">
-        <v>42</v>
-      </c>
-      <c r="D28" s="12" t="s">
-        <v>43</v>
-      </c>
+      <c r="C28" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="D28" s="12"/>
       <c r="E28" s="21">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F28" s="24">
         <v>1</v>
       </c>
       <c r="G28" s="21">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H28" s="21">
-        <f t="shared" si="1"/>
-        <v>4</v>
+        <f>SUM(E28:G28)</f>
+        <v>5</v>
       </c>
       <c r="I28" s="9">
         <v>0</v>
@@ -1883,114 +1884,112 @@
     </row>
     <row r="29" spans="2:14" ht="47.25" x14ac:dyDescent="0.25">
       <c r="B29" s="9">
-        <f t="shared" si="5"/>
+        <f>B28+1</f>
         <v>25</v>
       </c>
-      <c r="C29" s="4" t="s">
-        <v>5</v>
+      <c r="C29" s="26" t="s">
+        <v>42</v>
       </c>
       <c r="D29" s="12" t="s">
-        <v>6</v>
+        <v>43</v>
       </c>
       <c r="E29" s="21">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F29" s="24">
         <v>1</v>
       </c>
       <c r="G29" s="21">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H29" s="21">
-        <f t="shared" si="1"/>
+        <f>SUM(E29:G29)</f>
         <v>4</v>
       </c>
       <c r="I29" s="9">
         <v>0</v>
       </c>
+      <c r="J29" s="20"/>
       <c r="K29" s="1"/>
       <c r="L29" s="1"/>
       <c r="M29" s="1"/>
       <c r="N29" s="1"/>
     </row>
-    <row r="30" spans="2:14" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B30" s="48">
-        <f t="shared" si="5"/>
+    <row r="30" spans="2:14" ht="47.25" x14ac:dyDescent="0.25">
+      <c r="B30" s="9">
+        <f>B29+1</f>
         <v>26</v>
       </c>
-      <c r="C30" s="44" t="s">
-        <v>44</v>
-      </c>
-      <c r="D30" s="50" t="s">
-        <v>45</v>
-      </c>
-      <c r="E30" s="46">
-        <v>2</v>
-      </c>
-      <c r="F30" s="47">
-        <v>1</v>
-      </c>
-      <c r="G30" s="46">
-        <v>1</v>
-      </c>
-      <c r="H30" s="46">
-        <f t="shared" si="1"/>
+      <c r="C30" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="D30" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="E30" s="21">
+        <v>1</v>
+      </c>
+      <c r="F30" s="24">
+        <v>1</v>
+      </c>
+      <c r="G30" s="21">
+        <v>2</v>
+      </c>
+      <c r="H30" s="21">
+        <f>SUM(E30:G30)</f>
         <v>4</v>
       </c>
-      <c r="I30" s="48">
-        <v>5</v>
-      </c>
-      <c r="J30" s="20"/>
+      <c r="I30" s="9">
+        <v>0</v>
+      </c>
       <c r="K30" s="1"/>
       <c r="L30" s="1"/>
       <c r="M30" s="1"/>
       <c r="N30" s="1"/>
     </row>
-    <row r="31" spans="2:14" ht="78.75" x14ac:dyDescent="0.25">
-      <c r="B31" s="9">
-        <f t="shared" si="5"/>
+    <row r="31" spans="2:14" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B31" s="48">
+        <f>B30+1</f>
         <v>27</v>
       </c>
-      <c r="C31" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="D31" s="12" t="s">
-        <v>34</v>
-      </c>
-      <c r="E31" s="21">
-        <v>1</v>
-      </c>
-      <c r="F31" s="24">
-        <v>1</v>
-      </c>
-      <c r="G31" s="21">
-        <v>2</v>
-      </c>
-      <c r="H31" s="21">
-        <f t="shared" si="1"/>
+      <c r="C31" s="44" t="s">
+        <v>44</v>
+      </c>
+      <c r="D31" s="50" t="s">
+        <v>45</v>
+      </c>
+      <c r="E31" s="46">
+        <v>2</v>
+      </c>
+      <c r="F31" s="47">
+        <v>1</v>
+      </c>
+      <c r="G31" s="46">
+        <v>1</v>
+      </c>
+      <c r="H31" s="46">
+        <f>SUM(E31:G31)</f>
         <v>4</v>
       </c>
-      <c r="I31" s="9">
-        <v>2</v>
-      </c>
-      <c r="J31" s="20" t="s">
-        <v>51</v>
-      </c>
+      <c r="I31" s="48">
+        <v>5</v>
+      </c>
+      <c r="J31" s="20"/>
       <c r="K31" s="1"/>
       <c r="L31" s="1"/>
       <c r="M31" s="1"/>
       <c r="N31" s="1"/>
     </row>
-    <row r="32" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:14" ht="78.75" x14ac:dyDescent="0.25">
       <c r="B32" s="9">
-        <f t="shared" si="5"/>
+        <f>B31+1</f>
         <v>28</v>
       </c>
-      <c r="C32" s="5" t="s">
-        <v>7</v>
+      <c r="C32" s="4" t="s">
+        <v>33</v>
       </c>
       <c r="D32" s="12" t="s">
-        <v>8</v>
+        <v>34</v>
       </c>
       <c r="E32" s="21">
         <v>1</v>
@@ -2002,28 +2001,30 @@
         <v>2</v>
       </c>
       <c r="H32" s="21">
-        <f t="shared" si="1"/>
+        <f>SUM(E32:G32)</f>
         <v>4</v>
       </c>
       <c r="I32" s="9">
-        <v>0</v>
-      </c>
-      <c r="J32" s="20"/>
+        <v>2</v>
+      </c>
+      <c r="J32" s="20" t="s">
+        <v>51</v>
+      </c>
       <c r="K32" s="1"/>
       <c r="L32" s="1"/>
       <c r="M32" s="1"/>
       <c r="N32" s="1"/>
     </row>
-    <row r="33" spans="2:14" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B33" s="9">
-        <f t="shared" si="5"/>
+        <f>B32+1</f>
         <v>29</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>37</v>
+        <v>7</v>
       </c>
       <c r="D33" s="12" t="s">
-        <v>38</v>
+        <v>8</v>
       </c>
       <c r="E33" s="21">
         <v>1</v>
@@ -2035,7 +2036,7 @@
         <v>2</v>
       </c>
       <c r="H33" s="21">
-        <f t="shared" si="1"/>
+        <f>SUM(E33:G33)</f>
         <v>4</v>
       </c>
       <c r="I33" s="9">
@@ -2049,14 +2050,14 @@
     </row>
     <row r="34" spans="2:14" ht="31.5" x14ac:dyDescent="0.25">
       <c r="B34" s="9">
-        <f t="shared" si="5"/>
+        <f>B33+1</f>
         <v>30</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="D34" s="12" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="E34" s="21">
         <v>1</v>
@@ -2068,7 +2069,7 @@
         <v>2</v>
       </c>
       <c r="H34" s="21">
-        <f t="shared" si="1"/>
+        <f>SUM(E34:G34)</f>
         <v>4</v>
       </c>
       <c r="I34" s="9">
@@ -2082,27 +2083,27 @@
     </row>
     <row r="35" spans="2:14" ht="31.5" x14ac:dyDescent="0.25">
       <c r="B35" s="9">
-        <f t="shared" si="5"/>
+        <f>B34+1</f>
         <v>31</v>
       </c>
-      <c r="C35" s="4" t="s">
-        <v>3</v>
+      <c r="C35" s="5" t="s">
+        <v>40</v>
       </c>
       <c r="D35" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="E35" s="21">
+        <v>1</v>
+      </c>
+      <c r="F35" s="24">
+        <v>1</v>
+      </c>
+      <c r="G35" s="21">
+        <v>2</v>
+      </c>
+      <c r="H35" s="21">
+        <f>SUM(E35:G35)</f>
         <v>4</v>
-      </c>
-      <c r="E35" s="21">
-        <v>1</v>
-      </c>
-      <c r="F35" s="24">
-        <v>1</v>
-      </c>
-      <c r="G35" s="21">
-        <v>1</v>
-      </c>
-      <c r="H35" s="21">
-        <f t="shared" si="1"/>
-        <v>3</v>
       </c>
       <c r="I35" s="9">
         <v>0</v>
@@ -2113,15 +2114,17 @@
       <c r="M35" s="1"/>
       <c r="N35" s="1"/>
     </row>
-    <row r="36" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:14" ht="31.5" x14ac:dyDescent="0.25">
       <c r="B36" s="9">
-        <f t="shared" si="5"/>
+        <f>B35+1</f>
         <v>32</v>
       </c>
-      <c r="C36" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="D36" s="12"/>
+      <c r="C36" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="D36" s="12" t="s">
+        <v>4</v>
+      </c>
       <c r="E36" s="21">
         <v>1</v>
       </c>
@@ -2132,7 +2135,7 @@
         <v>1</v>
       </c>
       <c r="H36" s="21">
-        <f t="shared" si="1"/>
+        <f>SUM(E36:G36)</f>
         <v>3</v>
       </c>
       <c r="I36" s="9">
@@ -2144,29 +2147,29 @@
       <c r="M36" s="1"/>
       <c r="N36" s="1"/>
     </row>
-    <row r="37" spans="2:14" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B37" s="9">
-        <f t="shared" si="5"/>
+        <f>B36+1</f>
         <v>33</v>
       </c>
-      <c r="C37" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="D37" s="13"/>
-      <c r="E37" s="22">
-        <v>1</v>
-      </c>
-      <c r="F37" s="25">
-        <v>1</v>
-      </c>
-      <c r="G37" s="22">
-        <v>1</v>
-      </c>
-      <c r="H37" s="22">
-        <f t="shared" si="1"/>
-        <v>3</v>
-      </c>
-      <c r="I37" s="28">
+      <c r="C37" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D37" s="12"/>
+      <c r="E37" s="21">
+        <v>1</v>
+      </c>
+      <c r="F37" s="24">
+        <v>1</v>
+      </c>
+      <c r="G37" s="21">
+        <v>1</v>
+      </c>
+      <c r="H37" s="21">
+        <f>SUM(E37:G37)</f>
+        <v>3</v>
+      </c>
+      <c r="I37" s="9">
         <v>0</v>
       </c>
       <c r="J37" s="20"/>
@@ -2175,8 +2178,31 @@
       <c r="M37" s="1"/>
       <c r="N37" s="1"/>
     </row>
-    <row r="38" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="I38" s="10"/>
+    <row r="38" spans="2:14" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B38" s="9">
+        <f>B37+1</f>
+        <v>34</v>
+      </c>
+      <c r="C38" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="D38" s="13"/>
+      <c r="E38" s="22">
+        <v>1</v>
+      </c>
+      <c r="F38" s="25">
+        <v>1</v>
+      </c>
+      <c r="G38" s="22">
+        <v>1</v>
+      </c>
+      <c r="H38" s="22">
+        <f>SUM(E38:G38)</f>
+        <v>3</v>
+      </c>
+      <c r="I38" s="28">
+        <v>0</v>
+      </c>
       <c r="J38" s="20"/>
       <c r="K38" s="1"/>
       <c r="L38" s="1"/>
@@ -2184,13 +2210,6 @@
       <c r="N38" s="1"/>
     </row>
     <row r="39" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B39" s="10"/>
-      <c r="C39" s="26"/>
-      <c r="D39" s="27"/>
-      <c r="E39" s="20"/>
-      <c r="F39" s="20"/>
-      <c r="G39" s="20"/>
-      <c r="H39" s="20"/>
       <c r="I39" s="10"/>
       <c r="J39" s="20"/>
       <c r="K39" s="1"/>
@@ -2199,13 +2218,13 @@
       <c r="N39" s="1"/>
     </row>
     <row r="40" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B40" s="1"/>
-      <c r="C40" s="7"/>
-      <c r="D40" s="2"/>
-      <c r="E40" s="10"/>
-      <c r="F40" s="10"/>
-      <c r="G40" s="10"/>
-      <c r="H40" s="10"/>
+      <c r="B40" s="10"/>
+      <c r="C40" s="26"/>
+      <c r="D40" s="27"/>
+      <c r="E40" s="20"/>
+      <c r="F40" s="20"/>
+      <c r="G40" s="20"/>
+      <c r="H40" s="20"/>
       <c r="I40" s="10"/>
       <c r="J40" s="20"/>
       <c r="K40" s="1"/>
@@ -2348,8 +2367,23 @@
       <c r="M49" s="1"/>
       <c r="N49" s="1"/>
     </row>
+    <row r="50" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B50" s="1"/>
+      <c r="C50" s="7"/>
+      <c r="D50" s="2"/>
+      <c r="E50" s="10"/>
+      <c r="F50" s="10"/>
+      <c r="G50" s="10"/>
+      <c r="H50" s="10"/>
+      <c r="I50" s="10"/>
+      <c r="J50" s="20"/>
+      <c r="K50" s="1"/>
+      <c r="L50" s="1"/>
+      <c r="M50" s="1"/>
+      <c r="N50" s="1"/>
+    </row>
   </sheetData>
-  <autoFilter ref="B3:I37" xr:uid="{11BA4F79-2AB7-4A24-A4BE-758442E1F8CB}">
+  <autoFilter ref="B3:I38" xr:uid="{11BA4F79-2AB7-4A24-A4BE-758442E1F8CB}">
     <filterColumn colId="7">
       <filters>
         <filter val="0"/>
@@ -2359,16 +2393,16 @@
         <filter val="4"/>
       </filters>
     </filterColumn>
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B5:I37">
-      <sortCondition descending="1" ref="H4:H37"/>
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B5:I38">
+      <sortCondition descending="1" ref="H4:H38"/>
     </sortState>
   </autoFilter>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B5:J37">
-    <sortCondition descending="1" ref="H4:H37"/>
-    <sortCondition descending="1" ref="E4:E37"/>
-    <sortCondition descending="1" ref="F4:F37"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B5:J38">
+    <sortCondition descending="1" ref="H4:H38"/>
+    <sortCondition descending="1" ref="E4:E38"/>
+    <sortCondition descending="1" ref="F4:F38"/>
   </sortState>
-  <conditionalFormatting sqref="H4:H37">
+  <conditionalFormatting sqref="H4:H38">
     <cfRule type="colorScale" priority="3">
       <colorScale>
         <cfvo type="min"/>
@@ -2380,7 +2414,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I4:I37">
+  <conditionalFormatting sqref="I4:I38">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>

</xml_diff>

<commit_message>
added picture and updated .ged
</commit_message>
<xml_diff>
--- a/Future Features/New Features - Family Tree.xlsx
+++ b/Future Features/New Features - Family Tree.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://srcincgov1-my.sharepoint.us/personal/lauko_srcinc_com/Documents/Desktop/Personal/geneology/GED Keepers/Future Features/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="470" documentId="8_{D1FEEEA7-0E84-49B9-AD17-37D0BB95FB37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8E01A5AA-71DE-484F-A541-9F11353F4AEF}"/>
+  <xr:revisionPtr revIDLastSave="473" documentId="8_{D1FEEEA7-0E84-49B9-AD17-37D0BB95FB37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E84B52FE-654F-48A3-8B89-57460E638892}"/>
   <bookViews>
-    <workbookView xWindow="-135" yWindow="-135" windowWidth="29070" windowHeight="15750" xr2:uid="{8067922A-00B7-4646-9500-13902203F407}"/>
+    <workbookView minimized="1" xWindow="0" yWindow="1635" windowWidth="21600" windowHeight="11295" xr2:uid="{8067922A-00B7-4646-9500-13902203F407}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1597,7 +1597,7 @@
       <c r="M18" s="1"/>
       <c r="N18" s="1"/>
     </row>
-    <row r="19" spans="2:14" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:14" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="B19" s="48">
         <f t="shared" si="1"/>
         <v>16</v>
@@ -1710,17 +1710,17 @@
         <v>80</v>
       </c>
       <c r="E22" s="21">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F22" s="24">
         <v>2</v>
       </c>
       <c r="G22" s="21">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H22" s="21">
         <f>SUM(E22:G22)</f>
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="I22" s="9">
         <v>0</v>

</xml_diff>

<commit_message>
added thumbnail viewing of attachments
</commit_message>
<xml_diff>
--- a/Future Features/New Features - Family Tree.xlsx
+++ b/Future Features/New Features - Family Tree.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://srcincgov1-my.sharepoint.us/personal/lauko_srcinc_com/Documents/Desktop/Personal/geneology/GED Keepers/Future Features/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="473" documentId="8_{D1FEEEA7-0E84-49B9-AD17-37D0BB95FB37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E84B52FE-654F-48A3-8B89-57460E638892}"/>
+  <xr:revisionPtr revIDLastSave="481" documentId="8_{D1FEEEA7-0E84-49B9-AD17-37D0BB95FB37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{97353DF2-41C5-4880-9545-0681CDEB6265}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="0" yWindow="1635" windowWidth="21600" windowHeight="11295" xr2:uid="{8067922A-00B7-4646-9500-13902203F407}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{8067922A-00B7-4646-9500-13902203F407}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$B$3:$I$41</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$B$3:$I$42</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="87">
   <si>
     <t>Feature</t>
   </si>
@@ -294,6 +294,12 @@
   </si>
   <si>
     <t>add a button that will bring the tree back to its starting spot</t>
+  </si>
+  <si>
+    <t>Trace back to "home" individual</t>
+  </si>
+  <si>
+    <t>Add a trace function that shows the relationship between a selected individual and the "home" individual</t>
   </si>
 </sst>
 </file>
@@ -1037,25 +1043,25 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{11BA4F79-2AB7-4A24-A4BE-758442E1F8CB}">
   <sheetPr filterMode="1"/>
-  <dimension ref="B1:N53"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="B1:N54"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="3" max="3" width="49.28515625" style="8" customWidth="1"/>
-    <col min="4" max="4" width="57.85546875" style="3" customWidth="1"/>
-    <col min="5" max="5" width="9.140625" style="11"/>
-    <col min="6" max="6" width="12.42578125" style="11" customWidth="1"/>
-    <col min="7" max="8" width="9.140625" style="11"/>
-    <col min="9" max="9" width="14.28515625" style="11" customWidth="1"/>
-    <col min="10" max="10" width="65.7109375" style="41" customWidth="1"/>
+    <col min="3" max="3" width="49.33203125" style="8" customWidth="1"/>
+    <col min="4" max="4" width="57.88671875" style="3" customWidth="1"/>
+    <col min="5" max="5" width="9.109375" style="11"/>
+    <col min="6" max="6" width="12.44140625" style="11" customWidth="1"/>
+    <col min="7" max="8" width="9.109375" style="11"/>
+    <col min="9" max="9" width="14.33203125" style="11" customWidth="1"/>
+    <col min="10" max="10" width="65.6640625" style="41" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="1" spans="2:14" x14ac:dyDescent="0.3">
       <c r="E1" s="19"/>
       <c r="F1" s="19"/>
       <c r="G1" s="19"/>
       <c r="H1" s="19"/>
     </row>
-    <row r="2" spans="2:14" ht="63.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:14" ht="63" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B2" s="10"/>
       <c r="C2" s="20"/>
       <c r="D2" s="20"/>
@@ -1076,7 +1082,7 @@
       <c r="M2" s="1"/>
       <c r="N2" s="1"/>
     </row>
-    <row r="3" spans="2:14" s="3" customFormat="1" ht="48" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:14" s="3" customFormat="1" ht="47.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B3" s="18"/>
       <c r="C3" s="15" t="s">
         <v>0</v>
@@ -1105,7 +1111,7 @@
       <c r="M3" s="2"/>
       <c r="N3" s="2"/>
     </row>
-    <row r="4" spans="2:14" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:14" ht="31.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="B4" s="14">
         <v>1</v>
       </c>
@@ -1137,9 +1143,9 @@
       <c r="M4" s="1"/>
       <c r="N4" s="1"/>
     </row>
-    <row r="5" spans="2:14" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:14" ht="31.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="B5" s="48">
-        <f>B4+1</f>
+        <f t="shared" ref="B5:B16" si="1">B4+1</f>
         <v>2</v>
       </c>
       <c r="C5" s="44" t="s">
@@ -1156,7 +1162,7 @@
         <v>2</v>
       </c>
       <c r="H5" s="46">
-        <f>SUM(E5:G5)</f>
+        <f t="shared" ref="H5:H19" si="2">SUM(E5:G5)</f>
         <v>8</v>
       </c>
       <c r="I5" s="48">
@@ -1168,9 +1174,9 @@
       <c r="M5" s="1"/>
       <c r="N5" s="1"/>
     </row>
-    <row r="6" spans="2:14" ht="47.25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:14" ht="46.8" hidden="1" x14ac:dyDescent="0.3">
       <c r="B6" s="9">
-        <f>B5+1</f>
+        <f t="shared" si="1"/>
         <v>3</v>
       </c>
       <c r="C6" s="44" t="s">
@@ -1189,7 +1195,7 @@
         <v>2</v>
       </c>
       <c r="H6" s="46">
-        <f>SUM(E6:G6)</f>
+        <f t="shared" si="2"/>
         <v>7</v>
       </c>
       <c r="I6" s="48">
@@ -1201,9 +1207,9 @@
       <c r="M6" s="1"/>
       <c r="N6" s="1"/>
     </row>
-    <row r="7" spans="2:14" ht="78.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:14" ht="78" hidden="1" x14ac:dyDescent="0.3">
       <c r="B7" s="9">
-        <f>B6+1</f>
+        <f t="shared" si="1"/>
         <v>4</v>
       </c>
       <c r="C7" s="30" t="s">
@@ -1222,7 +1228,7 @@
         <v>3</v>
       </c>
       <c r="H7" s="32">
-        <f>SUM(E7:G7)</f>
+        <f t="shared" si="2"/>
         <v>7</v>
       </c>
       <c r="I7" s="34">
@@ -1234,9 +1240,9 @@
       <c r="M7" s="1"/>
       <c r="N7" s="1"/>
     </row>
-    <row r="8" spans="2:14" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:14" ht="31.2" x14ac:dyDescent="0.3">
       <c r="B8" s="9">
-        <f>B7+1</f>
+        <f t="shared" si="1"/>
         <v>5</v>
       </c>
       <c r="C8" s="4" t="s">
@@ -1255,7 +1261,7 @@
         <v>2</v>
       </c>
       <c r="H8" s="21">
-        <f>SUM(E8:G8)</f>
+        <f t="shared" si="2"/>
         <v>7</v>
       </c>
       <c r="I8" s="9">
@@ -1267,9 +1273,9 @@
       <c r="M8" s="1"/>
       <c r="N8" s="1"/>
     </row>
-    <row r="9" spans="2:14" ht="47.25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:14" ht="46.8" hidden="1" x14ac:dyDescent="0.3">
       <c r="B9" s="9">
-        <f>B8+1</f>
+        <f t="shared" si="1"/>
         <v>6</v>
       </c>
       <c r="C9" s="44" t="s">
@@ -1288,7 +1294,7 @@
         <v>3</v>
       </c>
       <c r="H9" s="46">
-        <f>SUM(E9:G9)</f>
+        <f t="shared" si="2"/>
         <v>9</v>
       </c>
       <c r="I9" s="48">
@@ -1299,9 +1305,9 @@
       <c r="M9" s="1"/>
       <c r="N9" s="1"/>
     </row>
-    <row r="10" spans="2:14" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:14" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B10" s="48">
-        <f>B9+1</f>
+        <f t="shared" si="1"/>
         <v>7</v>
       </c>
       <c r="C10" s="44" t="s">
@@ -1320,7 +1326,7 @@
         <v>3</v>
       </c>
       <c r="H10" s="46">
-        <f>SUM(E10:G10)</f>
+        <f t="shared" si="2"/>
         <v>8</v>
       </c>
       <c r="I10" s="48">
@@ -1331,9 +1337,9 @@
       <c r="M10" s="1"/>
       <c r="N10" s="1"/>
     </row>
-    <row r="11" spans="2:14" ht="47.25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:14" ht="46.8" hidden="1" x14ac:dyDescent="0.3">
       <c r="B11" s="48">
-        <f>B10+1</f>
+        <f t="shared" si="1"/>
         <v>8</v>
       </c>
       <c r="C11" s="44" t="s">
@@ -1352,7 +1358,7 @@
         <v>2</v>
       </c>
       <c r="H11" s="46">
-        <f>SUM(E11:G11)</f>
+        <f t="shared" si="2"/>
         <v>7</v>
       </c>
       <c r="I11" s="48">
@@ -1363,9 +1369,9 @@
       <c r="M11" s="1"/>
       <c r="N11" s="1"/>
     </row>
-    <row r="12" spans="2:14" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:14" ht="31.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="B12" s="48">
-        <f>B11+1</f>
+        <f t="shared" si="1"/>
         <v>9</v>
       </c>
       <c r="C12" s="49" t="s">
@@ -1382,7 +1388,7 @@
         <v>3</v>
       </c>
       <c r="H12" s="46">
-        <f>SUM(E12:G12)</f>
+        <f t="shared" si="2"/>
         <v>7</v>
       </c>
       <c r="I12" s="48">
@@ -1396,9 +1402,9 @@
       <c r="M12" s="1"/>
       <c r="N12" s="1"/>
     </row>
-    <row r="13" spans="2:14" ht="63" hidden="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:14" ht="62.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="B13" s="9">
-        <f>B12+1</f>
+        <f t="shared" si="1"/>
         <v>10</v>
       </c>
       <c r="C13" s="30" t="s">
@@ -1417,7 +1423,7 @@
         <v>2</v>
       </c>
       <c r="H13" s="32">
-        <f>SUM(E13:G13)</f>
+        <f t="shared" si="2"/>
         <v>6</v>
       </c>
       <c r="I13" s="34">
@@ -1429,9 +1435,9 @@
       <c r="M13" s="1"/>
       <c r="N13" s="1"/>
     </row>
-    <row r="14" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B14" s="9">
-        <f>B13+1</f>
+        <f t="shared" si="1"/>
         <v>11</v>
       </c>
       <c r="C14" s="35" t="s">
@@ -1450,7 +1456,7 @@
         <v>2</v>
       </c>
       <c r="H14" s="21">
-        <f>SUM(E14:G14)</f>
+        <f t="shared" si="2"/>
         <v>7</v>
       </c>
       <c r="I14" s="9">
@@ -1464,9 +1470,9 @@
       <c r="M14" s="1"/>
       <c r="N14" s="1"/>
     </row>
-    <row r="15" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B15" s="9">
-        <f>B14+1</f>
+        <f t="shared" si="1"/>
         <v>12</v>
       </c>
       <c r="C15" s="4" t="s">
@@ -1485,7 +1491,7 @@
         <v>2</v>
       </c>
       <c r="H15" s="21">
-        <f>SUM(E15:G15)</f>
+        <f t="shared" si="2"/>
         <v>7</v>
       </c>
       <c r="I15" s="9">
@@ -1497,9 +1503,9 @@
       <c r="M15" s="1"/>
       <c r="N15" s="1"/>
     </row>
-    <row r="16" spans="2:14" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:14" ht="31.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="B16" s="48">
-        <f>B15+1</f>
+        <f t="shared" si="1"/>
         <v>13</v>
       </c>
       <c r="C16" s="44" t="s">
@@ -1518,7 +1524,7 @@
         <v>2</v>
       </c>
       <c r="H16" s="46">
-        <f>SUM(E16:G16)</f>
+        <f t="shared" si="2"/>
         <v>7</v>
       </c>
       <c r="I16" s="48">
@@ -1529,9 +1535,9 @@
       <c r="M16" s="1"/>
       <c r="N16" s="1"/>
     </row>
-    <row r="17" spans="2:14" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:14" ht="31.2" x14ac:dyDescent="0.3">
       <c r="B17" s="9">
-        <f t="shared" ref="B17:B20" si="1">B16+1</f>
+        <f t="shared" ref="B17:B21" si="3">B16+1</f>
         <v>14</v>
       </c>
       <c r="C17" s="56" t="s">
@@ -1550,7 +1556,7 @@
         <v>3</v>
       </c>
       <c r="H17" s="52">
-        <f>SUM(E17:G17)</f>
+        <f t="shared" si="2"/>
         <v>7</v>
       </c>
       <c r="I17" s="58">
@@ -1562,119 +1568,117 @@
       <c r="M17" s="1"/>
       <c r="N17" s="1"/>
     </row>
-    <row r="18" spans="2:14" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:14" ht="31.2" x14ac:dyDescent="0.3">
       <c r="B18" s="9">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>15</v>
       </c>
-      <c r="C18" s="35" t="s">
-        <v>66</v>
-      </c>
-      <c r="D18" s="35" t="s">
-        <v>69</v>
-      </c>
-      <c r="E18" s="42">
-        <v>2</v>
-      </c>
-      <c r="F18" s="43">
-        <v>2</v>
-      </c>
-      <c r="G18" s="42">
-        <v>3</v>
-      </c>
-      <c r="H18" s="21">
-        <f>SUM(E18:G18)</f>
-        <v>7</v>
-      </c>
-      <c r="I18" s="9">
-        <v>3</v>
-      </c>
-      <c r="J18" s="20" t="s">
-        <v>70</v>
-      </c>
+      <c r="C18" s="56" t="s">
+        <v>85</v>
+      </c>
+      <c r="D18" s="51" t="s">
+        <v>86</v>
+      </c>
+      <c r="E18" s="52">
+        <v>2</v>
+      </c>
+      <c r="F18" s="53">
+        <v>2</v>
+      </c>
+      <c r="G18" s="52">
+        <v>2</v>
+      </c>
+      <c r="H18" s="52">
+        <f t="shared" si="2"/>
+        <v>6</v>
+      </c>
+      <c r="I18" s="58">
+        <v>0</v>
+      </c>
+      <c r="J18" s="57"/>
       <c r="K18" s="1"/>
       <c r="L18" s="1"/>
       <c r="M18" s="1"/>
       <c r="N18" s="1"/>
     </row>
-    <row r="19" spans="2:14" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B19" s="48">
-        <f t="shared" si="1"/>
+    <row r="19" spans="2:14" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="B19" s="9">
+        <f t="shared" si="3"/>
         <v>16</v>
       </c>
-      <c r="C19" s="49" t="s">
-        <v>83</v>
-      </c>
-      <c r="D19" s="49" t="s">
-        <v>84</v>
-      </c>
-      <c r="E19" s="59">
-        <v>3</v>
-      </c>
-      <c r="F19" s="60">
-        <v>2</v>
-      </c>
-      <c r="G19" s="59">
-        <v>3</v>
-      </c>
-      <c r="H19" s="46">
-        <f t="shared" ref="H19:H20" si="2">SUM(E19:G19)</f>
-        <v>8</v>
-      </c>
-      <c r="I19" s="48">
-        <v>5</v>
-      </c>
-      <c r="J19" s="61"/>
+      <c r="C19" s="35" t="s">
+        <v>66</v>
+      </c>
+      <c r="D19" s="35" t="s">
+        <v>69</v>
+      </c>
+      <c r="E19" s="42">
+        <v>2</v>
+      </c>
+      <c r="F19" s="43">
+        <v>2</v>
+      </c>
+      <c r="G19" s="42">
+        <v>3</v>
+      </c>
+      <c r="H19" s="21">
+        <f t="shared" si="2"/>
+        <v>7</v>
+      </c>
+      <c r="I19" s="9">
+        <v>3</v>
+      </c>
+      <c r="J19" s="20" t="s">
+        <v>70</v>
+      </c>
       <c r="K19" s="1"/>
       <c r="L19" s="1"/>
       <c r="M19" s="1"/>
       <c r="N19" s="1"/>
     </row>
-    <row r="20" spans="2:14" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="B20" s="9">
-        <f t="shared" si="1"/>
+    <row r="20" spans="2:14" ht="31.2" hidden="1" x14ac:dyDescent="0.3">
+      <c r="B20" s="48">
+        <f t="shared" si="3"/>
         <v>17</v>
       </c>
-      <c r="C20" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="D20" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="E20" s="21">
-        <v>2</v>
-      </c>
-      <c r="F20" s="24">
-        <v>2</v>
-      </c>
-      <c r="G20" s="21">
-        <v>2</v>
-      </c>
-      <c r="H20" s="21">
-        <f t="shared" si="2"/>
-        <v>6</v>
-      </c>
-      <c r="I20" s="9">
-        <v>2</v>
-      </c>
-      <c r="J20" s="20" t="s">
-        <v>63</v>
-      </c>
+      <c r="C20" s="49" t="s">
+        <v>83</v>
+      </c>
+      <c r="D20" s="49" t="s">
+        <v>84</v>
+      </c>
+      <c r="E20" s="59">
+        <v>3</v>
+      </c>
+      <c r="F20" s="60">
+        <v>2</v>
+      </c>
+      <c r="G20" s="59">
+        <v>3</v>
+      </c>
+      <c r="H20" s="46">
+        <f t="shared" ref="H20:H21" si="4">SUM(E20:G20)</f>
+        <v>8</v>
+      </c>
+      <c r="I20" s="48">
+        <v>5</v>
+      </c>
+      <c r="J20" s="61"/>
       <c r="K20" s="1"/>
       <c r="L20" s="1"/>
       <c r="M20" s="1"/>
       <c r="N20" s="1"/>
     </row>
-    <row r="21" spans="2:14" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:14" ht="31.2" x14ac:dyDescent="0.3">
       <c r="B21" s="9">
-        <f>B20+1</f>
+        <f t="shared" si="3"/>
         <v>18</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="D21" s="23" t="s">
-        <v>21</v>
+        <v>11</v>
+      </c>
+      <c r="D21" s="5" t="s">
+        <v>12</v>
       </c>
       <c r="E21" s="21">
         <v>2</v>
@@ -1686,41 +1690,43 @@
         <v>2</v>
       </c>
       <c r="H21" s="21">
-        <f>SUM(E21:G21)</f>
+        <f t="shared" si="4"/>
         <v>6</v>
       </c>
       <c r="I21" s="9">
-        <v>0</v>
-      </c>
-      <c r="J21" s="20"/>
+        <v>2</v>
+      </c>
+      <c r="J21" s="20" t="s">
+        <v>63</v>
+      </c>
       <c r="K21" s="1"/>
       <c r="L21" s="1"/>
       <c r="M21" s="1"/>
       <c r="N21" s="1"/>
     </row>
-    <row r="22" spans="2:14" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:14" ht="31.2" x14ac:dyDescent="0.3">
       <c r="B22" s="9">
-        <f>B21+1</f>
+        <f t="shared" ref="B22:B29" si="5">B21+1</f>
         <v>19</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>79</v>
+        <v>20</v>
       </c>
       <c r="D22" s="23" t="s">
-        <v>80</v>
+        <v>21</v>
       </c>
       <c r="E22" s="21">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F22" s="24">
         <v>2</v>
       </c>
       <c r="G22" s="21">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H22" s="21">
-        <f>SUM(E22:G22)</f>
-        <v>4</v>
+        <f t="shared" ref="H22:H42" si="6">SUM(E22:G22)</f>
+        <v>6</v>
       </c>
       <c r="I22" s="9">
         <v>0</v>
@@ -1731,29 +1737,29 @@
       <c r="M22" s="1"/>
       <c r="N22" s="1"/>
     </row>
-    <row r="23" spans="2:14" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:14" ht="31.2" x14ac:dyDescent="0.3">
       <c r="B23" s="9">
-        <f>B22+1</f>
+        <f t="shared" si="5"/>
         <v>20</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="D23" s="5" t="s">
-        <v>48</v>
+        <v>79</v>
+      </c>
+      <c r="D23" s="23" t="s">
+        <v>80</v>
       </c>
       <c r="E23" s="21">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F23" s="24">
         <v>2</v>
       </c>
       <c r="G23" s="21">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H23" s="21">
-        <f>SUM(E23:G23)</f>
-        <v>6</v>
+        <f t="shared" si="6"/>
+        <v>4</v>
       </c>
       <c r="I23" s="9">
         <v>0</v>
@@ -1764,32 +1770,32 @@
       <c r="M23" s="1"/>
       <c r="N23" s="1"/>
     </row>
-    <row r="24" spans="2:14" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B24" s="48">
-        <f>B23+1</f>
+    <row r="24" spans="2:14" ht="46.8" x14ac:dyDescent="0.3">
+      <c r="B24" s="9">
+        <f t="shared" si="5"/>
         <v>21</v>
       </c>
-      <c r="C24" s="44" t="s">
-        <v>39</v>
-      </c>
-      <c r="D24" s="50" t="s">
-        <v>71</v>
-      </c>
-      <c r="E24" s="46">
-        <v>1</v>
-      </c>
-      <c r="F24" s="47">
-        <v>2</v>
-      </c>
-      <c r="G24" s="46">
-        <v>3</v>
-      </c>
-      <c r="H24" s="46">
-        <f>SUM(E24:G24)</f>
+      <c r="C24" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="D24" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="E24" s="21">
+        <v>2</v>
+      </c>
+      <c r="F24" s="24">
+        <v>2</v>
+      </c>
+      <c r="G24" s="21">
+        <v>2</v>
+      </c>
+      <c r="H24" s="21">
+        <f t="shared" si="6"/>
         <v>6</v>
       </c>
-      <c r="I24" s="48">
-        <v>5</v>
+      <c r="I24" s="9">
+        <v>0</v>
       </c>
       <c r="J24" s="20"/>
       <c r="K24" s="1"/>
@@ -1797,32 +1803,32 @@
       <c r="M24" s="1"/>
       <c r="N24" s="1"/>
     </row>
-    <row r="25" spans="2:14" ht="47.25" x14ac:dyDescent="0.25">
-      <c r="B25" s="9">
-        <f>B24+1</f>
+    <row r="25" spans="2:14" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+      <c r="B25" s="48">
+        <f t="shared" si="5"/>
         <v>22</v>
       </c>
-      <c r="C25" s="23" t="s">
-        <v>22</v>
-      </c>
-      <c r="D25" s="23" t="s">
-        <v>23</v>
-      </c>
-      <c r="E25" s="21">
-        <v>2</v>
-      </c>
-      <c r="F25" s="24">
-        <v>2</v>
-      </c>
-      <c r="G25" s="21">
-        <v>1</v>
-      </c>
-      <c r="H25" s="21">
-        <f>SUM(E25:G25)</f>
+      <c r="C25" s="44" t="s">
+        <v>39</v>
+      </c>
+      <c r="D25" s="50" t="s">
+        <v>71</v>
+      </c>
+      <c r="E25" s="46">
+        <v>1</v>
+      </c>
+      <c r="F25" s="47">
+        <v>2</v>
+      </c>
+      <c r="G25" s="46">
+        <v>3</v>
+      </c>
+      <c r="H25" s="46">
+        <f t="shared" si="6"/>
+        <v>6</v>
+      </c>
+      <c r="I25" s="48">
         <v>5</v>
-      </c>
-      <c r="I25" s="9">
-        <v>0</v>
       </c>
       <c r="J25" s="20"/>
       <c r="K25" s="1"/>
@@ -1830,28 +1836,28 @@
       <c r="M25" s="1"/>
       <c r="N25" s="1"/>
     </row>
-    <row r="26" spans="2:14" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:14" ht="46.8" x14ac:dyDescent="0.3">
       <c r="B26" s="9">
-        <f>B25+1</f>
+        <f t="shared" si="5"/>
         <v>23</v>
       </c>
-      <c r="C26" s="5" t="s">
-        <v>56</v>
+      <c r="C26" s="23" t="s">
+        <v>22</v>
       </c>
       <c r="D26" s="23" t="s">
-        <v>57</v>
+        <v>23</v>
       </c>
       <c r="E26" s="21">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F26" s="24">
         <v>2</v>
       </c>
       <c r="G26" s="21">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H26" s="21">
-        <f>SUM(E26:G26)</f>
+        <f t="shared" si="6"/>
         <v>5</v>
       </c>
       <c r="I26" s="9">
@@ -1863,16 +1869,16 @@
       <c r="M26" s="1"/>
       <c r="N26" s="1"/>
     </row>
-    <row r="27" spans="2:14" ht="83.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:14" ht="31.2" x14ac:dyDescent="0.3">
       <c r="B27" s="9">
-        <f>B26+1</f>
+        <f t="shared" si="5"/>
         <v>24</v>
       </c>
-      <c r="C27" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="D27" s="12" t="s">
-        <v>35</v>
+      <c r="C27" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="D27" s="23" t="s">
+        <v>57</v>
       </c>
       <c r="E27" s="21">
         <v>1</v>
@@ -1884,74 +1890,76 @@
         <v>2</v>
       </c>
       <c r="H27" s="21">
-        <f>SUM(E27:G27)</f>
+        <f t="shared" si="6"/>
         <v>5</v>
       </c>
       <c r="I27" s="9">
         <v>0</v>
       </c>
+      <c r="J27" s="20"/>
       <c r="K27" s="1"/>
       <c r="L27" s="1"/>
       <c r="M27" s="1"/>
       <c r="N27" s="1"/>
     </row>
-    <row r="28" spans="2:14" ht="83.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B28" s="29">
-        <f>B27+1</f>
+    <row r="28" spans="2:14" ht="83.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B28" s="9">
+        <f t="shared" si="5"/>
         <v>25</v>
       </c>
-      <c r="C28" s="30" t="s">
-        <v>31</v>
-      </c>
-      <c r="D28" s="31" t="s">
-        <v>32</v>
-      </c>
-      <c r="E28" s="32">
-        <v>2</v>
-      </c>
-      <c r="F28" s="33">
-        <v>1</v>
-      </c>
-      <c r="G28" s="32">
-        <v>3</v>
-      </c>
-      <c r="H28" s="32">
-        <f>SUM(E28:G28)</f>
-        <v>6</v>
-      </c>
-      <c r="I28" s="34">
+      <c r="C28" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="D28" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="E28" s="21">
+        <v>1</v>
+      </c>
+      <c r="F28" s="24">
+        <v>2</v>
+      </c>
+      <c r="G28" s="21">
+        <v>2</v>
+      </c>
+      <c r="H28" s="21">
+        <f t="shared" si="6"/>
         <v>5</v>
       </c>
-      <c r="J28" s="20"/>
+      <c r="I28" s="9">
+        <v>0</v>
+      </c>
       <c r="K28" s="1"/>
       <c r="L28" s="1"/>
       <c r="M28" s="1"/>
       <c r="N28" s="1"/>
     </row>
-    <row r="29" spans="2:14" ht="83.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B29" s="9">
-        <f>B27+1</f>
-        <v>25</v>
-      </c>
-      <c r="C29" s="35" t="s">
-        <v>64</v>
-      </c>
-      <c r="D29" s="51"/>
-      <c r="E29" s="52">
-        <v>1</v>
-      </c>
-      <c r="F29" s="53">
-        <v>1</v>
-      </c>
-      <c r="G29" s="52">
-        <v>3</v>
-      </c>
-      <c r="H29" s="52">
-        <f>SUM(E29:G29)</f>
+    <row r="29" spans="2:14" ht="83.25" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B29" s="29">
+        <f t="shared" si="5"/>
+        <v>26</v>
+      </c>
+      <c r="C29" s="30" t="s">
+        <v>31</v>
+      </c>
+      <c r="D29" s="31" t="s">
+        <v>32</v>
+      </c>
+      <c r="E29" s="32">
+        <v>2</v>
+      </c>
+      <c r="F29" s="33">
+        <v>1</v>
+      </c>
+      <c r="G29" s="32">
+        <v>3</v>
+      </c>
+      <c r="H29" s="32">
+        <f t="shared" si="6"/>
+        <v>6</v>
+      </c>
+      <c r="I29" s="34">
         <v>5</v>
-      </c>
-      <c r="I29" s="9">
-        <v>0</v>
       </c>
       <c r="J29" s="20"/>
       <c r="K29" s="1"/>
@@ -1959,32 +1967,30 @@
       <c r="M29" s="1"/>
       <c r="N29" s="1"/>
     </row>
-    <row r="30" spans="2:14" ht="83.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B30" s="34">
-        <f>B29+1</f>
+    <row r="30" spans="2:14" ht="83.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B30" s="9">
+        <f>B28+1</f>
         <v>26</v>
       </c>
-      <c r="C30" s="54" t="s">
-        <v>62</v>
-      </c>
-      <c r="D30" s="55" t="s">
-        <v>61</v>
-      </c>
-      <c r="E30" s="32">
-        <v>2</v>
-      </c>
-      <c r="F30" s="33">
-        <v>2</v>
-      </c>
-      <c r="G30" s="32">
-        <v>2</v>
-      </c>
-      <c r="H30" s="32">
-        <f>SUM(E30:G30)</f>
-        <v>6</v>
-      </c>
-      <c r="I30" s="34">
+      <c r="C30" s="35" t="s">
+        <v>64</v>
+      </c>
+      <c r="D30" s="51"/>
+      <c r="E30" s="52">
+        <v>1</v>
+      </c>
+      <c r="F30" s="53">
+        <v>1</v>
+      </c>
+      <c r="G30" s="52">
+        <v>3</v>
+      </c>
+      <c r="H30" s="52">
+        <f t="shared" si="6"/>
         <v>5</v>
+      </c>
+      <c r="I30" s="9">
+        <v>0</v>
       </c>
       <c r="J30" s="20"/>
       <c r="K30" s="1"/>
@@ -1992,29 +1998,31 @@
       <c r="M30" s="1"/>
       <c r="N30" s="1"/>
     </row>
-    <row r="31" spans="2:14" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B31" s="48">
-        <f>B30+1</f>
+    <row r="31" spans="2:14" ht="83.25" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B31" s="34">
+        <f t="shared" ref="B31:B42" si="7">B30+1</f>
         <v>27</v>
       </c>
-      <c r="C31" s="49" t="s">
-        <v>59</v>
-      </c>
-      <c r="D31" s="50"/>
-      <c r="E31" s="46">
-        <v>1</v>
-      </c>
-      <c r="F31" s="47">
-        <v>1</v>
-      </c>
-      <c r="G31" s="46">
-        <v>3</v>
-      </c>
-      <c r="H31" s="46">
-        <f>SUM(E31:G31)</f>
-        <v>5</v>
-      </c>
-      <c r="I31" s="48">
+      <c r="C31" s="54" t="s">
+        <v>62</v>
+      </c>
+      <c r="D31" s="55" t="s">
+        <v>61</v>
+      </c>
+      <c r="E31" s="32">
+        <v>2</v>
+      </c>
+      <c r="F31" s="33">
+        <v>2</v>
+      </c>
+      <c r="G31" s="32">
+        <v>2</v>
+      </c>
+      <c r="H31" s="32">
+        <f t="shared" si="6"/>
+        <v>6</v>
+      </c>
+      <c r="I31" s="34">
         <v>5</v>
       </c>
       <c r="J31" s="20"/>
@@ -2023,32 +2031,30 @@
       <c r="M31" s="1"/>
       <c r="N31" s="1"/>
     </row>
-    <row r="32" spans="2:14" ht="47.25" x14ac:dyDescent="0.25">
-      <c r="B32" s="9">
-        <f>B31+1</f>
+    <row r="32" spans="2:14" ht="31.2" hidden="1" x14ac:dyDescent="0.3">
+      <c r="B32" s="48">
+        <f t="shared" si="7"/>
         <v>28</v>
       </c>
-      <c r="C32" s="26" t="s">
-        <v>42</v>
-      </c>
-      <c r="D32" s="12" t="s">
-        <v>43</v>
-      </c>
-      <c r="E32" s="21">
-        <v>2</v>
-      </c>
-      <c r="F32" s="24">
-        <v>1</v>
-      </c>
-      <c r="G32" s="21">
-        <v>1</v>
-      </c>
-      <c r="H32" s="21">
-        <f>SUM(E32:G32)</f>
-        <v>4</v>
-      </c>
-      <c r="I32" s="9">
-        <v>0</v>
+      <c r="C32" s="49" t="s">
+        <v>59</v>
+      </c>
+      <c r="D32" s="50"/>
+      <c r="E32" s="46">
+        <v>1</v>
+      </c>
+      <c r="F32" s="47">
+        <v>1</v>
+      </c>
+      <c r="G32" s="46">
+        <v>3</v>
+      </c>
+      <c r="H32" s="46">
+        <f t="shared" si="6"/>
+        <v>5</v>
+      </c>
+      <c r="I32" s="48">
+        <v>5</v>
       </c>
       <c r="J32" s="20"/>
       <c r="K32" s="1"/>
@@ -2056,149 +2062,149 @@
       <c r="M32" s="1"/>
       <c r="N32" s="1"/>
     </row>
-    <row r="33" spans="2:14" ht="47.25" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B33" s="48">
-        <f>B32+1</f>
+    <row r="33" spans="2:14" ht="46.8" x14ac:dyDescent="0.3">
+      <c r="B33" s="9">
+        <f t="shared" si="7"/>
         <v>29</v>
       </c>
-      <c r="C33" s="49" t="s">
-        <v>5</v>
-      </c>
-      <c r="D33" s="50" t="s">
-        <v>6</v>
-      </c>
-      <c r="E33" s="46">
-        <v>1</v>
-      </c>
-      <c r="F33" s="47">
-        <v>1</v>
-      </c>
-      <c r="G33" s="46">
-        <v>2</v>
-      </c>
-      <c r="H33" s="46">
-        <f>SUM(E33:G33)</f>
+      <c r="C33" s="26" t="s">
+        <v>42</v>
+      </c>
+      <c r="D33" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="E33" s="21">
+        <v>2</v>
+      </c>
+      <c r="F33" s="24">
+        <v>1</v>
+      </c>
+      <c r="G33" s="21">
+        <v>1</v>
+      </c>
+      <c r="H33" s="21">
+        <f t="shared" si="6"/>
         <v>4</v>
       </c>
-      <c r="I33" s="48">
-        <v>5</v>
-      </c>
+      <c r="I33" s="9">
+        <v>0</v>
+      </c>
+      <c r="J33" s="20"/>
       <c r="K33" s="1"/>
       <c r="L33" s="1"/>
       <c r="M33" s="1"/>
       <c r="N33" s="1"/>
     </row>
-    <row r="34" spans="2:14" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:14" ht="31.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="B34" s="48">
-        <f>B33+1</f>
+        <f t="shared" si="7"/>
         <v>30</v>
       </c>
-      <c r="C34" s="44" t="s">
-        <v>44</v>
+      <c r="C34" s="49" t="s">
+        <v>5</v>
       </c>
       <c r="D34" s="50" t="s">
-        <v>45</v>
+        <v>6</v>
       </c>
       <c r="E34" s="46">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F34" s="47">
         <v>1</v>
       </c>
       <c r="G34" s="46">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H34" s="46">
-        <f>SUM(E34:G34)</f>
+        <f t="shared" si="6"/>
         <v>4</v>
       </c>
       <c r="I34" s="48">
         <v>5</v>
       </c>
-      <c r="J34" s="20"/>
       <c r="K34" s="1"/>
       <c r="L34" s="1"/>
       <c r="M34" s="1"/>
       <c r="N34" s="1"/>
     </row>
-    <row r="35" spans="2:14" ht="78.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:14" ht="31.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="B35" s="48">
-        <f>B34+1</f>
+        <f t="shared" si="7"/>
         <v>31</v>
       </c>
-      <c r="C35" s="49" t="s">
-        <v>33</v>
+      <c r="C35" s="44" t="s">
+        <v>44</v>
       </c>
       <c r="D35" s="50" t="s">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="E35" s="46">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F35" s="47">
         <v>1</v>
       </c>
       <c r="G35" s="46">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H35" s="46">
-        <f>SUM(E35:G35)</f>
+        <f t="shared" si="6"/>
         <v>4</v>
       </c>
       <c r="I35" s="48">
         <v>5</v>
       </c>
-      <c r="J35" s="20" t="s">
-        <v>51</v>
-      </c>
+      <c r="J35" s="20"/>
       <c r="K35" s="1"/>
       <c r="L35" s="1"/>
       <c r="M35" s="1"/>
       <c r="N35" s="1"/>
     </row>
-    <row r="36" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B36" s="9">
-        <f>B35+1</f>
+    <row r="36" spans="2:14" ht="78" hidden="1" x14ac:dyDescent="0.3">
+      <c r="B36" s="48">
+        <f t="shared" si="7"/>
         <v>32</v>
       </c>
-      <c r="C36" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="D36" s="12" t="s">
-        <v>8</v>
-      </c>
-      <c r="E36" s="21">
-        <v>1</v>
-      </c>
-      <c r="F36" s="24">
-        <v>1</v>
-      </c>
-      <c r="G36" s="21">
-        <v>2</v>
-      </c>
-      <c r="H36" s="21">
-        <f>SUM(E36:G36)</f>
+      <c r="C36" s="49" t="s">
+        <v>33</v>
+      </c>
+      <c r="D36" s="50" t="s">
+        <v>34</v>
+      </c>
+      <c r="E36" s="46">
+        <v>1</v>
+      </c>
+      <c r="F36" s="47">
+        <v>1</v>
+      </c>
+      <c r="G36" s="46">
+        <v>2</v>
+      </c>
+      <c r="H36" s="46">
+        <f t="shared" si="6"/>
         <v>4</v>
       </c>
-      <c r="I36" s="9">
-        <v>0</v>
-      </c>
-      <c r="J36" s="20"/>
+      <c r="I36" s="48">
+        <v>5</v>
+      </c>
+      <c r="J36" s="20" t="s">
+        <v>51</v>
+      </c>
       <c r="K36" s="1"/>
       <c r="L36" s="1"/>
       <c r="M36" s="1"/>
       <c r="N36" s="1"/>
     </row>
-    <row r="37" spans="2:14" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B37" s="9">
-        <f>B36+1</f>
+        <f t="shared" si="7"/>
         <v>33</v>
       </c>
       <c r="C37" s="5" t="s">
-        <v>37</v>
+        <v>7</v>
       </c>
       <c r="D37" s="12" t="s">
-        <v>38</v>
+        <v>8</v>
       </c>
       <c r="E37" s="21">
         <v>1</v>
@@ -2210,7 +2216,7 @@
         <v>2</v>
       </c>
       <c r="H37" s="21">
-        <f>SUM(E37:G37)</f>
+        <f t="shared" si="6"/>
         <v>4</v>
       </c>
       <c r="I37" s="9">
@@ -2222,16 +2228,16 @@
       <c r="M37" s="1"/>
       <c r="N37" s="1"/>
     </row>
-    <row r="38" spans="2:14" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:14" ht="31.2" x14ac:dyDescent="0.3">
       <c r="B38" s="9">
-        <f>B37+1</f>
+        <f t="shared" si="7"/>
         <v>34</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="D38" s="12" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="E38" s="21">
         <v>1</v>
@@ -2243,7 +2249,7 @@
         <v>2</v>
       </c>
       <c r="H38" s="21">
-        <f>SUM(E38:G38)</f>
+        <f t="shared" si="6"/>
         <v>4</v>
       </c>
       <c r="I38" s="9">
@@ -2255,29 +2261,29 @@
       <c r="M38" s="1"/>
       <c r="N38" s="1"/>
     </row>
-    <row r="39" spans="2:14" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:14" ht="31.2" x14ac:dyDescent="0.3">
       <c r="B39" s="9">
-        <f>B38+1</f>
+        <f t="shared" si="7"/>
         <v>35</v>
       </c>
-      <c r="C39" s="4" t="s">
-        <v>3</v>
+      <c r="C39" s="5" t="s">
+        <v>40</v>
       </c>
       <c r="D39" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="E39" s="21">
+        <v>1</v>
+      </c>
+      <c r="F39" s="24">
+        <v>1</v>
+      </c>
+      <c r="G39" s="21">
+        <v>2</v>
+      </c>
+      <c r="H39" s="21">
+        <f t="shared" si="6"/>
         <v>4</v>
-      </c>
-      <c r="E39" s="21">
-        <v>1</v>
-      </c>
-      <c r="F39" s="24">
-        <v>1</v>
-      </c>
-      <c r="G39" s="21">
-        <v>1</v>
-      </c>
-      <c r="H39" s="21">
-        <f>SUM(E39:G39)</f>
-        <v>3</v>
       </c>
       <c r="I39" s="9">
         <v>0</v>
@@ -2288,15 +2294,17 @@
       <c r="M39" s="1"/>
       <c r="N39" s="1"/>
     </row>
-    <row r="40" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:14" ht="31.2" x14ac:dyDescent="0.3">
       <c r="B40" s="9">
-        <f>B39+1</f>
+        <f t="shared" si="7"/>
         <v>36</v>
       </c>
-      <c r="C40" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="D40" s="12"/>
+      <c r="C40" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="D40" s="12" t="s">
+        <v>4</v>
+      </c>
       <c r="E40" s="21">
         <v>1</v>
       </c>
@@ -2307,7 +2315,7 @@
         <v>1</v>
       </c>
       <c r="H40" s="21">
-        <f>SUM(E40:G40)</f>
+        <f t="shared" si="6"/>
         <v>3</v>
       </c>
       <c r="I40" s="9">
@@ -2319,29 +2327,29 @@
       <c r="M40" s="1"/>
       <c r="N40" s="1"/>
     </row>
-    <row r="41" spans="2:14" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="2:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B41" s="9">
-        <f>B40+1</f>
+        <f t="shared" si="7"/>
         <v>37</v>
       </c>
-      <c r="C41" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="D41" s="13"/>
-      <c r="E41" s="22">
-        <v>1</v>
-      </c>
-      <c r="F41" s="25">
-        <v>1</v>
-      </c>
-      <c r="G41" s="22">
-        <v>1</v>
-      </c>
-      <c r="H41" s="22">
-        <f>SUM(E41:G41)</f>
-        <v>3</v>
-      </c>
-      <c r="I41" s="28">
+      <c r="C41" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D41" s="12"/>
+      <c r="E41" s="21">
+        <v>1</v>
+      </c>
+      <c r="F41" s="24">
+        <v>1</v>
+      </c>
+      <c r="G41" s="21">
+        <v>1</v>
+      </c>
+      <c r="H41" s="21">
+        <f t="shared" si="6"/>
+        <v>3</v>
+      </c>
+      <c r="I41" s="9">
         <v>0</v>
       </c>
       <c r="J41" s="20"/>
@@ -2350,22 +2358,38 @@
       <c r="M41" s="1"/>
       <c r="N41" s="1"/>
     </row>
-    <row r="42" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="I42" s="10"/>
+    <row r="42" spans="2:14" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B42" s="9">
+        <f t="shared" si="7"/>
+        <v>38</v>
+      </c>
+      <c r="C42" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="D42" s="13"/>
+      <c r="E42" s="22">
+        <v>1</v>
+      </c>
+      <c r="F42" s="25">
+        <v>1</v>
+      </c>
+      <c r="G42" s="22">
+        <v>1</v>
+      </c>
+      <c r="H42" s="22">
+        <f t="shared" si="6"/>
+        <v>3</v>
+      </c>
+      <c r="I42" s="28">
+        <v>0</v>
+      </c>
       <c r="J42" s="20"/>
       <c r="K42" s="1"/>
       <c r="L42" s="1"/>
       <c r="M42" s="1"/>
       <c r="N42" s="1"/>
     </row>
-    <row r="43" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B43" s="10"/>
-      <c r="C43" s="26"/>
-      <c r="D43" s="27"/>
-      <c r="E43" s="20"/>
-      <c r="F43" s="20"/>
-      <c r="G43" s="20"/>
-      <c r="H43" s="20"/>
+    <row r="43" spans="2:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="I43" s="10"/>
       <c r="J43" s="20"/>
       <c r="K43" s="1"/>
@@ -2373,14 +2397,14 @@
       <c r="M43" s="1"/>
       <c r="N43" s="1"/>
     </row>
-    <row r="44" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B44" s="1"/>
-      <c r="C44" s="7"/>
-      <c r="D44" s="2"/>
-      <c r="E44" s="10"/>
-      <c r="F44" s="10"/>
-      <c r="G44" s="10"/>
-      <c r="H44" s="10"/>
+    <row r="44" spans="2:14" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B44" s="10"/>
+      <c r="C44" s="26"/>
+      <c r="D44" s="27"/>
+      <c r="E44" s="20"/>
+      <c r="F44" s="20"/>
+      <c r="G44" s="20"/>
+      <c r="H44" s="20"/>
       <c r="I44" s="10"/>
       <c r="J44" s="20"/>
       <c r="K44" s="1"/>
@@ -2388,7 +2412,7 @@
       <c r="M44" s="1"/>
       <c r="N44" s="1"/>
     </row>
-    <row r="45" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B45" s="1"/>
       <c r="C45" s="7"/>
       <c r="D45" s="2"/>
@@ -2403,7 +2427,7 @@
       <c r="M45" s="1"/>
       <c r="N45" s="1"/>
     </row>
-    <row r="46" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B46" s="1"/>
       <c r="C46" s="7"/>
       <c r="D46" s="2"/>
@@ -2418,7 +2442,7 @@
       <c r="M46" s="1"/>
       <c r="N46" s="1"/>
     </row>
-    <row r="47" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B47" s="1"/>
       <c r="C47" s="7"/>
       <c r="D47" s="2"/>
@@ -2433,7 +2457,7 @@
       <c r="M47" s="1"/>
       <c r="N47" s="1"/>
     </row>
-    <row r="48" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B48" s="1"/>
       <c r="C48" s="7"/>
       <c r="D48" s="2"/>
@@ -2448,7 +2472,7 @@
       <c r="M48" s="1"/>
       <c r="N48" s="1"/>
     </row>
-    <row r="49" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="49" spans="2:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B49" s="1"/>
       <c r="C49" s="7"/>
       <c r="D49" s="2"/>
@@ -2463,7 +2487,7 @@
       <c r="M49" s="1"/>
       <c r="N49" s="1"/>
     </row>
-    <row r="50" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="50" spans="2:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B50" s="1"/>
       <c r="C50" s="7"/>
       <c r="D50" s="2"/>
@@ -2478,7 +2502,7 @@
       <c r="M50" s="1"/>
       <c r="N50" s="1"/>
     </row>
-    <row r="51" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="51" spans="2:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B51" s="1"/>
       <c r="C51" s="7"/>
       <c r="D51" s="2"/>
@@ -2493,7 +2517,7 @@
       <c r="M51" s="1"/>
       <c r="N51" s="1"/>
     </row>
-    <row r="52" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="52" spans="2:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B52" s="1"/>
       <c r="C52" s="7"/>
       <c r="D52" s="2"/>
@@ -2508,7 +2532,7 @@
       <c r="M52" s="1"/>
       <c r="N52" s="1"/>
     </row>
-    <row r="53" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="53" spans="2:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B53" s="1"/>
       <c r="C53" s="7"/>
       <c r="D53" s="2"/>
@@ -2523,8 +2547,23 @@
       <c r="M53" s="1"/>
       <c r="N53" s="1"/>
     </row>
+    <row r="54" spans="2:14" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B54" s="1"/>
+      <c r="C54" s="7"/>
+      <c r="D54" s="2"/>
+      <c r="E54" s="10"/>
+      <c r="F54" s="10"/>
+      <c r="G54" s="10"/>
+      <c r="H54" s="10"/>
+      <c r="I54" s="10"/>
+      <c r="J54" s="20"/>
+      <c r="K54" s="1"/>
+      <c r="L54" s="1"/>
+      <c r="M54" s="1"/>
+      <c r="N54" s="1"/>
+    </row>
   </sheetData>
-  <autoFilter ref="B3:I41" xr:uid="{11BA4F79-2AB7-4A24-A4BE-758442E1F8CB}">
+  <autoFilter ref="B3:I42" xr:uid="{11BA4F79-2AB7-4A24-A4BE-758442E1F8CB}">
     <filterColumn colId="7">
       <filters>
         <filter val="0"/>
@@ -2534,16 +2573,16 @@
         <filter val="4"/>
       </filters>
     </filterColumn>
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B5:I41">
-      <sortCondition descending="1" ref="H4:H41"/>
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B5:I42">
+      <sortCondition descending="1" ref="H4:H42"/>
     </sortState>
   </autoFilter>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B5:J41">
-    <sortCondition descending="1" ref="H4:H41"/>
-    <sortCondition descending="1" ref="E4:E41"/>
-    <sortCondition descending="1" ref="F4:F41"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B5:J42">
+    <sortCondition descending="1" ref="H4:H42"/>
+    <sortCondition descending="1" ref="E4:E42"/>
+    <sortCondition descending="1" ref="F4:F42"/>
   </sortState>
-  <conditionalFormatting sqref="H4:H41">
+  <conditionalFormatting sqref="H4:H42">
     <cfRule type="colorScale" priority="3">
       <colorScale>
         <cfvo type="min"/>
@@ -2555,7 +2594,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I4:I41">
+  <conditionalFormatting sqref="I4:I42">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>

</xml_diff>

<commit_message>
Beautification and cleaned up attachment menus
</commit_message>
<xml_diff>
--- a/Future Features/New Features - Family Tree.xlsx
+++ b/Future Features/New Features - Family Tree.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://srcincgov1-my.sharepoint.us/personal/lauko_srcinc_com/Documents/Desktop/Personal/geneology/GED Keepers/Future Features/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="481" documentId="8_{D1FEEEA7-0E84-49B9-AD17-37D0BB95FB37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{97353DF2-41C5-4880-9545-0681CDEB6265}"/>
+  <xr:revisionPtr revIDLastSave="534" documentId="8_{D1FEEEA7-0E84-49B9-AD17-37D0BB95FB37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{90957F79-ADA8-4ACC-9952-E83B048C1BDD}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{8067922A-00B7-4646-9500-13902203F407}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$B$3:$I$42</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$B$3:$I$46</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="98">
   <si>
     <t>Feature</t>
   </si>
@@ -300,6 +300,39 @@
   </si>
   <si>
     <t>Add a trace function that shows the relationship between a selected individual and the "home" individual</t>
+  </si>
+  <si>
+    <t>Change attachment storage</t>
+  </si>
+  <si>
+    <t>create thumbnails at frontend instead of backend.  Simplify the backend to just accept files (pdf, jpg,mpg, etc…) and store them in the correct space.  Create a app.post for thumbnails and one for files, or maybe just one app.post that has both in the message.</t>
+  </si>
+  <si>
+    <t>done for images and pdfs, need to do it for movies</t>
+  </si>
+  <si>
+    <t>enhance attachments</t>
+  </si>
+  <si>
+    <t>Add a date stamp to each attachment that may help sort how the attachments are presented, earliest first…  or add arrows to allow attachments to be moved up or down the display list…  Maybe a checkbox to make the image visible  or not in the attachment panel?</t>
+  </si>
+  <si>
+    <t>give other the ability to edit existing tree nodes</t>
+  </si>
+  <si>
+    <t>others the ability to add additional nodes</t>
+  </si>
+  <si>
+    <t>will require coordination with other ancestry applications</t>
+  </si>
+  <si>
+    <t>will require flexible external storage</t>
+  </si>
+  <si>
+    <t>add parents and children</t>
+  </si>
+  <si>
+    <t>1.  change birth and death dates, add bio information, etc…</t>
   </si>
 </sst>
 </file>
@@ -723,6 +756,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1043,25 +1080,25 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{11BA4F79-2AB7-4A24-A4BE-758442E1F8CB}">
   <sheetPr filterMode="1"/>
-  <dimension ref="B1:N54"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="B1:N58"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="3" width="49.33203125" style="8" customWidth="1"/>
-    <col min="4" max="4" width="57.88671875" style="3" customWidth="1"/>
-    <col min="5" max="5" width="9.109375" style="11"/>
-    <col min="6" max="6" width="12.44140625" style="11" customWidth="1"/>
-    <col min="7" max="8" width="9.109375" style="11"/>
-    <col min="9" max="9" width="14.33203125" style="11" customWidth="1"/>
-    <col min="10" max="10" width="65.6640625" style="41" customWidth="1"/>
+    <col min="3" max="3" width="49.28515625" style="8" customWidth="1"/>
+    <col min="4" max="4" width="57.85546875" style="3" customWidth="1"/>
+    <col min="5" max="5" width="9.140625" style="11"/>
+    <col min="6" max="6" width="12.42578125" style="11" customWidth="1"/>
+    <col min="7" max="8" width="9.140625" style="11"/>
+    <col min="9" max="9" width="14.28515625" style="11" customWidth="1"/>
+    <col min="10" max="10" width="65.7109375" style="41" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="1" spans="2:14" x14ac:dyDescent="0.25">
       <c r="E1" s="19"/>
       <c r="F1" s="19"/>
       <c r="G1" s="19"/>
       <c r="H1" s="19"/>
     </row>
-    <row r="2" spans="2:14" ht="63" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:14" ht="63.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B2" s="10"/>
       <c r="C2" s="20"/>
       <c r="D2" s="20"/>
@@ -1082,7 +1119,7 @@
       <c r="M2" s="1"/>
       <c r="N2" s="1"/>
     </row>
-    <row r="3" spans="2:14" s="3" customFormat="1" ht="47.4" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:14" s="3" customFormat="1" ht="48" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="18"/>
       <c r="C3" s="15" t="s">
         <v>0</v>
@@ -1111,7 +1148,7 @@
       <c r="M3" s="2"/>
       <c r="N3" s="2"/>
     </row>
-    <row r="4" spans="2:14" ht="31.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:14" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="B4" s="14">
         <v>1</v>
       </c>
@@ -1143,9 +1180,9 @@
       <c r="M4" s="1"/>
       <c r="N4" s="1"/>
     </row>
-    <row r="5" spans="2:14" ht="31.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:14" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="B5" s="48">
-        <f t="shared" ref="B5:B16" si="1">B4+1</f>
+        <f t="shared" ref="B5:B7" si="1">B4+1</f>
         <v>2</v>
       </c>
       <c r="C5" s="44" t="s">
@@ -1162,7 +1199,7 @@
         <v>2</v>
       </c>
       <c r="H5" s="46">
-        <f t="shared" ref="H5:H19" si="2">SUM(E5:G5)</f>
+        <f t="shared" ref="H5:H7" si="2">SUM(E5:G5)</f>
         <v>8</v>
       </c>
       <c r="I5" s="48">
@@ -1174,7 +1211,7 @@
       <c r="M5" s="1"/>
       <c r="N5" s="1"/>
     </row>
-    <row r="6" spans="2:14" ht="46.8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:14" ht="47.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="B6" s="9">
         <f t="shared" si="1"/>
         <v>3</v>
@@ -1207,7 +1244,7 @@
       <c r="M6" s="1"/>
       <c r="N6" s="1"/>
     </row>
-    <row r="7" spans="2:14" ht="78" hidden="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:14" ht="78.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="B7" s="9">
         <f t="shared" si="1"/>
         <v>4</v>
@@ -1240,42 +1277,44 @@
       <c r="M7" s="1"/>
       <c r="N7" s="1"/>
     </row>
-    <row r="8" spans="2:14" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:14" ht="78.75" x14ac:dyDescent="0.25">
       <c r="B8" s="9">
-        <f t="shared" si="1"/>
+        <f t="shared" ref="B8:B31" si="3">B7+1</f>
         <v>5</v>
       </c>
-      <c r="C8" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="D8" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="E8" s="21">
-        <v>3</v>
-      </c>
-      <c r="F8" s="24">
-        <v>2</v>
-      </c>
-      <c r="G8" s="21">
+      <c r="C8" s="35" t="s">
+        <v>87</v>
+      </c>
+      <c r="D8" s="35" t="s">
+        <v>88</v>
+      </c>
+      <c r="E8" s="42">
+        <v>3</v>
+      </c>
+      <c r="F8" s="43">
+        <v>3</v>
+      </c>
+      <c r="G8" s="42">
         <v>2</v>
       </c>
       <c r="H8" s="21">
-        <f t="shared" si="2"/>
-        <v>7</v>
+        <f t="shared" ref="H8:H46" si="4">SUM(E8:G8)</f>
+        <v>8</v>
       </c>
       <c r="I8" s="9">
-        <v>1</v>
-      </c>
-      <c r="J8" s="20"/>
+        <v>4</v>
+      </c>
+      <c r="J8" s="41" t="s">
+        <v>89</v>
+      </c>
       <c r="K8" s="1"/>
       <c r="L8" s="1"/>
       <c r="M8" s="1"/>
       <c r="N8" s="1"/>
     </row>
-    <row r="9" spans="2:14" ht="46.8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:14" ht="47.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="B9" s="9">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>6</v>
       </c>
       <c r="C9" s="44" t="s">
@@ -1294,7 +1333,7 @@
         <v>3</v>
       </c>
       <c r="H9" s="46">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>9</v>
       </c>
       <c r="I9" s="48">
@@ -1305,9 +1344,9 @@
       <c r="M9" s="1"/>
       <c r="N9" s="1"/>
     </row>
-    <row r="10" spans="2:14" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:14" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="B10" s="48">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>7</v>
       </c>
       <c r="C10" s="44" t="s">
@@ -1326,7 +1365,7 @@
         <v>3</v>
       </c>
       <c r="H10" s="46">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>8</v>
       </c>
       <c r="I10" s="48">
@@ -1337,9 +1376,9 @@
       <c r="M10" s="1"/>
       <c r="N10" s="1"/>
     </row>
-    <row r="11" spans="2:14" ht="46.8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:14" ht="47.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="B11" s="48">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>8</v>
       </c>
       <c r="C11" s="44" t="s">
@@ -1358,7 +1397,7 @@
         <v>2</v>
       </c>
       <c r="H11" s="46">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>7</v>
       </c>
       <c r="I11" s="48">
@@ -1369,9 +1408,9 @@
       <c r="M11" s="1"/>
       <c r="N11" s="1"/>
     </row>
-    <row r="12" spans="2:14" ht="31.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:14" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="B12" s="48">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>9</v>
       </c>
       <c r="C12" s="49" t="s">
@@ -1388,7 +1427,7 @@
         <v>3</v>
       </c>
       <c r="H12" s="46">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>7</v>
       </c>
       <c r="I12" s="48">
@@ -1402,9 +1441,9 @@
       <c r="M12" s="1"/>
       <c r="N12" s="1"/>
     </row>
-    <row r="13" spans="2:14" ht="62.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:14" ht="63" hidden="1" x14ac:dyDescent="0.25">
       <c r="B13" s="9">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>10</v>
       </c>
       <c r="C13" s="30" t="s">
@@ -1423,7 +1462,7 @@
         <v>2</v>
       </c>
       <c r="H13" s="32">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>6</v>
       </c>
       <c r="I13" s="34">
@@ -1435,51 +1474,49 @@
       <c r="M13" s="1"/>
       <c r="N13" s="1"/>
     </row>
-    <row r="14" spans="2:14" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:14" ht="31.5" x14ac:dyDescent="0.25">
       <c r="B14" s="9">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>11</v>
       </c>
-      <c r="C14" s="35" t="s">
-        <v>52</v>
-      </c>
-      <c r="D14" s="35" t="s">
-        <v>53</v>
-      </c>
-      <c r="E14" s="42">
-        <v>3</v>
-      </c>
-      <c r="F14" s="43">
-        <v>2</v>
-      </c>
-      <c r="G14" s="42">
+      <c r="C14" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="D14" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="E14" s="21">
+        <v>3</v>
+      </c>
+      <c r="F14" s="24">
+        <v>2</v>
+      </c>
+      <c r="G14" s="21">
         <v>2</v>
       </c>
       <c r="H14" s="21">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>7</v>
       </c>
       <c r="I14" s="9">
-        <v>4</v>
-      </c>
-      <c r="J14" s="41" t="s">
-        <v>65</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="J14" s="20"/>
       <c r="K14" s="1"/>
       <c r="L14" s="1"/>
       <c r="M14" s="1"/>
       <c r="N14" s="1"/>
     </row>
-    <row r="15" spans="2:14" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:14" ht="78.75" x14ac:dyDescent="0.25">
       <c r="B15" s="9">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>12</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>67</v>
+        <v>90</v>
       </c>
       <c r="D15" s="12" t="s">
-        <v>68</v>
+        <v>91</v>
       </c>
       <c r="E15" s="21">
         <v>3</v>
@@ -1491,7 +1528,7 @@
         <v>2</v>
       </c>
       <c r="H15" s="21">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>7</v>
       </c>
       <c r="I15" s="9">
@@ -1503,349 +1540,355 @@
       <c r="M15" s="1"/>
       <c r="N15" s="1"/>
     </row>
-    <row r="16" spans="2:14" ht="31.2" hidden="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="48">
-        <f t="shared" si="1"/>
+    <row r="16" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B16" s="9">
+        <f t="shared" si="3"/>
         <v>13</v>
       </c>
-      <c r="C16" s="44" t="s">
-        <v>9</v>
-      </c>
-      <c r="D16" s="50" t="s">
-        <v>10</v>
-      </c>
-      <c r="E16" s="46">
-        <v>3</v>
-      </c>
-      <c r="F16" s="47">
-        <v>2</v>
-      </c>
-      <c r="G16" s="46">
-        <v>2</v>
-      </c>
-      <c r="H16" s="46">
-        <f t="shared" si="2"/>
+      <c r="C16" s="35" t="s">
+        <v>52</v>
+      </c>
+      <c r="D16" s="35" t="s">
+        <v>53</v>
+      </c>
+      <c r="E16" s="42">
+        <v>3</v>
+      </c>
+      <c r="F16" s="43">
+        <v>2</v>
+      </c>
+      <c r="G16" s="42">
+        <v>2</v>
+      </c>
+      <c r="H16" s="21">
+        <f t="shared" si="4"/>
         <v>7</v>
       </c>
-      <c r="I16" s="48">
-        <v>5</v>
+      <c r="I16" s="9">
+        <v>4</v>
+      </c>
+      <c r="J16" s="41" t="s">
+        <v>65</v>
       </c>
       <c r="K16" s="1"/>
       <c r="L16" s="1"/>
       <c r="M16" s="1"/>
       <c r="N16" s="1"/>
     </row>
-    <row r="17" spans="2:14" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B17" s="9">
-        <f t="shared" ref="B17:B21" si="3">B16+1</f>
+        <f t="shared" si="3"/>
         <v>14</v>
       </c>
-      <c r="C17" s="56" t="s">
-        <v>81</v>
-      </c>
-      <c r="D17" s="51" t="s">
-        <v>82</v>
-      </c>
-      <c r="E17" s="52">
-        <v>2</v>
-      </c>
-      <c r="F17" s="53">
-        <v>2</v>
-      </c>
-      <c r="G17" s="52">
-        <v>3</v>
-      </c>
-      <c r="H17" s="52">
-        <f t="shared" si="2"/>
+      <c r="C17" s="35" t="s">
+        <v>93</v>
+      </c>
+      <c r="D17" s="35" t="s">
+        <v>96</v>
+      </c>
+      <c r="E17" s="42">
+        <v>3</v>
+      </c>
+      <c r="F17" s="43">
+        <v>2</v>
+      </c>
+      <c r="G17" s="42">
+        <v>2</v>
+      </c>
+      <c r="H17" s="21">
+        <f t="shared" si="4"/>
         <v>7</v>
       </c>
-      <c r="I17" s="58">
+      <c r="I17" s="9">
         <v>0</v>
       </c>
-      <c r="J17" s="57"/>
+      <c r="J17" s="41" t="s">
+        <v>94</v>
+      </c>
       <c r="K17" s="1"/>
       <c r="L17" s="1"/>
       <c r="M17" s="1"/>
       <c r="N17" s="1"/>
     </row>
-    <row r="18" spans="2:14" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:14" ht="31.5" x14ac:dyDescent="0.25">
       <c r="B18" s="9">
         <f t="shared" si="3"/>
         <v>15</v>
       </c>
-      <c r="C18" s="56" t="s">
-        <v>85</v>
-      </c>
-      <c r="D18" s="51" t="s">
-        <v>86</v>
-      </c>
-      <c r="E18" s="52">
-        <v>2</v>
-      </c>
-      <c r="F18" s="53">
-        <v>2</v>
-      </c>
-      <c r="G18" s="52">
-        <v>2</v>
-      </c>
-      <c r="H18" s="52">
-        <f t="shared" si="2"/>
-        <v>6</v>
-      </c>
-      <c r="I18" s="58">
-        <v>0</v>
-      </c>
-      <c r="J18" s="57"/>
+      <c r="C18" s="35" t="s">
+        <v>92</v>
+      </c>
+      <c r="D18" s="35" t="s">
+        <v>97</v>
+      </c>
+      <c r="E18" s="42">
+        <v>3</v>
+      </c>
+      <c r="F18" s="43">
+        <v>2</v>
+      </c>
+      <c r="G18" s="42">
+        <v>2</v>
+      </c>
+      <c r="H18" s="21">
+        <f t="shared" si="4"/>
+        <v>7</v>
+      </c>
+      <c r="I18" s="9">
+        <v>2</v>
+      </c>
+      <c r="J18" s="41" t="s">
+        <v>95</v>
+      </c>
       <c r="K18" s="1"/>
       <c r="L18" s="1"/>
       <c r="M18" s="1"/>
       <c r="N18" s="1"/>
     </row>
-    <row r="19" spans="2:14" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B19" s="9">
         <f t="shared" si="3"/>
         <v>16</v>
       </c>
-      <c r="C19" s="35" t="s">
-        <v>66</v>
-      </c>
-      <c r="D19" s="35" t="s">
-        <v>69</v>
-      </c>
-      <c r="E19" s="42">
-        <v>2</v>
-      </c>
-      <c r="F19" s="43">
-        <v>2</v>
-      </c>
-      <c r="G19" s="42">
-        <v>3</v>
+      <c r="C19" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="D19" s="12" t="s">
+        <v>68</v>
+      </c>
+      <c r="E19" s="21">
+        <v>3</v>
+      </c>
+      <c r="F19" s="24">
+        <v>2</v>
+      </c>
+      <c r="G19" s="21">
+        <v>2</v>
       </c>
       <c r="H19" s="21">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>7</v>
       </c>
       <c r="I19" s="9">
-        <v>3</v>
-      </c>
-      <c r="J19" s="20" t="s">
-        <v>70</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="J19" s="20"/>
       <c r="K19" s="1"/>
       <c r="L19" s="1"/>
       <c r="M19" s="1"/>
       <c r="N19" s="1"/>
     </row>
-    <row r="20" spans="2:14" ht="31.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:14" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="B20" s="48">
         <f t="shared" si="3"/>
         <v>17</v>
       </c>
-      <c r="C20" s="49" t="s">
-        <v>83</v>
-      </c>
-      <c r="D20" s="49" t="s">
-        <v>84</v>
-      </c>
-      <c r="E20" s="59">
-        <v>3</v>
-      </c>
-      <c r="F20" s="60">
-        <v>2</v>
-      </c>
-      <c r="G20" s="59">
-        <v>3</v>
+      <c r="C20" s="44" t="s">
+        <v>9</v>
+      </c>
+      <c r="D20" s="50" t="s">
+        <v>10</v>
+      </c>
+      <c r="E20" s="46">
+        <v>3</v>
+      </c>
+      <c r="F20" s="47">
+        <v>2</v>
+      </c>
+      <c r="G20" s="46">
+        <v>2</v>
       </c>
       <c r="H20" s="46">
-        <f t="shared" ref="H20:H21" si="4">SUM(E20:G20)</f>
-        <v>8</v>
+        <f t="shared" si="4"/>
+        <v>7</v>
       </c>
       <c r="I20" s="48">
         <v>5</v>
       </c>
-      <c r="J20" s="61"/>
       <c r="K20" s="1"/>
       <c r="L20" s="1"/>
       <c r="M20" s="1"/>
       <c r="N20" s="1"/>
     </row>
-    <row r="21" spans="2:14" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:14" ht="31.5" x14ac:dyDescent="0.25">
       <c r="B21" s="9">
         <f t="shared" si="3"/>
         <v>18</v>
       </c>
-      <c r="C21" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="D21" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="E21" s="21">
-        <v>2</v>
-      </c>
-      <c r="F21" s="24">
-        <v>2</v>
-      </c>
-      <c r="G21" s="21">
-        <v>2</v>
-      </c>
-      <c r="H21" s="21">
-        <f t="shared" si="4"/>
-        <v>6</v>
-      </c>
-      <c r="I21" s="9">
-        <v>2</v>
-      </c>
-      <c r="J21" s="20" t="s">
-        <v>63</v>
-      </c>
+      <c r="C21" s="56" t="s">
+        <v>81</v>
+      </c>
+      <c r="D21" s="51" t="s">
+        <v>82</v>
+      </c>
+      <c r="E21" s="52">
+        <v>2</v>
+      </c>
+      <c r="F21" s="53">
+        <v>2</v>
+      </c>
+      <c r="G21" s="52">
+        <v>3</v>
+      </c>
+      <c r="H21" s="52">
+        <f t="shared" si="4"/>
+        <v>7</v>
+      </c>
+      <c r="I21" s="58">
+        <v>0</v>
+      </c>
+      <c r="J21" s="57"/>
       <c r="K21" s="1"/>
       <c r="L21" s="1"/>
       <c r="M21" s="1"/>
       <c r="N21" s="1"/>
     </row>
-    <row r="22" spans="2:14" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:14" ht="31.5" x14ac:dyDescent="0.25">
       <c r="B22" s="9">
-        <f t="shared" ref="B22:B29" si="5">B21+1</f>
+        <f t="shared" si="3"/>
         <v>19</v>
       </c>
-      <c r="C22" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="D22" s="23" t="s">
-        <v>21</v>
-      </c>
-      <c r="E22" s="21">
-        <v>2</v>
-      </c>
-      <c r="F22" s="24">
-        <v>2</v>
-      </c>
-      <c r="G22" s="21">
-        <v>2</v>
+      <c r="C22" s="35" t="s">
+        <v>66</v>
+      </c>
+      <c r="D22" s="35" t="s">
+        <v>69</v>
+      </c>
+      <c r="E22" s="42">
+        <v>2</v>
+      </c>
+      <c r="F22" s="43">
+        <v>2</v>
+      </c>
+      <c r="G22" s="42">
+        <v>3</v>
       </c>
       <c r="H22" s="21">
-        <f t="shared" ref="H22:H42" si="6">SUM(E22:G22)</f>
-        <v>6</v>
+        <f t="shared" si="4"/>
+        <v>7</v>
       </c>
       <c r="I22" s="9">
-        <v>0</v>
-      </c>
-      <c r="J22" s="20"/>
+        <v>3</v>
+      </c>
+      <c r="J22" s="20" t="s">
+        <v>70</v>
+      </c>
       <c r="K22" s="1"/>
       <c r="L22" s="1"/>
       <c r="M22" s="1"/>
       <c r="N22" s="1"/>
     </row>
-    <row r="23" spans="2:14" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:14" ht="31.5" x14ac:dyDescent="0.25">
       <c r="B23" s="9">
-        <f t="shared" si="5"/>
+        <f t="shared" si="3"/>
         <v>20</v>
       </c>
-      <c r="C23" s="5" t="s">
-        <v>79</v>
-      </c>
-      <c r="D23" s="23" t="s">
-        <v>80</v>
-      </c>
-      <c r="E23" s="21">
-        <v>1</v>
-      </c>
-      <c r="F23" s="24">
-        <v>2</v>
-      </c>
-      <c r="G23" s="21">
-        <v>1</v>
-      </c>
-      <c r="H23" s="21">
-        <f t="shared" si="6"/>
-        <v>4</v>
-      </c>
-      <c r="I23" s="9">
+      <c r="C23" s="56" t="s">
+        <v>85</v>
+      </c>
+      <c r="D23" s="51" t="s">
+        <v>86</v>
+      </c>
+      <c r="E23" s="52">
+        <v>2</v>
+      </c>
+      <c r="F23" s="53">
+        <v>2</v>
+      </c>
+      <c r="G23" s="52">
+        <v>2</v>
+      </c>
+      <c r="H23" s="52">
+        <f t="shared" si="4"/>
+        <v>6</v>
+      </c>
+      <c r="I23" s="58">
         <v>0</v>
       </c>
-      <c r="J23" s="20"/>
+      <c r="J23" s="57"/>
       <c r="K23" s="1"/>
       <c r="L23" s="1"/>
       <c r="M23" s="1"/>
       <c r="N23" s="1"/>
     </row>
-    <row r="24" spans="2:14" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="B24" s="9">
-        <f t="shared" si="5"/>
+    <row r="24" spans="2:14" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B24" s="48">
+        <f t="shared" si="3"/>
         <v>21</v>
       </c>
-      <c r="C24" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="D24" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="E24" s="21">
-        <v>2</v>
-      </c>
-      <c r="F24" s="24">
-        <v>2</v>
-      </c>
-      <c r="G24" s="21">
-        <v>2</v>
-      </c>
-      <c r="H24" s="21">
-        <f t="shared" si="6"/>
-        <v>6</v>
-      </c>
-      <c r="I24" s="9">
-        <v>0</v>
-      </c>
-      <c r="J24" s="20"/>
+      <c r="C24" s="49" t="s">
+        <v>83</v>
+      </c>
+      <c r="D24" s="49" t="s">
+        <v>84</v>
+      </c>
+      <c r="E24" s="59">
+        <v>3</v>
+      </c>
+      <c r="F24" s="60">
+        <v>2</v>
+      </c>
+      <c r="G24" s="59">
+        <v>3</v>
+      </c>
+      <c r="H24" s="46">
+        <f t="shared" si="4"/>
+        <v>8</v>
+      </c>
+      <c r="I24" s="48">
+        <v>5</v>
+      </c>
+      <c r="J24" s="61"/>
       <c r="K24" s="1"/>
       <c r="L24" s="1"/>
       <c r="M24" s="1"/>
       <c r="N24" s="1"/>
     </row>
-    <row r="25" spans="2:14" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
-      <c r="B25" s="48">
-        <f t="shared" si="5"/>
+    <row r="25" spans="2:14" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="B25" s="9">
+        <f t="shared" si="3"/>
         <v>22</v>
       </c>
-      <c r="C25" s="44" t="s">
-        <v>39</v>
-      </c>
-      <c r="D25" s="50" t="s">
-        <v>71</v>
-      </c>
-      <c r="E25" s="46">
-        <v>1</v>
-      </c>
-      <c r="F25" s="47">
-        <v>2</v>
-      </c>
-      <c r="G25" s="46">
-        <v>3</v>
-      </c>
-      <c r="H25" s="46">
-        <f t="shared" si="6"/>
+      <c r="C25" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D25" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E25" s="21">
+        <v>2</v>
+      </c>
+      <c r="F25" s="24">
+        <v>2</v>
+      </c>
+      <c r="G25" s="21">
+        <v>2</v>
+      </c>
+      <c r="H25" s="21">
+        <f t="shared" si="4"/>
         <v>6</v>
       </c>
-      <c r="I25" s="48">
-        <v>5</v>
-      </c>
-      <c r="J25" s="20"/>
+      <c r="I25" s="9">
+        <v>2</v>
+      </c>
+      <c r="J25" s="20" t="s">
+        <v>63</v>
+      </c>
       <c r="K25" s="1"/>
       <c r="L25" s="1"/>
       <c r="M25" s="1"/>
       <c r="N25" s="1"/>
     </row>
-    <row r="26" spans="2:14" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:14" ht="31.5" x14ac:dyDescent="0.25">
       <c r="B26" s="9">
-        <f t="shared" si="5"/>
+        <f t="shared" si="3"/>
         <v>23</v>
       </c>
-      <c r="C26" s="23" t="s">
-        <v>22</v>
+      <c r="C26" s="5" t="s">
+        <v>20</v>
       </c>
       <c r="D26" s="23" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="E26" s="21">
         <v>2</v>
@@ -1854,11 +1897,11 @@
         <v>2</v>
       </c>
       <c r="G26" s="21">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H26" s="21">
-        <f t="shared" si="6"/>
-        <v>5</v>
+        <f t="shared" si="4"/>
+        <v>6</v>
       </c>
       <c r="I26" s="9">
         <v>0</v>
@@ -1869,19 +1912,19 @@
       <c r="M26" s="1"/>
       <c r="N26" s="1"/>
     </row>
-    <row r="27" spans="2:14" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:14" ht="47.25" x14ac:dyDescent="0.25">
       <c r="B27" s="9">
-        <f t="shared" si="5"/>
+        <f t="shared" si="3"/>
         <v>24</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="D27" s="23" t="s">
-        <v>57</v>
+        <v>36</v>
+      </c>
+      <c r="D27" s="5" t="s">
+        <v>48</v>
       </c>
       <c r="E27" s="21">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F27" s="24">
         <v>2</v>
@@ -1890,8 +1933,8 @@
         <v>2</v>
       </c>
       <c r="H27" s="21">
-        <f t="shared" si="6"/>
-        <v>5</v>
+        <f t="shared" si="4"/>
+        <v>6</v>
       </c>
       <c r="I27" s="9">
         <v>0</v>
@@ -1902,63 +1945,64 @@
       <c r="M27" s="1"/>
       <c r="N27" s="1"/>
     </row>
-    <row r="28" spans="2:14" ht="83.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:14" ht="47.25" x14ac:dyDescent="0.25">
       <c r="B28" s="9">
-        <f t="shared" si="5"/>
+        <f t="shared" si="3"/>
         <v>25</v>
       </c>
-      <c r="C28" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="D28" s="12" t="s">
-        <v>35</v>
+      <c r="C28" s="23" t="s">
+        <v>22</v>
+      </c>
+      <c r="D28" s="23" t="s">
+        <v>23</v>
       </c>
       <c r="E28" s="21">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F28" s="24">
         <v>2</v>
       </c>
       <c r="G28" s="21">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H28" s="21">
-        <f t="shared" si="6"/>
+        <f t="shared" si="4"/>
         <v>5</v>
       </c>
       <c r="I28" s="9">
         <v>0</v>
       </c>
+      <c r="J28" s="20"/>
       <c r="K28" s="1"/>
       <c r="L28" s="1"/>
       <c r="M28" s="1"/>
       <c r="N28" s="1"/>
     </row>
-    <row r="29" spans="2:14" ht="83.25" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B29" s="29">
-        <f t="shared" si="5"/>
+    <row r="29" spans="2:14" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B29" s="48">
+        <f t="shared" si="3"/>
         <v>26</v>
       </c>
-      <c r="C29" s="30" t="s">
-        <v>31</v>
-      </c>
-      <c r="D29" s="31" t="s">
-        <v>32</v>
-      </c>
-      <c r="E29" s="32">
-        <v>2</v>
-      </c>
-      <c r="F29" s="33">
-        <v>1</v>
-      </c>
-      <c r="G29" s="32">
-        <v>3</v>
-      </c>
-      <c r="H29" s="32">
-        <f t="shared" si="6"/>
+      <c r="C29" s="44" t="s">
+        <v>39</v>
+      </c>
+      <c r="D29" s="50" t="s">
+        <v>71</v>
+      </c>
+      <c r="E29" s="46">
+        <v>1</v>
+      </c>
+      <c r="F29" s="47">
+        <v>2</v>
+      </c>
+      <c r="G29" s="46">
+        <v>3</v>
+      </c>
+      <c r="H29" s="46">
+        <f t="shared" si="4"/>
         <v>6</v>
       </c>
-      <c r="I29" s="34">
+      <c r="I29" s="48">
         <v>5</v>
       </c>
       <c r="J29" s="20"/>
@@ -1967,26 +2011,28 @@
       <c r="M29" s="1"/>
       <c r="N29" s="1"/>
     </row>
-    <row r="30" spans="2:14" ht="83.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:14" ht="31.5" x14ac:dyDescent="0.25">
       <c r="B30" s="9">
-        <f>B28+1</f>
-        <v>26</v>
-      </c>
-      <c r="C30" s="35" t="s">
-        <v>64</v>
-      </c>
-      <c r="D30" s="51"/>
-      <c r="E30" s="52">
-        <v>1</v>
-      </c>
-      <c r="F30" s="53">
-        <v>1</v>
-      </c>
-      <c r="G30" s="52">
-        <v>3</v>
-      </c>
-      <c r="H30" s="52">
-        <f t="shared" si="6"/>
+        <f t="shared" si="3"/>
+        <v>27</v>
+      </c>
+      <c r="C30" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="D30" s="23" t="s">
+        <v>57</v>
+      </c>
+      <c r="E30" s="21">
+        <v>1</v>
+      </c>
+      <c r="F30" s="24">
+        <v>2</v>
+      </c>
+      <c r="G30" s="21">
+        <v>2</v>
+      </c>
+      <c r="H30" s="21">
+        <f t="shared" si="4"/>
         <v>5</v>
       </c>
       <c r="I30" s="9">
@@ -1998,63 +2044,62 @@
       <c r="M30" s="1"/>
       <c r="N30" s="1"/>
     </row>
-    <row r="31" spans="2:14" ht="83.25" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B31" s="34">
-        <f t="shared" ref="B31:B42" si="7">B30+1</f>
-        <v>27</v>
-      </c>
-      <c r="C31" s="54" t="s">
-        <v>62</v>
-      </c>
-      <c r="D31" s="55" t="s">
-        <v>61</v>
-      </c>
-      <c r="E31" s="32">
-        <v>2</v>
-      </c>
-      <c r="F31" s="33">
-        <v>2</v>
-      </c>
-      <c r="G31" s="32">
-        <v>2</v>
-      </c>
-      <c r="H31" s="32">
-        <f t="shared" si="6"/>
-        <v>6</v>
-      </c>
-      <c r="I31" s="34">
+    <row r="31" spans="2:14" ht="78.75" x14ac:dyDescent="0.25">
+      <c r="B31" s="9">
+        <f t="shared" si="3"/>
+        <v>28</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="D31" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="E31" s="21">
+        <v>1</v>
+      </c>
+      <c r="F31" s="24">
+        <v>2</v>
+      </c>
+      <c r="G31" s="21">
+        <v>2</v>
+      </c>
+      <c r="H31" s="21">
+        <f t="shared" si="4"/>
         <v>5</v>
       </c>
-      <c r="J31" s="20"/>
+      <c r="I31" s="9">
+        <v>0</v>
+      </c>
       <c r="K31" s="1"/>
       <c r="L31" s="1"/>
       <c r="M31" s="1"/>
       <c r="N31" s="1"/>
     </row>
-    <row r="32" spans="2:14" ht="31.2" hidden="1" x14ac:dyDescent="0.3">
-      <c r="B32" s="48">
-        <f t="shared" si="7"/>
+    <row r="32" spans="2:14" ht="83.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B32" s="9">
+        <f>B30+1</f>
         <v>28</v>
       </c>
-      <c r="C32" s="49" t="s">
-        <v>59</v>
-      </c>
-      <c r="D32" s="50"/>
-      <c r="E32" s="46">
-        <v>1</v>
-      </c>
-      <c r="F32" s="47">
-        <v>1</v>
-      </c>
-      <c r="G32" s="46">
-        <v>3</v>
-      </c>
-      <c r="H32" s="46">
-        <f t="shared" si="6"/>
+      <c r="C32" s="35" t="s">
+        <v>64</v>
+      </c>
+      <c r="D32" s="51"/>
+      <c r="E32" s="52">
+        <v>1</v>
+      </c>
+      <c r="F32" s="53">
+        <v>1</v>
+      </c>
+      <c r="G32" s="52">
+        <v>3</v>
+      </c>
+      <c r="H32" s="52">
+        <f t="shared" si="4"/>
         <v>5</v>
       </c>
-      <c r="I32" s="48">
-        <v>5</v>
+      <c r="I32" s="9">
+        <v>0</v>
       </c>
       <c r="J32" s="20"/>
       <c r="K32" s="1"/>
@@ -2062,32 +2107,32 @@
       <c r="M32" s="1"/>
       <c r="N32" s="1"/>
     </row>
-    <row r="33" spans="2:14" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="B33" s="9">
-        <f t="shared" si="7"/>
+    <row r="33" spans="2:14" ht="83.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B33" s="29">
+        <f t="shared" ref="B33:B46" si="5">B32+1</f>
         <v>29</v>
       </c>
-      <c r="C33" s="26" t="s">
-        <v>42</v>
-      </c>
-      <c r="D33" s="12" t="s">
-        <v>43</v>
-      </c>
-      <c r="E33" s="21">
-        <v>2</v>
-      </c>
-      <c r="F33" s="24">
-        <v>1</v>
-      </c>
-      <c r="G33" s="21">
-        <v>1</v>
-      </c>
-      <c r="H33" s="21">
-        <f t="shared" si="6"/>
-        <v>4</v>
-      </c>
-      <c r="I33" s="9">
-        <v>0</v>
+      <c r="C33" s="30" t="s">
+        <v>31</v>
+      </c>
+      <c r="D33" s="31" t="s">
+        <v>32</v>
+      </c>
+      <c r="E33" s="32">
+        <v>2</v>
+      </c>
+      <c r="F33" s="33">
+        <v>1</v>
+      </c>
+      <c r="G33" s="32">
+        <v>3</v>
+      </c>
+      <c r="H33" s="32">
+        <f t="shared" si="4"/>
+        <v>6</v>
+      </c>
+      <c r="I33" s="34">
+        <v>5</v>
       </c>
       <c r="J33" s="20"/>
       <c r="K33" s="1"/>
@@ -2095,63 +2140,64 @@
       <c r="M33" s="1"/>
       <c r="N33" s="1"/>
     </row>
-    <row r="34" spans="2:14" ht="31.2" hidden="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="48">
-        <f t="shared" si="7"/>
+    <row r="34" spans="2:14" ht="83.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B34" s="9">
+        <f t="shared" si="5"/>
         <v>30</v>
       </c>
-      <c r="C34" s="49" t="s">
-        <v>5</v>
-      </c>
-      <c r="D34" s="50" t="s">
-        <v>6</v>
-      </c>
-      <c r="E34" s="46">
-        <v>1</v>
-      </c>
-      <c r="F34" s="47">
-        <v>1</v>
-      </c>
-      <c r="G34" s="46">
-        <v>2</v>
-      </c>
-      <c r="H34" s="46">
-        <f t="shared" si="6"/>
+      <c r="C34" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="D34" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="E34" s="21">
+        <v>2</v>
+      </c>
+      <c r="F34" s="24">
+        <v>1</v>
+      </c>
+      <c r="G34" s="21">
+        <v>1</v>
+      </c>
+      <c r="H34" s="21">
+        <f t="shared" si="4"/>
         <v>4</v>
       </c>
-      <c r="I34" s="48">
-        <v>5</v>
-      </c>
+      <c r="I34" s="9">
+        <v>0</v>
+      </c>
+      <c r="J34" s="20"/>
       <c r="K34" s="1"/>
       <c r="L34" s="1"/>
       <c r="M34" s="1"/>
       <c r="N34" s="1"/>
     </row>
-    <row r="35" spans="2:14" ht="31.2" hidden="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="48">
-        <f t="shared" si="7"/>
+    <row r="35" spans="2:14" ht="83.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B35" s="34">
+        <f t="shared" si="5"/>
         <v>31</v>
       </c>
-      <c r="C35" s="44" t="s">
-        <v>44</v>
-      </c>
-      <c r="D35" s="50" t="s">
-        <v>45</v>
-      </c>
-      <c r="E35" s="46">
-        <v>2</v>
-      </c>
-      <c r="F35" s="47">
-        <v>1</v>
-      </c>
-      <c r="G35" s="46">
-        <v>1</v>
-      </c>
-      <c r="H35" s="46">
-        <f t="shared" si="6"/>
-        <v>4</v>
-      </c>
-      <c r="I35" s="48">
+      <c r="C35" s="54" t="s">
+        <v>62</v>
+      </c>
+      <c r="D35" s="55" t="s">
+        <v>61</v>
+      </c>
+      <c r="E35" s="32">
+        <v>2</v>
+      </c>
+      <c r="F35" s="33">
+        <v>2</v>
+      </c>
+      <c r="G35" s="32">
+        <v>2</v>
+      </c>
+      <c r="H35" s="32">
+        <f t="shared" si="4"/>
+        <v>6</v>
+      </c>
+      <c r="I35" s="34">
         <v>5</v>
       </c>
       <c r="J35" s="20"/>
@@ -2160,17 +2206,15 @@
       <c r="M35" s="1"/>
       <c r="N35" s="1"/>
     </row>
-    <row r="36" spans="2:14" ht="78" hidden="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:14" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="B36" s="48">
-        <f t="shared" si="7"/>
+        <f t="shared" si="5"/>
         <v>32</v>
       </c>
       <c r="C36" s="49" t="s">
-        <v>33</v>
-      </c>
-      <c r="D36" s="50" t="s">
-        <v>34</v>
-      </c>
+        <v>59</v>
+      </c>
+      <c r="D36" s="50"/>
       <c r="E36" s="46">
         <v>1</v>
       </c>
@@ -2178,45 +2222,43 @@
         <v>1</v>
       </c>
       <c r="G36" s="46">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H36" s="46">
-        <f t="shared" si="6"/>
-        <v>4</v>
+        <f t="shared" si="4"/>
+        <v>5</v>
       </c>
       <c r="I36" s="48">
         <v>5</v>
       </c>
-      <c r="J36" s="20" t="s">
-        <v>51</v>
-      </c>
+      <c r="J36" s="20"/>
       <c r="K36" s="1"/>
       <c r="L36" s="1"/>
       <c r="M36" s="1"/>
       <c r="N36" s="1"/>
     </row>
-    <row r="37" spans="2:14" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:14" ht="31.5" x14ac:dyDescent="0.25">
       <c r="B37" s="9">
-        <f t="shared" si="7"/>
+        <f t="shared" si="5"/>
         <v>33</v>
       </c>
-      <c r="C37" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="D37" s="12" t="s">
-        <v>8</v>
+      <c r="C37" s="26" t="s">
+        <v>79</v>
+      </c>
+      <c r="D37" s="23" t="s">
+        <v>80</v>
       </c>
       <c r="E37" s="21">
         <v>1</v>
       </c>
       <c r="F37" s="24">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G37" s="21">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H37" s="21">
-        <f t="shared" si="6"/>
+        <f t="shared" si="4"/>
         <v>4</v>
       </c>
       <c r="I37" s="9">
@@ -2228,65 +2270,64 @@
       <c r="M37" s="1"/>
       <c r="N37" s="1"/>
     </row>
-    <row r="38" spans="2:14" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="B38" s="9">
-        <f t="shared" si="7"/>
+    <row r="38" spans="2:14" ht="47.25" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B38" s="48">
+        <f t="shared" si="5"/>
         <v>34</v>
       </c>
-      <c r="C38" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="D38" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="E38" s="21">
-        <v>1</v>
-      </c>
-      <c r="F38" s="24">
-        <v>1</v>
-      </c>
-      <c r="G38" s="21">
-        <v>2</v>
-      </c>
-      <c r="H38" s="21">
-        <f t="shared" si="6"/>
+      <c r="C38" s="49" t="s">
+        <v>5</v>
+      </c>
+      <c r="D38" s="50" t="s">
+        <v>6</v>
+      </c>
+      <c r="E38" s="46">
+        <v>1</v>
+      </c>
+      <c r="F38" s="47">
+        <v>1</v>
+      </c>
+      <c r="G38" s="46">
+        <v>2</v>
+      </c>
+      <c r="H38" s="46">
+        <f t="shared" si="4"/>
         <v>4</v>
       </c>
-      <c r="I38" s="9">
-        <v>0</v>
-      </c>
-      <c r="J38" s="20"/>
+      <c r="I38" s="48">
+        <v>5</v>
+      </c>
       <c r="K38" s="1"/>
       <c r="L38" s="1"/>
       <c r="M38" s="1"/>
       <c r="N38" s="1"/>
     </row>
-    <row r="39" spans="2:14" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="B39" s="9">
-        <f t="shared" si="7"/>
+    <row r="39" spans="2:14" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B39" s="48">
+        <f t="shared" si="5"/>
         <v>35</v>
       </c>
-      <c r="C39" s="5" t="s">
-        <v>40</v>
-      </c>
-      <c r="D39" s="12" t="s">
-        <v>41</v>
-      </c>
-      <c r="E39" s="21">
-        <v>1</v>
-      </c>
-      <c r="F39" s="24">
-        <v>1</v>
-      </c>
-      <c r="G39" s="21">
-        <v>2</v>
-      </c>
-      <c r="H39" s="21">
-        <f t="shared" si="6"/>
+      <c r="C39" s="44" t="s">
+        <v>44</v>
+      </c>
+      <c r="D39" s="50" t="s">
+        <v>45</v>
+      </c>
+      <c r="E39" s="46">
+        <v>2</v>
+      </c>
+      <c r="F39" s="47">
+        <v>1</v>
+      </c>
+      <c r="G39" s="46">
+        <v>1</v>
+      </c>
+      <c r="H39" s="46">
+        <f t="shared" si="4"/>
         <v>4</v>
       </c>
-      <c r="I39" s="9">
-        <v>0</v>
+      <c r="I39" s="48">
+        <v>5</v>
       </c>
       <c r="J39" s="20"/>
       <c r="K39" s="1"/>
@@ -2294,48 +2335,52 @@
       <c r="M39" s="1"/>
       <c r="N39" s="1"/>
     </row>
-    <row r="40" spans="2:14" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="B40" s="9">
-        <f t="shared" si="7"/>
+    <row r="40" spans="2:14" ht="78.75" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B40" s="48">
+        <f t="shared" si="5"/>
         <v>36</v>
       </c>
-      <c r="C40" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="D40" s="12" t="s">
+      <c r="C40" s="49" t="s">
+        <v>33</v>
+      </c>
+      <c r="D40" s="50" t="s">
+        <v>34</v>
+      </c>
+      <c r="E40" s="46">
+        <v>1</v>
+      </c>
+      <c r="F40" s="47">
+        <v>1</v>
+      </c>
+      <c r="G40" s="46">
+        <v>2</v>
+      </c>
+      <c r="H40" s="46">
+        <f t="shared" si="4"/>
         <v>4</v>
       </c>
-      <c r="E40" s="21">
-        <v>1</v>
-      </c>
-      <c r="F40" s="24">
-        <v>1</v>
-      </c>
-      <c r="G40" s="21">
-        <v>1</v>
-      </c>
-      <c r="H40" s="21">
-        <f t="shared" si="6"/>
-        <v>3</v>
-      </c>
-      <c r="I40" s="9">
-        <v>0</v>
-      </c>
-      <c r="J40" s="20"/>
+      <c r="I40" s="48">
+        <v>5</v>
+      </c>
+      <c r="J40" s="20" t="s">
+        <v>51</v>
+      </c>
       <c r="K40" s="1"/>
       <c r="L40" s="1"/>
       <c r="M40" s="1"/>
       <c r="N40" s="1"/>
     </row>
-    <row r="41" spans="2:14" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="41" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B41" s="9">
-        <f t="shared" si="7"/>
+        <f t="shared" si="5"/>
         <v>37</v>
       </c>
       <c r="C41" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="D41" s="12"/>
+        <v>7</v>
+      </c>
+      <c r="D41" s="12" t="s">
+        <v>8</v>
+      </c>
       <c r="E41" s="21">
         <v>1</v>
       </c>
@@ -2343,11 +2388,11 @@
         <v>1</v>
       </c>
       <c r="G41" s="21">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H41" s="21">
-        <f t="shared" si="6"/>
-        <v>3</v>
+        <f t="shared" si="4"/>
+        <v>4</v>
       </c>
       <c r="I41" s="9">
         <v>0</v>
@@ -2358,29 +2403,31 @@
       <c r="M41" s="1"/>
       <c r="N41" s="1"/>
     </row>
-    <row r="42" spans="2:14" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="2:14" ht="31.5" x14ac:dyDescent="0.25">
       <c r="B42" s="9">
-        <f t="shared" si="7"/>
+        <f t="shared" si="5"/>
         <v>38</v>
       </c>
-      <c r="C42" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="D42" s="13"/>
-      <c r="E42" s="22">
-        <v>1</v>
-      </c>
-      <c r="F42" s="25">
-        <v>1</v>
-      </c>
-      <c r="G42" s="22">
-        <v>1</v>
-      </c>
-      <c r="H42" s="22">
-        <f t="shared" si="6"/>
-        <v>3</v>
-      </c>
-      <c r="I42" s="28">
+      <c r="C42" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="D42" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="E42" s="21">
+        <v>1</v>
+      </c>
+      <c r="F42" s="24">
+        <v>1</v>
+      </c>
+      <c r="G42" s="21">
+        <v>2</v>
+      </c>
+      <c r="H42" s="21">
+        <f t="shared" si="4"/>
+        <v>4</v>
+      </c>
+      <c r="I42" s="9">
         <v>0</v>
       </c>
       <c r="J42" s="20"/>
@@ -2389,67 +2436,135 @@
       <c r="M42" s="1"/>
       <c r="N42" s="1"/>
     </row>
-    <row r="43" spans="2:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="I43" s="10"/>
+    <row r="43" spans="2:14" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="B43" s="9">
+        <f t="shared" si="5"/>
+        <v>39</v>
+      </c>
+      <c r="C43" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="D43" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="E43" s="21">
+        <v>1</v>
+      </c>
+      <c r="F43" s="24">
+        <v>1</v>
+      </c>
+      <c r="G43" s="21">
+        <v>2</v>
+      </c>
+      <c r="H43" s="21">
+        <f t="shared" si="4"/>
+        <v>4</v>
+      </c>
+      <c r="I43" s="9">
+        <v>0</v>
+      </c>
       <c r="J43" s="20"/>
       <c r="K43" s="1"/>
       <c r="L43" s="1"/>
       <c r="M43" s="1"/>
       <c r="N43" s="1"/>
     </row>
-    <row r="44" spans="2:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B44" s="10"/>
-      <c r="C44" s="26"/>
-      <c r="D44" s="27"/>
-      <c r="E44" s="20"/>
-      <c r="F44" s="20"/>
-      <c r="G44" s="20"/>
-      <c r="H44" s="20"/>
-      <c r="I44" s="10"/>
+    <row r="44" spans="2:14" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="B44" s="9">
+        <f t="shared" si="5"/>
+        <v>40</v>
+      </c>
+      <c r="C44" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="D44" s="12" t="s">
+        <v>4</v>
+      </c>
+      <c r="E44" s="21">
+        <v>1</v>
+      </c>
+      <c r="F44" s="24">
+        <v>1</v>
+      </c>
+      <c r="G44" s="21">
+        <v>1</v>
+      </c>
+      <c r="H44" s="21">
+        <f t="shared" si="4"/>
+        <v>3</v>
+      </c>
+      <c r="I44" s="9">
+        <v>0</v>
+      </c>
       <c r="J44" s="20"/>
       <c r="K44" s="1"/>
       <c r="L44" s="1"/>
       <c r="M44" s="1"/>
       <c r="N44" s="1"/>
     </row>
-    <row r="45" spans="2:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B45" s="1"/>
-      <c r="C45" s="7"/>
-      <c r="D45" s="2"/>
-      <c r="E45" s="10"/>
-      <c r="F45" s="10"/>
-      <c r="G45" s="10"/>
-      <c r="H45" s="10"/>
-      <c r="I45" s="10"/>
+    <row r="45" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B45" s="9">
+        <f t="shared" si="5"/>
+        <v>41</v>
+      </c>
+      <c r="C45" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D45" s="12"/>
+      <c r="E45" s="21">
+        <v>1</v>
+      </c>
+      <c r="F45" s="24">
+        <v>1</v>
+      </c>
+      <c r="G45" s="21">
+        <v>1</v>
+      </c>
+      <c r="H45" s="21">
+        <f t="shared" si="4"/>
+        <v>3</v>
+      </c>
+      <c r="I45" s="9">
+        <v>0</v>
+      </c>
       <c r="J45" s="20"/>
       <c r="K45" s="1"/>
       <c r="L45" s="1"/>
       <c r="M45" s="1"/>
       <c r="N45" s="1"/>
     </row>
-    <row r="46" spans="2:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B46" s="1"/>
-      <c r="C46" s="7"/>
-      <c r="D46" s="2"/>
-      <c r="E46" s="10"/>
-      <c r="F46" s="10"/>
-      <c r="G46" s="10"/>
-      <c r="H46" s="10"/>
-      <c r="I46" s="10"/>
+    <row r="46" spans="2:14" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B46" s="9">
+        <f t="shared" si="5"/>
+        <v>42</v>
+      </c>
+      <c r="C46" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="D46" s="13"/>
+      <c r="E46" s="22">
+        <v>1</v>
+      </c>
+      <c r="F46" s="25">
+        <v>1</v>
+      </c>
+      <c r="G46" s="22">
+        <v>1</v>
+      </c>
+      <c r="H46" s="22">
+        <f t="shared" si="4"/>
+        <v>3</v>
+      </c>
+      <c r="I46" s="28">
+        <v>0</v>
+      </c>
       <c r="J46" s="20"/>
       <c r="K46" s="1"/>
       <c r="L46" s="1"/>
       <c r="M46" s="1"/>
       <c r="N46" s="1"/>
     </row>
-    <row r="47" spans="2:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B47" s="1"/>
-      <c r="C47" s="7"/>
-      <c r="D47" s="2"/>
-      <c r="E47" s="10"/>
-      <c r="F47" s="10"/>
-      <c r="G47" s="10"/>
-      <c r="H47" s="10"/>
+    <row r="47" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="I47" s="10"/>
       <c r="J47" s="20"/>
       <c r="K47" s="1"/>
@@ -2457,14 +2572,14 @@
       <c r="M47" s="1"/>
       <c r="N47" s="1"/>
     </row>
-    <row r="48" spans="2:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B48" s="1"/>
-      <c r="C48" s="7"/>
-      <c r="D48" s="2"/>
-      <c r="E48" s="10"/>
-      <c r="F48" s="10"/>
-      <c r="G48" s="10"/>
-      <c r="H48" s="10"/>
+    <row r="48" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B48" s="10"/>
+      <c r="C48" s="26"/>
+      <c r="D48" s="27"/>
+      <c r="E48" s="20"/>
+      <c r="F48" s="20"/>
+      <c r="G48" s="20"/>
+      <c r="H48" s="20"/>
       <c r="I48" s="10"/>
       <c r="J48" s="20"/>
       <c r="K48" s="1"/>
@@ -2472,7 +2587,7 @@
       <c r="M48" s="1"/>
       <c r="N48" s="1"/>
     </row>
-    <row r="49" spans="2:14" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="49" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B49" s="1"/>
       <c r="C49" s="7"/>
       <c r="D49" s="2"/>
@@ -2487,7 +2602,7 @@
       <c r="M49" s="1"/>
       <c r="N49" s="1"/>
     </row>
-    <row r="50" spans="2:14" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="50" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B50" s="1"/>
       <c r="C50" s="7"/>
       <c r="D50" s="2"/>
@@ -2502,7 +2617,7 @@
       <c r="M50" s="1"/>
       <c r="N50" s="1"/>
     </row>
-    <row r="51" spans="2:14" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="51" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B51" s="1"/>
       <c r="C51" s="7"/>
       <c r="D51" s="2"/>
@@ -2517,7 +2632,7 @@
       <c r="M51" s="1"/>
       <c r="N51" s="1"/>
     </row>
-    <row r="52" spans="2:14" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="52" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B52" s="1"/>
       <c r="C52" s="7"/>
       <c r="D52" s="2"/>
@@ -2532,7 +2647,7 @@
       <c r="M52" s="1"/>
       <c r="N52" s="1"/>
     </row>
-    <row r="53" spans="2:14" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="53" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B53" s="1"/>
       <c r="C53" s="7"/>
       <c r="D53" s="2"/>
@@ -2547,7 +2662,7 @@
       <c r="M53" s="1"/>
       <c r="N53" s="1"/>
     </row>
-    <row r="54" spans="2:14" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="54" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B54" s="1"/>
       <c r="C54" s="7"/>
       <c r="D54" s="2"/>
@@ -2562,8 +2677,68 @@
       <c r="M54" s="1"/>
       <c r="N54" s="1"/>
     </row>
+    <row r="55" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B55" s="1"/>
+      <c r="C55" s="7"/>
+      <c r="D55" s="2"/>
+      <c r="E55" s="10"/>
+      <c r="F55" s="10"/>
+      <c r="G55" s="10"/>
+      <c r="H55" s="10"/>
+      <c r="I55" s="10"/>
+      <c r="J55" s="20"/>
+      <c r="K55" s="1"/>
+      <c r="L55" s="1"/>
+      <c r="M55" s="1"/>
+      <c r="N55" s="1"/>
+    </row>
+    <row r="56" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B56" s="1"/>
+      <c r="C56" s="7"/>
+      <c r="D56" s="2"/>
+      <c r="E56" s="10"/>
+      <c r="F56" s="10"/>
+      <c r="G56" s="10"/>
+      <c r="H56" s="10"/>
+      <c r="I56" s="10"/>
+      <c r="J56" s="20"/>
+      <c r="K56" s="1"/>
+      <c r="L56" s="1"/>
+      <c r="M56" s="1"/>
+      <c r="N56" s="1"/>
+    </row>
+    <row r="57" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B57" s="1"/>
+      <c r="C57" s="7"/>
+      <c r="D57" s="2"/>
+      <c r="E57" s="10"/>
+      <c r="F57" s="10"/>
+      <c r="G57" s="10"/>
+      <c r="H57" s="10"/>
+      <c r="I57" s="10"/>
+      <c r="J57" s="20"/>
+      <c r="K57" s="1"/>
+      <c r="L57" s="1"/>
+      <c r="M57" s="1"/>
+      <c r="N57" s="1"/>
+    </row>
+    <row r="58" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B58" s="1"/>
+      <c r="C58" s="7"/>
+      <c r="D58" s="2"/>
+      <c r="E58" s="10"/>
+      <c r="F58" s="10"/>
+      <c r="G58" s="10"/>
+      <c r="H58" s="10"/>
+      <c r="I58" s="10"/>
+      <c r="J58" s="20"/>
+      <c r="K58" s="1"/>
+      <c r="L58" s="1"/>
+      <c r="M58" s="1"/>
+      <c r="N58" s="1"/>
+    </row>
   </sheetData>
-  <autoFilter ref="B3:I42" xr:uid="{11BA4F79-2AB7-4A24-A4BE-758442E1F8CB}">
+  <autoFilter ref="B3:I46" xr:uid="{11BA4F79-2AB7-4A24-A4BE-758442E1F8CB}">
     <filterColumn colId="7">
       <filters>
         <filter val="0"/>
@@ -2573,16 +2748,16 @@
         <filter val="4"/>
       </filters>
     </filterColumn>
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B5:I42">
-      <sortCondition descending="1" ref="H4:H42"/>
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B5:I46">
+      <sortCondition descending="1" ref="H4:H46"/>
     </sortState>
   </autoFilter>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B5:J42">
-    <sortCondition descending="1" ref="H4:H42"/>
-    <sortCondition descending="1" ref="E4:E42"/>
-    <sortCondition descending="1" ref="F4:F42"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B8:J46">
+    <sortCondition descending="1" ref="H4:H46"/>
+    <sortCondition descending="1" ref="E4:E46"/>
+    <sortCondition descending="1" ref="F4:F46"/>
   </sortState>
-  <conditionalFormatting sqref="H4:H42">
+  <conditionalFormatting sqref="H4:H46">
     <cfRule type="colorScale" priority="3">
       <colorScale>
         <cfvo type="min"/>
@@ -2594,7 +2769,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I4:I42">
+  <conditionalFormatting sqref="I4:I46">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>

</xml_diff>